<commit_message>
Aktualizace dat - nova adresa Apimex (Steyr)
</commit_message>
<xml_diff>
--- a/Obst.xlsx
+++ b/Obst.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://herzjesugym-my.sharepoint.com/personal/denis_holub_herzjesugym_at/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="108" documentId="8_{16DF881F-28DA-49AF-8735-25E400E6511D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3055CFB9-0F6E-42B0-83FD-C3064401C8F3}"/>
+  <xr:revisionPtr revIDLastSave="110" documentId="8_{16DF881F-28DA-49AF-8735-25E400E6511D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E5B77351-CD77-42A2-9006-459057A5CE96}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{0E2E01CC-D03A-446C-9945-79710707EE2F}"/>
   </bookViews>
@@ -140,9 +140,6 @@
     <t>Apimex</t>
   </si>
   <si>
-    <t>Wels</t>
-  </si>
-  <si>
     <t>Gasteiger</t>
   </si>
   <si>
@@ -180,6 +177,9 @@
   </si>
   <si>
     <t>Geliefert</t>
+  </si>
+  <si>
+    <t>Interfruit, Weinzierlstraße 2, 4400 Steyr</t>
   </si>
 </sst>
 </file>
@@ -187,10 +187,10 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="_-&quot;€&quot;\ * #,##0.00_-;\-&quot;€&quot;\ * #,##0.00_-;_-&quot;€&quot;\ * &quot;-&quot;??_-;_-@_-"/>
-    <numFmt numFmtId="165" formatCode="0\ &quot;kg&quot;"/>
+    <numFmt numFmtId="44" formatCode="_-&quot;€&quot;\ * #,##0.00_-;\-&quot;€&quot;\ * #,##0.00_-;_-&quot;€&quot;\ * &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="164" formatCode="0\ &quot;kg&quot;"/>
   </numFmts>
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -225,6 +225,12 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -245,14 +251,14 @@
   </borders>
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="2"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
@@ -262,6 +268,7 @@
         </ext>
       </extLst>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Link" xfId="2" builtinId="8"/>
@@ -627,7 +634,7 @@
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B1" t="s">
         <v>0</v>
@@ -780,7 +787,7 @@
         <v>1200</v>
       </c>
       <c r="F8" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.35">
@@ -801,7 +808,7 @@
         <v>450</v>
       </c>
       <c r="F9" s="5" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="G9" t="s">
         <v>15</v>
@@ -909,7 +916,7 @@
         <v>1000</v>
       </c>
       <c r="F14" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.35">
@@ -951,7 +958,7 @@
         <v>300</v>
       </c>
       <c r="F16" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="G16" t="s">
         <v>29</v>
@@ -965,14 +972,14 @@
         <v>30</v>
       </c>
       <c r="C17" s="3">
-        <v>500</v>
+        <v>600</v>
       </c>
       <c r="D17" s="2">
         <v>1.4</v>
       </c>
       <c r="E17" s="2">
         <f t="shared" si="1"/>
-        <v>700</v>
+        <v>840</v>
       </c>
       <c r="F17" t="s">
         <v>31</v>
@@ -995,8 +1002,8 @@
         <f t="shared" si="1"/>
         <v>4500</v>
       </c>
-      <c r="F18" t="s">
-        <v>33</v>
+      <c r="F18" s="7" t="s">
+        <v>46</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.35">
@@ -1004,7 +1011,7 @@
         <v>0</v>
       </c>
       <c r="B19" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C19" s="3">
         <v>500</v>
@@ -1017,10 +1024,10 @@
         <v>750</v>
       </c>
       <c r="F19" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="G19" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.35">
@@ -1028,7 +1035,7 @@
         <v>0</v>
       </c>
       <c r="B20" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C20" s="3">
         <v>200</v>
@@ -1041,7 +1048,7 @@
         <v>300</v>
       </c>
       <c r="F20" s="4" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.35">
@@ -1049,7 +1056,7 @@
         <v>0</v>
       </c>
       <c r="B21" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C21" s="3">
         <v>200</v>
@@ -1062,7 +1069,7 @@
         <v>300</v>
       </c>
       <c r="F21" s="5" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.35">
@@ -1070,7 +1077,7 @@
         <v>0</v>
       </c>
       <c r="B22" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C22" s="3">
         <v>500</v>
@@ -1083,7 +1090,7 @@
         <v>750</v>
       </c>
       <c r="F22" s="5" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.35">
@@ -1100,12 +1107,12 @@
       </c>
       <c r="C24" s="3">
         <f>SUM(C2:C23)</f>
-        <v>12460</v>
+        <v>12560</v>
       </c>
       <c r="D24" s="2"/>
       <c r="E24" s="2">
         <f>SUM(E2:E23)</f>
-        <v>18140</v>
+        <v>18280</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
Podpora GPS souradnic v adrese/poznamce + oprava polohy Primushausl
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Obst.xlsx
+++ b/Obst.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://herzjesugym-my.sharepoint.com/personal/denis_holub_herzjesugym_at/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="110" documentId="8_{16DF881F-28DA-49AF-8735-25E400E6511D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E5B77351-CD77-42A2-9006-459057A5CE96}"/>
+  <xr:revisionPtr revIDLastSave="111" documentId="8_{16DF881F-28DA-49AF-8735-25E400E6511D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F32FA874-A872-4FA8-A462-215DCD38808F}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{0E2E01CC-D03A-446C-9945-79710707EE2F}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="48">
   <si>
     <t>Weichsel</t>
   </si>
@@ -180,6 +180,9 @@
   </si>
   <si>
     <t>Interfruit, Weinzierlstraße 2, 4400 Steyr</t>
+  </si>
+  <si>
+    <t>Primushäusl Edelbrände (47.7264661, 13.4350206)</t>
   </si>
 </sst>
 </file>
@@ -789,6 +792,9 @@
       <c r="F8" t="s">
         <v>39</v>
       </c>
+      <c r="G8" t="s">
+        <v>47</v>
+      </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A9" s="6" t="b">

</xml_diff>

<commit_message>
Dorucene zastavky zelene + novy zakaznik Maishofen
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Obst.xlsx
+++ b/Obst.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://herzjesugym-my.sharepoint.com/personal/denis_holub_herzjesugym_at/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="174" documentId="8_{16DF881F-28DA-49AF-8735-25E400E6511D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{82A7993C-EE13-4A2F-B412-89B38D0108CE}"/>
+  <xr:revisionPtr revIDLastSave="181" documentId="8_{16DF881F-28DA-49AF-8735-25E400E6511D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C6431279-148F-46D2-A1D3-7EBFBD04C7B1}"/>
   <bookViews>
     <workbookView xWindow="15690" yWindow="15110" windowWidth="6380" windowHeight="3340" xr2:uid="{0E2E01CC-D03A-446C-9945-79710707EE2F}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="59">
   <si>
     <t>Weichsel</t>
   </si>
@@ -207,6 +207,15 @@
   </si>
   <si>
     <t>Rest der Bestellung (3600 kg)</t>
+  </si>
+  <si>
+    <t>Maishofen (Anrufer)</t>
+  </si>
+  <si>
+    <t>5751 Maishofen</t>
+  </si>
+  <si>
+    <t>telefonisch bestellt, Name/Adresse ergänzen</t>
   </si>
 </sst>
 </file>
@@ -309,7 +318,18 @@
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
     <cellStyle name="Währung" xfId="1" builtinId="4"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="1">
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -1212,6 +1232,25 @@
       <c r="A26" s="6" t="b">
         <v>0</v>
       </c>
+      <c r="B26" t="s">
+        <v>56</v>
+      </c>
+      <c r="C26">
+        <v>1000</v>
+      </c>
+      <c r="D26">
+        <v>1.5</v>
+      </c>
+      <c r="E26">
+        <f>C26*D26</f>
+        <v>1500</v>
+      </c>
+      <c r="F26" t="s">
+        <v>57</v>
+      </c>
+      <c r="G26" t="s">
+        <v>58</v>
+      </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A27" s="6" t="b">
@@ -1264,12 +1303,12 @@
       </c>
       <c r="C36" s="3">
         <f>SUM(C2:C35)</f>
-        <v>13710</v>
+        <v>14710</v>
       </c>
       <c r="D36" s="3"/>
       <c r="E36" s="9">
         <f>SUM(E2:E35)</f>
-        <v>18940</v>
+        <v>20440</v>
       </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.35">
@@ -1363,6 +1402,11 @@
       </c>
     </row>
   </sheetData>
+  <conditionalFormatting sqref="A2:G35">
+    <cfRule type="expression" dxfId="0" priority="1" stopIfTrue="1">
+      <formula>$A2='TRUE'</formula>
+    </cfRule>
+  </conditionalFormatting>
   <hyperlinks>
     <hyperlink ref="F10" r:id="rId1" display="https://www.google.com/maps/place/data=!4m2!3m1!1s0x47747715538db01d:0x16d28a73419a5295?sa=X&amp;ved=1t:8290&amp;ictx=111" xr:uid="{D642E8DC-BBBD-4F4B-A4DC-252C3C0D6734}"/>
     <hyperlink ref="F13" r:id="rId2" display="https://www.google.com/maps/place/data=!4m2!3m1!1s0x4773af04442266fd:0x116ce1c69494bb32?sa=X&amp;ved=1t:8290&amp;ictx=111" xr:uid="{1745D04A-32DE-4B22-BE2A-10ABC6DB20F4}"/>

</xml_diff>

<commit_message>
Pridana objednavka: Christoph Olsinger, 300 kg, Kremsmunster
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Obst.xlsx
+++ b/Obst.xlsx
@@ -5,21 +5,18 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://herzjesugym-my.sharepoint.com/personal/denis_holub_herzjesugym_at/Documents/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://herzjesugym-my.sharepoint.com/personal/denis_holub_herzjesugym_at/Documents/Radtour 2026/mapa-rozvozu-ovoce/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="14" documentId="13_ncr:1_{BD9264F1-AD0B-4A45-8BA2-60A535DA1E6A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{88885897-78BB-40FD-9891-17A97C1C1D59}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="11_449FA02F188DA641CC72A8D655938E786A01E074" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="15350" yWindow="14770" windowWidth="6380" windowHeight="3340" xr2:uid="{0E2E01CC-D03A-446C-9945-79710707EE2F}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191028"/>
+  <calcPr calcId="191029"/>
   <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
         <xcalcf:feature name="microsoft.com:RD"/>
@@ -31,15 +28,15 @@
         <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="2"/>
-    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="64">
+  <si>
+    <t>Geliefert</t>
+  </si>
   <si>
     <t>Weichsel</t>
   </si>
@@ -59,12 +56,18 @@
     <t>Julia Eigner</t>
   </si>
   <si>
+    <t> Haagweg 7, 5550 Radstadt</t>
+  </si>
+  <si>
     <t>Manuela</t>
   </si>
   <si>
     <t>Bad Hall Eichenstraße 20</t>
   </si>
   <si>
+    <t>inkl. 40 € Trinkgeld</t>
+  </si>
+  <si>
     <t xml:space="preserve">Hannes Holzer </t>
   </si>
   <si>
@@ -83,9 +86,18 @@
     <t>Sigi Rieger</t>
   </si>
   <si>
+    <t>Forsthub 20, 5350 Abersee</t>
+  </si>
+  <si>
+    <t>Primushäusl Edelbrände (47.7264661, 13.4350206)</t>
+  </si>
+  <si>
     <t>Wolfgang Dexelheimer</t>
   </si>
   <si>
+    <t>Jaukenberg 31/32 4170 Haslach</t>
+  </si>
+  <si>
     <t>stadlbrennerei</t>
   </si>
   <si>
@@ -95,12 +107,24 @@
     <t>Stroiß 6, 4730 Waizenkirchen</t>
   </si>
   <si>
+    <t>Ernst Kadar</t>
+  </si>
+  <si>
+    <t>8992 Altaussee</t>
+  </si>
+  <si>
+    <t>abgeholt bei Kalteis (Waizenkirchen), für nächstes Jahr</t>
+  </si>
+  <si>
     <t>Lukas Undesser</t>
   </si>
   <si>
     <t>Koglerauer Weg 17, 4040 Gramastetten</t>
   </si>
   <si>
+    <t>inkl. 20 € Trinkgeld</t>
+  </si>
+  <si>
     <t>Heiner Burgstaller</t>
   </si>
   <si>
@@ -110,21 +134,21 @@
     <t>Christof Moser</t>
   </si>
   <si>
+    <t>Mistlberg 28, 4284 Tragwein</t>
+  </si>
+  <si>
     <t>Steiermark Selbstabholung</t>
   </si>
   <si>
+    <t>Selbstabholung, Krtely 70</t>
+  </si>
+  <si>
     <t>Werner</t>
   </si>
   <si>
     <t>Vöcklabruck</t>
   </si>
   <si>
-    <t>Mistlberg 28, 4284 Tragwein</t>
-  </si>
-  <si>
-    <t> Haagweg 7, 5550 Radstadt</t>
-  </si>
-  <si>
     <t>Milan</t>
   </si>
   <si>
@@ -140,51 +164,39 @@
     <t>Apimex</t>
   </si>
   <si>
+    <t>Interfruit, Weinzierlstraße 2, 4400 Steyr</t>
+  </si>
+  <si>
+    <t>geliefert 3000 kg, Rest von 3600 storniert</t>
+  </si>
+  <si>
     <t>Gasteiger</t>
   </si>
   <si>
+    <t>Auweg 73, 4820</t>
+  </si>
+  <si>
     <t>1 Großkiste</t>
   </si>
   <si>
+    <t>Flöckner</t>
+  </si>
+  <si>
     <t>Fahrenzaglstraße 4, Elixhausen</t>
   </si>
   <si>
-    <t>Flöckner</t>
-  </si>
-  <si>
     <t>Hageneder Roland</t>
   </si>
   <si>
+    <t>4551 Ried im Traunkreis. Rührndorf 2</t>
+  </si>
+  <si>
     <t>Peter Fuchs</t>
   </si>
   <si>
-    <t>Forsthub 20, 5350 Abersee</t>
-  </si>
-  <si>
-    <t>Jaukenberg 31/32 4170 Haslach</t>
-  </si>
-  <si>
-    <t>Selbstabholung, Krtely 70</t>
-  </si>
-  <si>
-    <t>Auweg 73, 4820</t>
-  </si>
-  <si>
-    <t>4551 Ried im Traunkreis. Rührndorf 2</t>
-  </si>
-  <si>
     <t>Lämmererweg 2 5321 Koppl </t>
   </si>
   <si>
-    <t>Geliefert</t>
-  </si>
-  <si>
-    <t>Interfruit, Weinzierlstraße 2, 4400 Steyr</t>
-  </si>
-  <si>
-    <t>Primushäusl Edelbrände (47.7264661, 13.4350206)</t>
-  </si>
-  <si>
     <t>Fuchs Freund</t>
   </si>
   <si>
@@ -200,24 +212,6 @@
     <t>pauschal 400 €</t>
   </si>
   <si>
-    <t>inkl. 20 € Trinkgeld</t>
-  </si>
-  <si>
-    <t>inkl. 40 € Trinkgeld</t>
-  </si>
-  <si>
-    <t>Ernst Kadar</t>
-  </si>
-  <si>
-    <t>8992 Altaussee</t>
-  </si>
-  <si>
-    <t>abgeholt bei Kalteis (Waizenkirchen), für nächstes Jahr</t>
-  </si>
-  <si>
-    <t>geliefert 3000 kg, Rest von 3600 storniert</t>
-  </si>
-  <si>
     <t>Werner Mitteregger</t>
   </si>
   <si>
@@ -225,6 +219,12 @@
   </si>
   <si>
     <t>telefonisch bestellt</t>
+  </si>
+  <si>
+    <t>Christoph Ölsinger</t>
+  </si>
+  <si>
+    <t>Guntendorf 10, 4550 Kremsmünster</t>
   </si>
 </sst>
 </file>
@@ -232,8 +232,8 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="_-&quot;€&quot;\ * #,##0.00_-;\-&quot;€&quot;\ * #,##0.00_-;_-&quot;€&quot;\ * &quot;-&quot;??_-;_-@_-"/>
-    <numFmt numFmtId="165" formatCode="0\ &quot;kg&quot;"/>
+    <numFmt numFmtId="44" formatCode="_-&quot;€&quot;\ * #,##0.00_-;\-&quot;€&quot;\ * #,##0.00_-;_-&quot;€&quot;\ * &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="164" formatCode="0\ &quot;kg&quot;"/>
   </numFmts>
   <fonts count="7" x14ac:knownFonts="1">
     <font>
@@ -301,26 +301,20 @@
   </borders>
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="44" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="2"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
-      <extLst>
-        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
-          <xfpb:xfComplement i="0"/>
-        </ext>
-      </extLst>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Link" xfId="2" builtinId="8"/>
@@ -349,23 +343,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/featurePropertyBag/featurePropertyBag.xml><?xml version="1.0" encoding="utf-8"?>
-<FeaturePropertyBags xmlns="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag">
-  <bag type="Checkbox"/>
-  <bag type="XFControls">
-    <bagId k="CellControl">0</bagId>
-  </bag>
-  <bag type="XFComplement">
-    <bagId k="XFControls">1</bagId>
-  </bag>
-  <bag type="XFComplements" extRef="XFComplementsMapperExtRef">
-    <a k="MappedFeaturePropertyBags">
-      <bagId>2</bagId>
-    </a>
-  </bag>
-</FeaturePropertyBags>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -684,7 +661,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8369C171-C908-4428-93B9-D851AB8988B4}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:H54"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -697,18 +674,18 @@
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
-        <v>45</v>
+        <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A2" s="6" t="b">
+      <c r="A2" t="b">
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C2" s="3">
         <v>600</v>
@@ -721,15 +698,15 @@
         <v>900</v>
       </c>
       <c r="F2" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A3" s="6" t="b">
+      <c r="A3" t="b">
         <v>0</v>
       </c>
       <c r="B3" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C3" s="3">
         <v>500</v>
@@ -738,19 +715,19 @@
         <v>1.5</v>
       </c>
       <c r="E3" s="2">
-        <f t="shared" ref="E3:E16" si="0">C3*D3</f>
+        <f>C3*D3</f>
         <v>750</v>
       </c>
       <c r="F3" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A4" s="6" t="b">
+      <c r="A4" t="b">
         <v>0</v>
       </c>
       <c r="B4" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C4" s="3">
         <v>1000</v>
@@ -759,19 +736,19 @@
         <v>1.5</v>
       </c>
       <c r="E4" s="2">
-        <f t="shared" si="0"/>
+        <f>C4*D4</f>
         <v>1500</v>
       </c>
       <c r="F4" t="s">
-        <v>27</v>
+        <v>7</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A5" s="6" t="b">
+      <c r="A5" t="b">
         <v>1</v>
       </c>
       <c r="B5" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="C5" s="3">
         <v>200</v>
@@ -783,18 +760,18 @@
         <v>340</v>
       </c>
       <c r="F5" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="G5" t="s">
-        <v>54</v>
+        <v>10</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A6" s="6" t="b">
+      <c r="A6" t="b">
         <v>0</v>
       </c>
       <c r="B6" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="C6" s="3">
         <v>500</v>
@@ -803,22 +780,22 @@
         <v>1.5</v>
       </c>
       <c r="E6" s="2">
-        <f t="shared" si="0"/>
+        <f t="shared" ref="E6:E11" si="0">C6*D6</f>
         <v>750</v>
       </c>
       <c r="F6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="G6" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A7" s="6" t="b">
+      <c r="A7" t="b">
         <v>0</v>
       </c>
       <c r="B7" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="C7" s="3">
         <v>350</v>
@@ -831,15 +808,15 @@
         <v>525</v>
       </c>
       <c r="F7" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A8" s="6" t="b">
+      <c r="A8" t="b">
         <v>0</v>
       </c>
       <c r="B8" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="C8" s="3">
         <v>800</v>
@@ -852,18 +829,18 @@
         <v>1200</v>
       </c>
       <c r="F8" t="s">
-        <v>39</v>
+        <v>17</v>
       </c>
       <c r="G8" t="s">
-        <v>47</v>
+        <v>18</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A9" s="6" t="b">
+      <c r="A9" t="b">
         <v>0</v>
       </c>
       <c r="B9" t="s">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="C9" s="3">
         <v>300</v>
@@ -876,18 +853,18 @@
         <v>450</v>
       </c>
       <c r="F9" s="5" t="s">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="G9" t="s">
-        <v>15</v>
+        <v>21</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A10" s="6" t="b">
+      <c r="A10" t="b">
         <v>1</v>
       </c>
       <c r="B10" t="s">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="C10" s="3">
         <v>400</v>
@@ -900,15 +877,15 @@
         <v>600</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A11" s="6" t="b">
+      <c r="A11" t="b">
         <v>1</v>
       </c>
       <c r="B11" t="s">
-        <v>55</v>
+        <v>24</v>
       </c>
       <c r="C11" s="3">
         <v>200</v>
@@ -917,22 +894,22 @@
         <v>1.5</v>
       </c>
       <c r="E11" s="2">
-        <f>C11*D11</f>
+        <f t="shared" si="0"/>
         <v>300</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>56</v>
+        <v>25</v>
       </c>
       <c r="G11" t="s">
-        <v>57</v>
+        <v>26</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A12" s="6" t="b">
+      <c r="A12" t="b">
         <v>1</v>
       </c>
       <c r="B12" t="s">
-        <v>18</v>
+        <v>27</v>
       </c>
       <c r="C12" s="3">
         <v>100</v>
@@ -944,18 +921,18 @@
         <v>170</v>
       </c>
       <c r="F12" t="s">
-        <v>19</v>
+        <v>28</v>
       </c>
       <c r="G12" t="s">
-        <v>53</v>
+        <v>29</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A13" s="6" t="b">
+      <c r="A13" t="b">
         <v>0</v>
       </c>
       <c r="B13" t="s">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="C13" s="3">
         <v>550</v>
@@ -964,19 +941,19 @@
         <v>1.5</v>
       </c>
       <c r="E13" s="2">
-        <f t="shared" si="0"/>
+        <f t="shared" ref="E13:E27" si="1">C13*D13</f>
         <v>825</v>
       </c>
       <c r="F13" t="s">
-        <v>21</v>
+        <v>31</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A14" s="6" t="b">
+      <c r="A14" t="b">
         <v>1</v>
       </c>
       <c r="B14" t="s">
-        <v>22</v>
+        <v>32</v>
       </c>
       <c r="C14" s="3">
         <v>900</v>
@@ -985,19 +962,19 @@
         <v>1.25</v>
       </c>
       <c r="E14" s="2">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>1125</v>
       </c>
       <c r="F14" s="1" t="s">
-        <v>26</v>
+        <v>33</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A15" s="6" t="b">
+      <c r="A15" t="b">
         <v>1</v>
       </c>
       <c r="B15" t="s">
-        <v>23</v>
+        <v>34</v>
       </c>
       <c r="C15" s="3">
         <v>1000</v>
@@ -1006,19 +983,19 @@
         <v>1</v>
       </c>
       <c r="E15" s="2">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>1000</v>
       </c>
       <c r="F15" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A16" s="6" t="b">
+      <c r="A16" t="b">
         <v>0</v>
       </c>
       <c r="B16" t="s">
-        <v>24</v>
+        <v>36</v>
       </c>
       <c r="C16" s="3">
         <v>60</v>
@@ -1027,19 +1004,19 @@
         <v>1.5</v>
       </c>
       <c r="E16" s="2">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>90</v>
       </c>
       <c r="F16" t="s">
-        <v>25</v>
+        <v>37</v>
       </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A17" s="6" t="b">
+      <c r="A17" t="b">
         <v>1</v>
       </c>
       <c r="B17" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="C17" s="3">
         <v>150</v>
@@ -1048,25 +1025,25 @@
         <v>1.5</v>
       </c>
       <c r="E17" s="2">
-        <f t="shared" ref="E17:E22" si="1">C17*D17</f>
+        <f t="shared" si="1"/>
         <v>225</v>
       </c>
       <c r="F17" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="G17" t="s">
-        <v>29</v>
+        <v>39</v>
       </c>
       <c r="H17">
         <v>6607174862</v>
       </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A18" s="6" t="b">
+      <c r="A18" t="b">
         <v>0</v>
       </c>
       <c r="B18" t="s">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="C18" s="3">
         <v>600</v>
@@ -1079,15 +1056,15 @@
         <v>840</v>
       </c>
       <c r="F18" t="s">
-        <v>31</v>
+        <v>41</v>
       </c>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A19" s="6" t="b">
+      <c r="A19" t="b">
         <v>1</v>
       </c>
       <c r="B19" t="s">
-        <v>32</v>
+        <v>42</v>
       </c>
       <c r="C19" s="3">
         <v>3000</v>
@@ -1099,19 +1076,19 @@
         <f t="shared" si="1"/>
         <v>3900</v>
       </c>
-      <c r="F19" s="7" t="s">
-        <v>46</v>
+      <c r="F19" s="6" t="s">
+        <v>43</v>
       </c>
       <c r="G19" t="s">
-        <v>58</v>
+        <v>44</v>
       </c>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A20" s="6" t="b">
+      <c r="A20" t="b">
         <v>0</v>
       </c>
       <c r="B20" t="s">
-        <v>33</v>
+        <v>45</v>
       </c>
       <c r="C20" s="3">
         <v>500</v>
@@ -1124,18 +1101,18 @@
         <v>750</v>
       </c>
       <c r="F20" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="G20" t="s">
-        <v>34</v>
+        <v>47</v>
       </c>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A21" s="6" t="b">
+      <c r="A21" t="b">
         <v>1</v>
       </c>
       <c r="B21" t="s">
-        <v>36</v>
+        <v>48</v>
       </c>
       <c r="C21" s="3">
         <v>200</v>
@@ -1148,15 +1125,15 @@
         <v>300</v>
       </c>
       <c r="F21" s="4" t="s">
-        <v>35</v>
+        <v>49</v>
       </c>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A22" s="6" t="b">
+      <c r="A22" t="b">
         <v>1</v>
       </c>
       <c r="B22" t="s">
-        <v>37</v>
+        <v>50</v>
       </c>
       <c r="C22" s="3">
         <v>200</v>
@@ -1169,15 +1146,15 @@
         <v>300</v>
       </c>
       <c r="F22" s="5" t="s">
-        <v>43</v>
+        <v>51</v>
       </c>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A23" s="6" t="b">
+      <c r="A23" t="b">
         <v>1</v>
       </c>
       <c r="B23" t="s">
-        <v>38</v>
+        <v>52</v>
       </c>
       <c r="C23" s="3">
         <v>540</v>
@@ -1186,19 +1163,19 @@
         <v>1.5</v>
       </c>
       <c r="E23" s="2">
-        <f>C23*D23</f>
+        <f t="shared" si="1"/>
         <v>810</v>
       </c>
       <c r="F23" s="5" t="s">
-        <v>44</v>
+        <v>53</v>
       </c>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A24" s="6" t="b">
+      <c r="A24" t="b">
         <v>1</v>
       </c>
       <c r="B24" t="s">
-        <v>48</v>
+        <v>54</v>
       </c>
       <c r="C24" s="3">
         <v>100</v>
@@ -1207,19 +1184,19 @@
         <v>1.5</v>
       </c>
       <c r="E24" s="2">
-        <f>C24*D24</f>
+        <f t="shared" si="1"/>
         <v>150</v>
       </c>
-      <c r="F24" s="8" t="s">
-        <v>49</v>
+      <c r="F24" s="7" t="s">
+        <v>55</v>
       </c>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A25" s="6" t="b">
+      <c r="A25" t="b">
         <v>1</v>
       </c>
       <c r="B25" t="s">
-        <v>50</v>
+        <v>56</v>
       </c>
       <c r="C25" s="3">
         <v>360</v>
@@ -1229,18 +1206,18 @@
         <v>1.1111111111111112</v>
       </c>
       <c r="E25" s="2">
-        <f>C25*D25</f>
+        <f t="shared" si="1"/>
         <v>400</v>
       </c>
-      <c r="F25" s="8" t="s">
-        <v>51</v>
+      <c r="F25" s="7" t="s">
+        <v>57</v>
       </c>
       <c r="G25" t="s">
-        <v>52</v>
+        <v>58</v>
       </c>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A26" s="6" t="b">
+      <c r="A26" t="b">
         <v>0</v>
       </c>
       <c r="B26" t="s">
@@ -1253,7 +1230,7 @@
         <v>1.5</v>
       </c>
       <c r="E26">
-        <f>C26*D26</f>
+        <f t="shared" si="1"/>
         <v>1500</v>
       </c>
       <c r="F26" t="s">
@@ -1264,151 +1241,168 @@
       </c>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A27" s="6" t="b">
-        <v>0</v>
-      </c>
+      <c r="A27" s="9" t="b">
+        <v>0</v>
+      </c>
+      <c r="B27" s="9" t="s">
+        <v>62</v>
+      </c>
+      <c r="C27" s="9">
+        <v>300</v>
+      </c>
+      <c r="D27" s="9">
+        <v>1.5</v>
+      </c>
+      <c r="E27" s="9">
+        <f t="shared" si="1"/>
+        <v>450</v>
+      </c>
+      <c r="F27" s="9" t="s">
+        <v>63</v>
+      </c>
+      <c r="G27" s="9"/>
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A28" s="6" t="b">
+      <c r="A28" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A29" s="6" t="b">
+      <c r="A29" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A30" s="6" t="b">
+      <c r="A30" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A31" s="6" t="b">
+      <c r="A31" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A32" s="6" t="b">
+      <c r="A32" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A33" s="6" t="b">
+      <c r="A33" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A34" s="6" t="b">
+      <c r="A34" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A35" s="6" t="b">
+      <c r="A35" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A36" s="6" t="b">
+      <c r="A36" t="b">
         <v>0</v>
       </c>
       <c r="C36" s="3">
         <f>SUM(C2:C35)</f>
-        <v>14110</v>
+        <v>14410</v>
       </c>
       <c r="D36" s="3"/>
-      <c r="E36" s="9">
+      <c r="E36" s="8">
         <f>SUM(E2:E35)</f>
-        <v>19700</v>
+        <v>20150</v>
       </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A37" s="6" t="b">
+      <c r="A37" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A38" s="6" t="b">
+      <c r="A38" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A39" s="6" t="b">
+      <c r="A39" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A40" s="6" t="b">
+      <c r="A40" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A41" s="6" t="b">
+      <c r="A41" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A42" s="6" t="b">
+      <c r="A42" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A43" s="6" t="b">
+      <c r="A43" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A44" s="6" t="b">
+      <c r="A44" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A45" s="6" t="b">
+      <c r="A45" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A46" s="6" t="b">
+      <c r="A46" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A47" s="6" t="b">
+      <c r="A47" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A48" s="6" t="b">
+      <c r="A48" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="49" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A49" s="6" t="b">
+      <c r="A49" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="50" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A50" s="6" t="b">
+      <c r="A50" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="51" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A51" s="6" t="b">
+      <c r="A51" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="52" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A52" s="6" t="b">
+      <c r="A52" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="53" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A53" s="6" t="b">
+      <c r="A53" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="54" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A54" s="6" t="b">
+      <c r="A54" t="b">
         <v>0</v>
       </c>
     </row>
@@ -1419,10 +1413,10 @@
     </cfRule>
   </conditionalFormatting>
   <hyperlinks>
-    <hyperlink ref="F10" r:id="rId1" display="https://www.google.com/maps/place/data=!4m2!3m1!1s0x47747715538db01d:0x16d28a73419a5295?sa=X&amp;ved=1t:8290&amp;ictx=111" xr:uid="{D642E8DC-BBBD-4F4B-A4DC-252C3C0D6734}"/>
-    <hyperlink ref="F14" r:id="rId2" display="https://www.google.com/maps/place/data=!4m2!3m1!1s0x4773af04442266fd:0x116ce1c69494bb32?sa=X&amp;ved=1t:8290&amp;ictx=111" xr:uid="{1745D04A-32DE-4B22-BE2A-10ABC6DB20F4}"/>
+    <hyperlink ref="F10" r:id="rId1" display="https://www.google.com/maps/place/data=!4m2!3m1!1s0x47747715538db01d:0x16d28a73419a5295?sa=X&amp;ved=1t:8290&amp;ictx=111" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
+    <hyperlink ref="F14" r:id="rId2" display="https://www.google.com/maps/place/data=!4m2!3m1!1s0x4773af04442266fd:0x116ce1c69494bb32?sa=X&amp;ved=1t:8290&amp;ictx=111" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId3"/>
+  <pageSetup paperSize="9" orientation="portrait"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Sigi Rieger: 800 -> 1000 kg
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Obst.xlsx
+++ b/Obst.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://herzjesugym-my.sharepoint.com/personal/denis_holub_herzjesugym_at/Documents/Radtour 2026/mapa-rozvozu-ovoce/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="11_449FA02F188DA641CC72A8D655938E786A01E074" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="11_2687DF7FF0BCAF626073A8D655D9D6FCC967FD68" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -819,14 +819,14 @@
         <v>16</v>
       </c>
       <c r="C8" s="3">
-        <v>800</v>
+        <v>1000</v>
       </c>
       <c r="D8" s="2">
         <v>1.5</v>
       </c>
       <c r="E8" s="2">
         <f t="shared" si="0"/>
-        <v>1200</v>
+        <v>1500</v>
       </c>
       <c r="F8" t="s">
         <v>17</v>
@@ -1308,12 +1308,12 @@
       </c>
       <c r="C36" s="3">
         <f>SUM(C2:C35)</f>
-        <v>14410</v>
+        <v>14610</v>
       </c>
       <c r="D36" s="3"/>
       <c r="E36" s="8">
         <f>SUM(E2:E35)</f>
-        <v>20150</v>
+        <v>20450</v>
       </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
Doruceno: Rieger, Gasteiger, Eckerstorfer, Olsinger, Weissenbacher
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Obst.xlsx
+++ b/Obst.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://herzjesugym-my.sharepoint.com/personal/denis_holub_herzjesugym_at/Documents/Radtour 2026/mapa-rozvozu-ovoce/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="11_2687DF7FF0BCAF626073A8D655D9D6FCC967FD68" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="6_{4285B377-05AC-4B9B-81F5-C935964084AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-38510" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -792,7 +792,7 @@
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A7" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B7" t="s">
         <v>14</v>
@@ -813,7 +813,7 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A8" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B8" t="s">
         <v>16</v>
@@ -1040,7 +1040,7 @@
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A18" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B18" t="s">
         <v>40</v>
@@ -1085,7 +1085,7 @@
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A20" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B20" t="s">
         <v>45</v>
@@ -1242,7 +1242,7 @@
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A27" s="9" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B27" s="9" t="s">
         <v>62</v>

</xml_diff>

<commit_message>
Kupper 400 kg misto 500, Holzer odstranen (nepojede se)
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Obst.xlsx
+++ b/Obst.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://herzjesugym-my.sharepoint.com/personal/denis_holub_herzjesugym_at/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="14" documentId="13_ncr:1_{BD9264F1-AD0B-4A45-8BA2-60A535DA1E6A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{88885897-78BB-40FD-9891-17A97C1C1D59}"/>
+  <xr:revisionPtr revIDLastSave="16" documentId="13_ncr:1_{BD9264F1-AD0B-4A45-8BA2-60A535DA1E6A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7F7E92A7-A50E-4CA5-9A67-64CDC7CA4D71}"/>
   <bookViews>
-    <workbookView xWindow="15350" yWindow="14770" windowWidth="6380" windowHeight="3340" xr2:uid="{0E2E01CC-D03A-446C-9945-79710707EE2F}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{0E2E01CC-D03A-446C-9945-79710707EE2F}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="59">
   <si>
     <t>Weichsel</t>
   </si>
@@ -63,15 +63,6 @@
   </si>
   <si>
     <t>Bad Hall Eichenstraße 20</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Hannes Holzer </t>
-  </si>
-  <si>
-    <t>Köppel 103, 8251 Brucfk an der Lafnitz</t>
-  </si>
-  <si>
-    <t>Graz</t>
   </si>
   <si>
     <t>Johannes Eckerstorfer</t>
@@ -685,7 +676,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8369C171-C908-4428-93B9-D851AB8988B4}">
-  <dimension ref="A1:H54"/>
+  <dimension ref="A1:H53"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="19" bestFit="1" customWidth="1"/>
@@ -695,15 +686,15 @@
     <col min="6" max="6" width="31.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="B1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A2" s="6" t="b">
         <v>1</v>
       </c>
@@ -724,7 +715,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A3" s="6" t="b">
         <v>0</v>
       </c>
@@ -732,20 +723,20 @@
         <v>3</v>
       </c>
       <c r="C3" s="3">
-        <v>500</v>
+        <v>400</v>
       </c>
       <c r="D3" s="2">
         <v>1.5</v>
       </c>
       <c r="E3" s="2">
-        <f t="shared" ref="E3:E16" si="0">C3*D3</f>
-        <v>750</v>
+        <f t="shared" ref="E3:E15" si="0">C3*D3</f>
+        <v>600</v>
       </c>
       <c r="F3" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A4" s="6" t="b">
         <v>0</v>
       </c>
@@ -763,10 +754,10 @@
         <v>1500</v>
       </c>
       <c r="F4" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A5" s="6" t="b">
         <v>1</v>
       </c>
@@ -786,10 +777,10 @@
         <v>7</v>
       </c>
       <c r="G5" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A6" s="6" t="b">
         <v>0</v>
       </c>
@@ -797,345 +788,342 @@
         <v>8</v>
       </c>
       <c r="C6" s="3">
-        <v>500</v>
+        <v>350</v>
       </c>
       <c r="D6" s="2">
         <v>1.5</v>
       </c>
       <c r="E6" s="2">
         <f t="shared" si="0"/>
-        <v>750</v>
+        <v>525</v>
       </c>
       <c r="F6" t="s">
         <v>9</v>
       </c>
-      <c r="G6" t="s">
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A7" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="B7" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A7" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="B7" t="s">
-        <v>11</v>
-      </c>
       <c r="C7" s="3">
-        <v>350</v>
+        <v>800</v>
       </c>
       <c r="D7" s="2">
         <v>1.5</v>
       </c>
       <c r="E7" s="2">
         <f t="shared" si="0"/>
-        <v>525</v>
+        <v>1200</v>
       </c>
       <c r="F7" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
+        <v>36</v>
+      </c>
+      <c r="G7" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A8" s="6" t="b">
         <v>0</v>
       </c>
       <c r="B8" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="C8" s="3">
-        <v>800</v>
+        <v>300</v>
       </c>
       <c r="D8" s="2">
         <v>1.5</v>
       </c>
       <c r="E8" s="2">
         <f t="shared" si="0"/>
-        <v>1200</v>
-      </c>
-      <c r="F8" t="s">
-        <v>39</v>
+        <v>450</v>
+      </c>
+      <c r="F8" s="5" t="s">
+        <v>37</v>
       </c>
       <c r="G8" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A9" s="6" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B9" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C9" s="3">
-        <v>300</v>
+        <v>400</v>
       </c>
       <c r="D9" s="2">
         <v>1.5</v>
       </c>
       <c r="E9" s="2">
         <f t="shared" si="0"/>
-        <v>450</v>
-      </c>
-      <c r="F9" s="5" t="s">
-        <v>40</v>
-      </c>
-      <c r="G9" t="s">
+        <v>600</v>
+      </c>
+      <c r="F9" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A10" s="6" t="b">
+        <v>1</v>
+      </c>
+      <c r="B10" t="s">
+        <v>52</v>
+      </c>
+      <c r="C10" s="3">
+        <v>200</v>
+      </c>
+      <c r="D10" s="2">
+        <v>1.5</v>
+      </c>
+      <c r="E10" s="2">
+        <f>C10*D10</f>
+        <v>300</v>
+      </c>
+      <c r="F10" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="G10" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A11" s="6" t="b">
+        <v>1</v>
+      </c>
+      <c r="B11" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A10" s="6" t="b">
-        <v>1</v>
-      </c>
-      <c r="B10" t="s">
+      <c r="C11" s="3">
+        <v>100</v>
+      </c>
+      <c r="D11" s="2">
+        <v>1.5</v>
+      </c>
+      <c r="E11" s="2">
+        <v>170</v>
+      </c>
+      <c r="F11" t="s">
         <v>16</v>
       </c>
-      <c r="C10" s="3">
-        <v>400</v>
-      </c>
-      <c r="D10" s="2">
-        <v>1.5</v>
-      </c>
-      <c r="E10" s="2">
+      <c r="G11" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A12" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="B12" t="s">
+        <v>17</v>
+      </c>
+      <c r="C12" s="3">
+        <v>550</v>
+      </c>
+      <c r="D12" s="2">
+        <v>1.5</v>
+      </c>
+      <c r="E12" s="2">
         <f t="shared" si="0"/>
-        <v>600</v>
-      </c>
-      <c r="F10" s="1" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A11" s="6" t="b">
-        <v>1</v>
-      </c>
-      <c r="B11" t="s">
-        <v>55</v>
-      </c>
-      <c r="C11" s="3">
-        <v>200</v>
-      </c>
-      <c r="D11" s="2">
-        <v>1.5</v>
-      </c>
-      <c r="E11" s="2">
-        <f>C11*D11</f>
-        <v>300</v>
-      </c>
-      <c r="F11" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="G11" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A12" s="6" t="b">
-        <v>1</v>
-      </c>
-      <c r="B12" t="s">
+        <v>825</v>
+      </c>
+      <c r="F12" t="s">
         <v>18</v>
       </c>
-      <c r="C12" s="3">
-        <v>100</v>
-      </c>
-      <c r="D12" s="2">
-        <v>1.5</v>
-      </c>
-      <c r="E12" s="2">
-        <v>170</v>
-      </c>
-      <c r="F12" t="s">
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A13" s="6" t="b">
+        <v>1</v>
+      </c>
+      <c r="B13" t="s">
         <v>19</v>
       </c>
-      <c r="G12" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A13" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="B13" t="s">
-        <v>20</v>
-      </c>
       <c r="C13" s="3">
-        <v>550</v>
+        <v>900</v>
       </c>
       <c r="D13" s="2">
-        <v>1.5</v>
+        <v>1.25</v>
       </c>
       <c r="E13" s="2">
         <f t="shared" si="0"/>
-        <v>825</v>
-      </c>
-      <c r="F13" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
+        <v>1125</v>
+      </c>
+      <c r="F13" s="1" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A14" s="6" t="b">
         <v>1</v>
       </c>
       <c r="B14" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="C14" s="3">
-        <v>900</v>
+        <v>1000</v>
       </c>
       <c r="D14" s="2">
-        <v>1.25</v>
+        <v>1</v>
       </c>
       <c r="E14" s="2">
         <f t="shared" si="0"/>
-        <v>1125</v>
-      </c>
-      <c r="F14" s="1" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.35">
+        <v>1000</v>
+      </c>
+      <c r="F14" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A15" s="6" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B15" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="C15" s="3">
-        <v>1000</v>
+        <v>60</v>
       </c>
       <c r="D15" s="2">
-        <v>1</v>
+        <v>1.5</v>
       </c>
       <c r="E15" s="2">
         <f t="shared" si="0"/>
-        <v>1000</v>
+        <v>90</v>
       </c>
       <c r="F15" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.35">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A16" s="6" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B16" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C16" s="3">
-        <v>60</v>
+        <v>150</v>
       </c>
       <c r="D16" s="2">
         <v>1.5</v>
       </c>
       <c r="E16" s="2">
-        <f t="shared" si="0"/>
-        <v>90</v>
+        <f t="shared" ref="E16:E21" si="1">C16*D16</f>
+        <v>225</v>
       </c>
       <c r="F16" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.35">
+        <v>38</v>
+      </c>
+      <c r="G16" t="s">
+        <v>26</v>
+      </c>
+      <c r="H16">
+        <v>6607174862</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A17" s="6" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B17" t="s">
+        <v>27</v>
+      </c>
+      <c r="C17" s="3">
+        <v>600</v>
+      </c>
+      <c r="D17" s="2">
+        <v>1.4</v>
+      </c>
+      <c r="E17" s="2">
+        <f t="shared" si="1"/>
+        <v>840</v>
+      </c>
+      <c r="F17" t="s">
         <v>28</v>
       </c>
-      <c r="C17" s="3">
-        <v>150</v>
-      </c>
-      <c r="D17" s="2">
-        <v>1.5</v>
-      </c>
-      <c r="E17" s="2">
-        <f t="shared" ref="E17:E22" si="1">C17*D17</f>
-        <v>225</v>
-      </c>
-      <c r="F17" t="s">
-        <v>41</v>
-      </c>
-      <c r="G17" t="s">
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A18" s="6" t="b">
+        <v>1</v>
+      </c>
+      <c r="B18" t="s">
         <v>29</v>
       </c>
-      <c r="H17">
-        <v>6607174862</v>
-      </c>
-    </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A18" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="B18" t="s">
-        <v>30</v>
-      </c>
       <c r="C18" s="3">
-        <v>600</v>
+        <v>3000</v>
       </c>
       <c r="D18" s="2">
-        <v>1.4</v>
+        <v>1.3</v>
       </c>
       <c r="E18" s="2">
         <f t="shared" si="1"/>
-        <v>840</v>
-      </c>
-      <c r="F18" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.35">
+        <v>3900</v>
+      </c>
+      <c r="F18" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="G18" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A19" s="6" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B19" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="C19" s="3">
-        <v>3000</v>
+        <v>500</v>
       </c>
       <c r="D19" s="2">
-        <v>1.3</v>
+        <v>1.5</v>
       </c>
       <c r="E19" s="2">
         <f t="shared" si="1"/>
-        <v>3900</v>
-      </c>
-      <c r="F19" s="7" t="s">
-        <v>46</v>
+        <v>750</v>
+      </c>
+      <c r="F19" t="s">
+        <v>39</v>
       </c>
       <c r="G19" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.35">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A20" s="6" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B20" t="s">
         <v>33</v>
       </c>
       <c r="C20" s="3">
-        <v>500</v>
+        <v>200</v>
       </c>
       <c r="D20" s="2">
         <v>1.5</v>
       </c>
       <c r="E20" s="2">
         <f t="shared" si="1"/>
-        <v>750</v>
-      </c>
-      <c r="F20" t="s">
-        <v>42</v>
-      </c>
-      <c r="G20" t="s">
+        <v>300</v>
+      </c>
+      <c r="F20" s="4" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A21" s="6" t="b">
+        <v>1</v>
+      </c>
+      <c r="B21" t="s">
         <v>34</v>
-      </c>
-    </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A21" s="6" t="b">
-        <v>1</v>
-      </c>
-      <c r="B21" t="s">
-        <v>36</v>
       </c>
       <c r="C21" s="3">
         <v>200</v>
@@ -1147,148 +1135,132 @@
         <f t="shared" si="1"/>
         <v>300</v>
       </c>
-      <c r="F21" s="4" t="s">
+      <c r="F21" s="5" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A22" s="6" t="b">
+        <v>1</v>
+      </c>
+      <c r="B22" t="s">
         <v>35</v>
       </c>
-    </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A22" s="6" t="b">
-        <v>1</v>
-      </c>
-      <c r="B22" t="s">
-        <v>37</v>
-      </c>
       <c r="C22" s="3">
-        <v>200</v>
+        <v>540</v>
       </c>
       <c r="D22" s="2">
         <v>1.5</v>
       </c>
       <c r="E22" s="2">
-        <f t="shared" si="1"/>
-        <v>300</v>
+        <f>C22*D22</f>
+        <v>810</v>
       </c>
       <c r="F22" s="5" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.35">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A23" s="6" t="b">
         <v>1</v>
       </c>
       <c r="B23" t="s">
-        <v>38</v>
+        <v>45</v>
       </c>
       <c r="C23" s="3">
-        <v>540</v>
+        <v>100</v>
       </c>
       <c r="D23" s="2">
         <v>1.5</v>
       </c>
       <c r="E23" s="2">
         <f>C23*D23</f>
-        <v>810</v>
-      </c>
-      <c r="F23" s="5" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.35">
+        <v>150</v>
+      </c>
+      <c r="F23" s="8" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A24" s="6" t="b">
         <v>1</v>
       </c>
       <c r="B24" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C24" s="3">
-        <v>100</v>
+        <v>360</v>
       </c>
       <c r="D24" s="2">
-        <v>1.5</v>
+        <f>400/360</f>
+        <v>1.1111111111111112</v>
       </c>
       <c r="E24" s="2">
         <f>C24*D24</f>
-        <v>150</v>
+        <v>400</v>
       </c>
       <c r="F24" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="G24" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A25" s="6" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B25" t="s">
-        <v>50</v>
-      </c>
-      <c r="C25" s="3">
-        <v>360</v>
-      </c>
-      <c r="D25" s="2">
-        <f>400/360</f>
-        <v>1.1111111111111112</v>
-      </c>
-      <c r="E25" s="2">
+        <v>56</v>
+      </c>
+      <c r="C25">
+        <v>1000</v>
+      </c>
+      <c r="D25">
+        <v>1.5</v>
+      </c>
+      <c r="E25">
         <f>C25*D25</f>
-        <v>400</v>
-      </c>
-      <c r="F25" s="8" t="s">
-        <v>51</v>
+        <v>1500</v>
+      </c>
+      <c r="F25" t="s">
+        <v>57</v>
       </c>
       <c r="G25" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.35">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A26" s="6" t="b">
         <v>0</v>
       </c>
-      <c r="B26" t="s">
-        <v>59</v>
-      </c>
-      <c r="C26">
-        <v>1000</v>
-      </c>
-      <c r="D26">
-        <v>1.5</v>
-      </c>
-      <c r="E26">
-        <f>C26*D26</f>
-        <v>1500</v>
-      </c>
-      <c r="F26" t="s">
-        <v>60</v>
-      </c>
-      <c r="G26" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.35">
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A27" s="6" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A28" s="6" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A29" s="6" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A30" s="6" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A31" s="6" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A32" s="6" t="b">
         <v>0</v>
       </c>
@@ -1307,20 +1279,20 @@
       <c r="A35" s="6" t="b">
         <v>0</v>
       </c>
+      <c r="C35" s="3">
+        <f>SUM(C2:C34)</f>
+        <v>13510</v>
+      </c>
+      <c r="D35" s="3"/>
+      <c r="E35" s="9">
+        <f>SUM(E2:E34)</f>
+        <v>18800</v>
+      </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A36" s="6" t="b">
         <v>0</v>
       </c>
-      <c r="C36" s="3">
-        <f>SUM(C2:C35)</f>
-        <v>14110</v>
-      </c>
-      <c r="D36" s="3"/>
-      <c r="E36" s="9">
-        <f>SUM(E2:E35)</f>
-        <v>19700</v>
-      </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A37" s="6" t="b">
@@ -1407,20 +1379,15 @@
         <v>0</v>
       </c>
     </row>
-    <row r="54" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A54" s="6" t="b">
-        <v>0</v>
-      </c>
-    </row>
   </sheetData>
-  <conditionalFormatting sqref="A2:G35">
+  <conditionalFormatting sqref="A2:G34">
     <cfRule type="expression" dxfId="0" priority="1" stopIfTrue="1">
       <formula>$A2=TRUE()</formula>
     </cfRule>
   </conditionalFormatting>
   <hyperlinks>
-    <hyperlink ref="F10" r:id="rId1" display="https://www.google.com/maps/place/data=!4m2!3m1!1s0x47747715538db01d:0x16d28a73419a5295?sa=X&amp;ved=1t:8290&amp;ictx=111" xr:uid="{D642E8DC-BBBD-4F4B-A4DC-252C3C0D6734}"/>
-    <hyperlink ref="F14" r:id="rId2" display="https://www.google.com/maps/place/data=!4m2!3m1!1s0x4773af04442266fd:0x116ce1c69494bb32?sa=X&amp;ved=1t:8290&amp;ictx=111" xr:uid="{1745D04A-32DE-4B22-BE2A-10ABC6DB20F4}"/>
+    <hyperlink ref="F9" r:id="rId1" display="https://www.google.com/maps/place/data=!4m2!3m1!1s0x47747715538db01d:0x16d28a73419a5295?sa=X&amp;ved=1t:8290&amp;ictx=111" xr:uid="{D642E8DC-BBBD-4F4B-A4DC-252C3C0D6734}"/>
+    <hyperlink ref="F13" r:id="rId2" display="https://www.google.com/maps/place/data=!4m2!3m1!1s0x4773af04442266fd:0x116ce1c69494bb32?sa=X&amp;ved=1t:8290&amp;ictx=111" xr:uid="{1745D04A-32DE-4B22-BE2A-10ABC6DB20F4}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId3"/>

</xml_diff>

<commit_message>
Kupper 400 kg, Holzer odstranen (oprava na aktualni data)
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Obst.xlsx
+++ b/Obst.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://herzjesugym-my.sharepoint.com/personal/denis_holub_herzjesugym_at/Documents/Radtour 2026/mapa-rozvozu-ovoce/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://herzjesugym-my.sharepoint.com/personal/denis_holub_herzjesugym_at/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="6_{4285B377-05AC-4B9B-81F5-C935964084AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="2" documentId="6_{4285B377-05AC-4B9B-81F5-C935964084AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FD21D797-E820-45A5-A622-3DAE06255763}"/>
   <bookViews>
-    <workbookView xWindow="-38510" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="61">
   <si>
     <t>Geliefert</t>
   </si>
@@ -66,15 +66,6 @@
   </si>
   <si>
     <t>inkl. 40 € Trinkgeld</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Hannes Holzer </t>
-  </si>
-  <si>
-    <t>Köppel 103, 8251 Brucfk an der Lafnitz</t>
-  </si>
-  <si>
-    <t>Graz</t>
   </si>
   <si>
     <t>Johannes Eckerstorfer</t>
@@ -232,8 +223,8 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
-    <numFmt numFmtId="44" formatCode="_-&quot;€&quot;\ * #,##0.00_-;\-&quot;€&quot;\ * #,##0.00_-;_-&quot;€&quot;\ * &quot;-&quot;??_-;_-@_-"/>
-    <numFmt numFmtId="164" formatCode="0\ &quot;kg&quot;"/>
+    <numFmt numFmtId="164" formatCode="_-&quot;€&quot;\ * #,##0.00_-;\-&quot;€&quot;\ * #,##0.00_-;_-&quot;€&quot;\ * &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="165" formatCode="0\ &quot;kg&quot;"/>
   </numFmts>
   <fonts count="7" x14ac:knownFonts="1">
     <font>
@@ -301,19 +292,19 @@
   </borders>
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="44" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="2"/>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="3">
@@ -662,7 +653,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H54"/>
+  <dimension ref="A1:H53"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="19" bestFit="1" customWidth="1"/>
@@ -672,7 +663,7 @@
     <col min="6" max="6" width="31.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -680,7 +671,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A2" t="b">
         <v>1</v>
       </c>
@@ -701,7 +692,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A3" t="b">
         <v>0</v>
       </c>
@@ -709,20 +700,20 @@
         <v>4</v>
       </c>
       <c r="C3" s="3">
-        <v>500</v>
+        <v>400</v>
       </c>
       <c r="D3" s="2">
         <v>1.5</v>
       </c>
       <c r="E3" s="2">
         <f>C3*D3</f>
-        <v>750</v>
+        <v>600</v>
       </c>
       <c r="F3" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A4" t="b">
         <v>0</v>
       </c>
@@ -743,7 +734,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A5" t="b">
         <v>1</v>
       </c>
@@ -766,121 +757,121 @@
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A6" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B6" t="s">
         <v>11</v>
       </c>
       <c r="C6" s="3">
-        <v>500</v>
+        <v>350</v>
       </c>
       <c r="D6" s="2">
         <v>1.5</v>
       </c>
       <c r="E6" s="2">
-        <f t="shared" ref="E6:E11" si="0">C6*D6</f>
-        <v>750</v>
+        <f t="shared" ref="E6:E10" si="0">C6*D6</f>
+        <v>525</v>
       </c>
       <c r="F6" t="s">
         <v>12</v>
       </c>
-      <c r="G6" t="s">
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A7" t="b">
+        <v>1</v>
+      </c>
+      <c r="B7" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A7" t="b">
-        <v>1</v>
-      </c>
-      <c r="B7" t="s">
-        <v>14</v>
-      </c>
       <c r="C7" s="3">
-        <v>350</v>
+        <v>1000</v>
       </c>
       <c r="D7" s="2">
         <v>1.5</v>
       </c>
       <c r="E7" s="2">
         <f t="shared" si="0"/>
-        <v>525</v>
+        <v>1500</v>
       </c>
       <c r="F7" t="s">
+        <v>14</v>
+      </c>
+      <c r="G7" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A8" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B8" t="s">
         <v>16</v>
       </c>
       <c r="C8" s="3">
-        <v>1000</v>
+        <v>300</v>
       </c>
       <c r="D8" s="2">
         <v>1.5</v>
       </c>
       <c r="E8" s="2">
         <f t="shared" si="0"/>
-        <v>1500</v>
-      </c>
-      <c r="F8" t="s">
+        <v>450</v>
+      </c>
+      <c r="F8" s="5" t="s">
         <v>17</v>
       </c>
       <c r="G8" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A9" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B9" t="s">
         <v>19</v>
       </c>
       <c r="C9" s="3">
-        <v>300</v>
+        <v>400</v>
       </c>
       <c r="D9" s="2">
         <v>1.5</v>
       </c>
       <c r="E9" s="2">
         <f t="shared" si="0"/>
-        <v>450</v>
-      </c>
-      <c r="F9" s="5" t="s">
+        <v>600</v>
+      </c>
+      <c r="F9" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="G9" t="s">
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A10" t="b">
+        <v>1</v>
+      </c>
+      <c r="B10" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A10" t="b">
-        <v>1</v>
-      </c>
-      <c r="B10" t="s">
-        <v>22</v>
-      </c>
       <c r="C10" s="3">
-        <v>400</v>
+        <v>200</v>
       </c>
       <c r="D10" s="2">
         <v>1.5</v>
       </c>
       <c r="E10" s="2">
         <f t="shared" si="0"/>
-        <v>600</v>
+        <v>300</v>
       </c>
       <c r="F10" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="G10" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A11" t="b">
         <v>1</v>
       </c>
@@ -888,178 +879,178 @@
         <v>24</v>
       </c>
       <c r="C11" s="3">
-        <v>200</v>
+        <v>100</v>
       </c>
       <c r="D11" s="2">
         <v>1.5</v>
       </c>
       <c r="E11" s="2">
-        <f t="shared" si="0"/>
-        <v>300</v>
-      </c>
-      <c r="F11" s="1" t="s">
+        <v>170</v>
+      </c>
+      <c r="F11" t="s">
         <v>25</v>
       </c>
       <c r="G11" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A12" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B12" t="s">
         <v>27</v>
       </c>
       <c r="C12" s="3">
-        <v>100</v>
+        <v>550</v>
       </c>
       <c r="D12" s="2">
         <v>1.5</v>
       </c>
       <c r="E12" s="2">
-        <v>170</v>
+        <f t="shared" ref="E12:E26" si="1">C12*D12</f>
+        <v>825</v>
       </c>
       <c r="F12" t="s">
         <v>28</v>
       </c>
-      <c r="G12" t="s">
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A13" t="b">
+        <v>1</v>
+      </c>
+      <c r="B13" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A13" t="b">
-        <v>0</v>
-      </c>
-      <c r="B13" t="s">
+      <c r="C13" s="3">
+        <v>900</v>
+      </c>
+      <c r="D13" s="2">
+        <v>1.25</v>
+      </c>
+      <c r="E13" s="2">
+        <f t="shared" si="1"/>
+        <v>1125</v>
+      </c>
+      <c r="F13" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="C13" s="3">
-        <v>550</v>
-      </c>
-      <c r="D13" s="2">
-        <v>1.5</v>
-      </c>
-      <c r="E13" s="2">
-        <f t="shared" ref="E13:E27" si="1">C13*D13</f>
-        <v>825</v>
-      </c>
-      <c r="F13" t="s">
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A14" t="b">
+        <v>1</v>
+      </c>
+      <c r="B14" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A14" t="b">
-        <v>1</v>
-      </c>
-      <c r="B14" t="s">
-        <v>32</v>
-      </c>
       <c r="C14" s="3">
-        <v>900</v>
+        <v>1000</v>
       </c>
       <c r="D14" s="2">
-        <v>1.25</v>
+        <v>1</v>
       </c>
       <c r="E14" s="2">
         <f t="shared" si="1"/>
-        <v>1125</v>
-      </c>
-      <c r="F14" s="1" t="s">
+        <v>1000</v>
+      </c>
+      <c r="F14" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A15" t="b">
+        <v>0</v>
+      </c>
+      <c r="B15" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A15" t="b">
-        <v>1</v>
-      </c>
-      <c r="B15" t="s">
-        <v>34</v>
-      </c>
       <c r="C15" s="3">
-        <v>1000</v>
+        <v>60</v>
       </c>
       <c r="D15" s="2">
-        <v>1</v>
+        <v>1.5</v>
       </c>
       <c r="E15" s="2">
         <f t="shared" si="1"/>
-        <v>1000</v>
+        <v>90</v>
       </c>
       <c r="F15" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A16" t="b">
+        <v>1</v>
+      </c>
+      <c r="B16" t="s">
         <v>35</v>
       </c>
-    </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A16" t="b">
-        <v>0</v>
-      </c>
-      <c r="B16" t="s">
-        <v>36</v>
-      </c>
       <c r="C16" s="3">
-        <v>60</v>
+        <v>150</v>
       </c>
       <c r="D16" s="2">
         <v>1.5</v>
       </c>
       <c r="E16" s="2">
         <f t="shared" si="1"/>
-        <v>90</v>
+        <v>225</v>
       </c>
       <c r="F16" t="s">
+        <v>32</v>
+      </c>
+      <c r="G16" t="s">
+        <v>36</v>
+      </c>
+      <c r="H16">
+        <v>6607174862</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A17" t="b">
+        <v>1</v>
+      </c>
+      <c r="B17" t="s">
         <v>37</v>
       </c>
-    </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A17" t="b">
-        <v>1</v>
-      </c>
-      <c r="B17" t="s">
-        <v>38</v>
-      </c>
       <c r="C17" s="3">
-        <v>150</v>
+        <v>600</v>
       </c>
       <c r="D17" s="2">
-        <v>1.5</v>
+        <v>1.4</v>
       </c>
       <c r="E17" s="2">
         <f t="shared" si="1"/>
-        <v>225</v>
+        <v>840</v>
       </c>
       <c r="F17" t="s">
-        <v>35</v>
-      </c>
-      <c r="G17" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A18" t="b">
+        <v>1</v>
+      </c>
+      <c r="B18" t="s">
         <v>39</v>
       </c>
-      <c r="H17">
-        <v>6607174862</v>
-      </c>
-    </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A18" t="b">
-        <v>1</v>
-      </c>
-      <c r="B18" t="s">
-        <v>40</v>
-      </c>
       <c r="C18" s="3">
-        <v>600</v>
+        <v>3000</v>
       </c>
       <c r="D18" s="2">
-        <v>1.4</v>
+        <v>1.3</v>
       </c>
       <c r="E18" s="2">
         <f t="shared" si="1"/>
-        <v>840</v>
-      </c>
-      <c r="F18" t="s">
+        <v>3900</v>
+      </c>
+      <c r="F18" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="G18" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A19" t="b">
         <v>1</v>
       </c>
@@ -1067,23 +1058,23 @@
         <v>42</v>
       </c>
       <c r="C19" s="3">
-        <v>3000</v>
+        <v>500</v>
       </c>
       <c r="D19" s="2">
-        <v>1.3</v>
+        <v>1.5</v>
       </c>
       <c r="E19" s="2">
         <f t="shared" si="1"/>
-        <v>3900</v>
-      </c>
-      <c r="F19" s="6" t="s">
+        <v>750</v>
+      </c>
+      <c r="F19" t="s">
         <v>43</v>
       </c>
       <c r="G19" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A20" t="b">
         <v>1</v>
       </c>
@@ -1091,28 +1082,25 @@
         <v>45</v>
       </c>
       <c r="C20" s="3">
-        <v>500</v>
+        <v>200</v>
       </c>
       <c r="D20" s="2">
         <v>1.5</v>
       </c>
       <c r="E20" s="2">
         <f t="shared" si="1"/>
-        <v>750</v>
-      </c>
-      <c r="F20" t="s">
+        <v>300</v>
+      </c>
+      <c r="F20" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="G20" t="s">
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A21" t="b">
+        <v>1</v>
+      </c>
+      <c r="B21" t="s">
         <v>47</v>
-      </c>
-    </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A21" t="b">
-        <v>1</v>
-      </c>
-      <c r="B21" t="s">
-        <v>48</v>
       </c>
       <c r="C21" s="3">
         <v>200</v>
@@ -1124,165 +1112,149 @@
         <f t="shared" si="1"/>
         <v>300</v>
       </c>
-      <c r="F21" s="4" t="s">
+      <c r="F21" s="5" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A22" t="b">
+        <v>1</v>
+      </c>
+      <c r="B22" t="s">
         <v>49</v>
       </c>
-    </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A22" t="b">
-        <v>1</v>
-      </c>
-      <c r="B22" t="s">
-        <v>50</v>
-      </c>
       <c r="C22" s="3">
-        <v>200</v>
+        <v>540</v>
       </c>
       <c r="D22" s="2">
         <v>1.5</v>
       </c>
       <c r="E22" s="2">
         <f t="shared" si="1"/>
-        <v>300</v>
+        <v>810</v>
       </c>
       <c r="F22" s="5" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A23" t="b">
+        <v>1</v>
+      </c>
+      <c r="B23" t="s">
         <v>51</v>
       </c>
-    </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A23" t="b">
-        <v>1</v>
-      </c>
-      <c r="B23" t="s">
-        <v>52</v>
-      </c>
       <c r="C23" s="3">
-        <v>540</v>
+        <v>100</v>
       </c>
       <c r="D23" s="2">
         <v>1.5</v>
       </c>
       <c r="E23" s="2">
         <f t="shared" si="1"/>
-        <v>810</v>
-      </c>
-      <c r="F23" s="5" t="s">
+        <v>150</v>
+      </c>
+      <c r="F23" s="7" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A24" t="b">
+        <v>1</v>
+      </c>
+      <c r="B24" t="s">
         <v>53</v>
       </c>
-    </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A24" t="b">
-        <v>1</v>
-      </c>
-      <c r="B24" t="s">
-        <v>54</v>
-      </c>
       <c r="C24" s="3">
-        <v>100</v>
+        <v>360</v>
       </c>
       <c r="D24" s="2">
-        <v>1.5</v>
+        <f>400/360</f>
+        <v>1.1111111111111112</v>
       </c>
       <c r="E24" s="2">
         <f t="shared" si="1"/>
-        <v>150</v>
+        <v>400</v>
       </c>
       <c r="F24" s="7" t="s">
+        <v>54</v>
+      </c>
+      <c r="G24" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A25" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B25" t="s">
         <v>56</v>
       </c>
-      <c r="C25" s="3">
-        <v>360</v>
-      </c>
-      <c r="D25" s="2">
-        <f>400/360</f>
-        <v>1.1111111111111112</v>
-      </c>
-      <c r="E25" s="2">
+      <c r="C25">
+        <v>1000</v>
+      </c>
+      <c r="D25">
+        <v>1.5</v>
+      </c>
+      <c r="E25">
         <f t="shared" si="1"/>
-        <v>400</v>
-      </c>
-      <c r="F25" s="7" t="s">
+        <v>1500</v>
+      </c>
+      <c r="F25" t="s">
         <v>57</v>
       </c>
       <c r="G25" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A26" t="b">
-        <v>0</v>
-      </c>
-      <c r="B26" t="s">
+    <row r="26" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A26" s="9" t="b">
+        <v>1</v>
+      </c>
+      <c r="B26" s="9" t="s">
         <v>59</v>
       </c>
-      <c r="C26">
-        <v>1000</v>
-      </c>
-      <c r="D26">
-        <v>1.5</v>
-      </c>
-      <c r="E26">
-        <f t="shared" si="1"/>
-        <v>1500</v>
-      </c>
-      <c r="F26" t="s">
-        <v>60</v>
-      </c>
-      <c r="G26" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A27" s="9" t="b">
-        <v>1</v>
-      </c>
-      <c r="B27" s="9" t="s">
-        <v>62</v>
-      </c>
-      <c r="C27" s="9">
+      <c r="C26" s="9">
         <v>300</v>
       </c>
-      <c r="D27" s="9">
-        <v>1.5</v>
-      </c>
-      <c r="E27" s="9">
+      <c r="D26" s="9">
+        <v>1.5</v>
+      </c>
+      <c r="E26" s="9">
         <f t="shared" si="1"/>
         <v>450</v>
       </c>
-      <c r="F27" s="9" t="s">
-        <v>63</v>
-      </c>
-      <c r="G27" s="9"/>
-    </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="F26" s="9" t="s">
+        <v>60</v>
+      </c>
+      <c r="G26" s="9"/>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A27" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A28" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A29" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A30" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A31" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A32" t="b">
         <v>0</v>
       </c>
@@ -1301,20 +1273,20 @@
       <c r="A35" t="b">
         <v>0</v>
       </c>
+      <c r="C35" s="3">
+        <f>SUM(C2:C34)</f>
+        <v>14010</v>
+      </c>
+      <c r="D35" s="3"/>
+      <c r="E35" s="8">
+        <f>SUM(E2:E34)</f>
+        <v>19550</v>
+      </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A36" t="b">
         <v>0</v>
       </c>
-      <c r="C36" s="3">
-        <f>SUM(C2:C35)</f>
-        <v>14610</v>
-      </c>
-      <c r="D36" s="3"/>
-      <c r="E36" s="8">
-        <f>SUM(E2:E35)</f>
-        <v>20450</v>
-      </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A37" t="b">
@@ -1401,20 +1373,15 @@
         <v>0</v>
       </c>
     </row>
-    <row r="54" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A54" t="b">
-        <v>0</v>
-      </c>
-    </row>
   </sheetData>
-  <conditionalFormatting sqref="A2:G35">
+  <conditionalFormatting sqref="A2:G34">
     <cfRule type="expression" dxfId="0" priority="1" stopIfTrue="1">
       <formula>$A2=TRUE()</formula>
     </cfRule>
   </conditionalFormatting>
   <hyperlinks>
-    <hyperlink ref="F10" r:id="rId1" display="https://www.google.com/maps/place/data=!4m2!3m1!1s0x47747715538db01d:0x16d28a73419a5295?sa=X&amp;ved=1t:8290&amp;ictx=111" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
-    <hyperlink ref="F14" r:id="rId2" display="https://www.google.com/maps/place/data=!4m2!3m1!1s0x4773af04442266fd:0x116ce1c69494bb32?sa=X&amp;ved=1t:8290&amp;ictx=111" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
+    <hyperlink ref="F9" r:id="rId1" display="https://www.google.com/maps/place/data=!4m2!3m1!1s0x47747715538db01d:0x16d28a73419a5295?sa=X&amp;ved=1t:8290&amp;ictx=111" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
+    <hyperlink ref="F13" r:id="rId2" display="https://www.google.com/maps/place/data=!4m2!3m1!1s0x4773af04442266fd:0x116ce1c69494bb32?sa=X&amp;ved=1t:8290&amp;ictx=111" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait"/>

</xml_diff>

<commit_message>
Doruceno: Eigner, Mitteregger 950 kg, Burgstaller 640 kg, Kupper 410 kg/600 EUR, Werner
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Obst.xlsx
+++ b/Obst.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://herzjesugym-my.sharepoint.com/personal/denis_holub_herzjesugym_at/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="10" documentId="6_{4285B377-05AC-4B9B-81F5-C935964084AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1B24B466-EEB3-4403-B3F4-0A050D45392A}"/>
+  <xr:revisionPtr revIDLastSave="11" documentId="6_{4285B377-05AC-4B9B-81F5-C935964084AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9168FC42-E469-44A5-9FA1-056CA04D195B}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -958,7 +958,7 @@
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A15" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B15" t="s">
         <v>33</v>

</xml_diff>

<commit_message>
Novy zakaznik: Briendl Michael, 250 kg, Sattledt
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Obst.xlsx
+++ b/Obst.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://herzjesugym-my.sharepoint.com/personal/denis_holub_herzjesugym_at/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="11" documentId="6_{4285B377-05AC-4B9B-81F5-C935964084AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9168FC42-E469-44A5-9FA1-056CA04D195B}"/>
+  <xr:revisionPtr revIDLastSave="20" documentId="6_{4285B377-05AC-4B9B-81F5-C935964084AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{66D0287D-5E36-4E6C-B8AC-7A9CAF1850E4}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="63">
   <si>
     <t>Geliefert</t>
   </si>
@@ -216,6 +216,12 @@
   </si>
   <si>
     <t>Guntendorf 10, 4550 Kremsmünster</t>
+  </si>
+  <si>
+    <t>Briendl Michael</t>
+  </si>
+  <si>
+    <t>Oberautal 12, 4642 Sattledt</t>
   </si>
 </sst>
 </file>
@@ -653,7 +659,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H53"/>
+  <dimension ref="A1:H54"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="19" bestFit="1" customWidth="1"/>
@@ -1258,91 +1264,107 @@
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A33" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A34" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A35" t="b">
         <v>0</v>
       </c>
-      <c r="C35" s="3">
-        <f>SUM(C2:C34)</f>
-        <v>14060</v>
-      </c>
-      <c r="D35" s="3"/>
-      <c r="E35" s="8">
-        <f>SUM(E2:E34)</f>
-        <v>19610</v>
-      </c>
-    </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="B35" t="s">
+        <v>61</v>
+      </c>
+      <c r="C35">
+        <v>250</v>
+      </c>
+      <c r="D35">
+        <v>1.5</v>
+      </c>
+      <c r="E35">
+        <f>C35*D35</f>
+        <v>375</v>
+      </c>
+      <c r="F35" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A36" t="b">
         <v>0</v>
       </c>
-    </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="C36" s="3">
+        <f>SUM(C2:C35)</f>
+        <v>14310</v>
+      </c>
+      <c r="D36" s="3"/>
+      <c r="E36" s="8">
+        <f>SUM(E2:E35)</f>
+        <v>19985</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A37" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A38" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A39" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A40" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A41" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A42" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A43" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A44" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A45" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A46" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A47" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A48" t="b">
         <v>0</v>
       </c>
@@ -1372,8 +1394,13 @@
         <v>0</v>
       </c>
     </row>
+    <row r="54" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A54" t="b">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="A2:G34">
+  <conditionalFormatting sqref="A2:G35">
     <cfRule type="expression" dxfId="0" priority="1" stopIfTrue="1">
       <formula>$A2=TRUE()</formula>
     </cfRule>

</xml_diff>

<commit_message>
Pridana objednavka: Hedegg Destillerie, 1000 kg, St. Johann im Pongau
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Obst.xlsx
+++ b/Obst.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://herzjesugym-my.sharepoint.com/personal/denis_holub_herzjesugym_at/Documents/Radtour 2026/mapa-rozvozu-ovoce/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="6_{4285B377-05AC-4B9B-81F5-C935964084AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="11_459F08A75986AC4C3672A8D655D9D6FCD960ED00" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-38510" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="66">
   <si>
     <t>Geliefert</t>
   </si>
@@ -225,6 +225,12 @@
   </si>
   <si>
     <t>Guntendorf 10, 4550 Kremsmünster</t>
+  </si>
+  <si>
+    <t>Hedegg Destillerie</t>
+  </si>
+  <si>
+    <t>Hedegg 35, 5600 St. Johann im Pongau</t>
   </si>
 </sst>
 </file>
@@ -941,7 +947,7 @@
         <v>1.5</v>
       </c>
       <c r="E13" s="2">
-        <f t="shared" ref="E13:E27" si="1">C13*D13</f>
+        <f t="shared" ref="E13:E28" si="1">C13*D13</f>
         <v>825</v>
       </c>
       <c r="F13" t="s">
@@ -1263,9 +1269,26 @@
       <c r="G27" s="9"/>
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A28" t="b">
-        <v>0</v>
-      </c>
+      <c r="A28" s="9" t="b">
+        <v>0</v>
+      </c>
+      <c r="B28" s="9" t="s">
+        <v>64</v>
+      </c>
+      <c r="C28" s="9">
+        <v>1000</v>
+      </c>
+      <c r="D28" s="9">
+        <v>1.5</v>
+      </c>
+      <c r="E28" s="9">
+        <f t="shared" si="1"/>
+        <v>1500</v>
+      </c>
+      <c r="F28" s="9" t="s">
+        <v>65</v>
+      </c>
+      <c r="G28" s="9"/>
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A29" t="b">
@@ -1308,12 +1331,12 @@
       </c>
       <c r="C36" s="3">
         <f>SUM(C2:C35)</f>
-        <v>14610</v>
+        <v>15610</v>
       </c>
       <c r="D36" s="3"/>
       <c r="E36" s="8">
         <f>SUM(E2:E35)</f>
-        <v>20450</v>
+        <v>21950</v>
       </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
Doruceno: Wolfgang Dexelheimer, 300 kg
</commit_message>
<xml_diff>
--- a/Obst.xlsx
+++ b/Obst.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://herzjesugym-my.sharepoint.com/personal/denis_holub_herzjesugym_at/Documents/Radtour 2026/mapa-rozvozu-ovoce/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="11_2687E87FFCD2F7693C72A8D65576C6B9F311FD35" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="11_459FEBA72342A575BE72A8D655D9D6FCD960F2F2" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-38510" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1520" yWindow="1520" windowWidth="28800" windowHeight="15370" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -815,7 +815,7 @@
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A8" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B8" t="s">
         <v>16</v>

</xml_diff>

<commit_message>
Nove objednavky: Zwetschken 600 kg (Gasthof Troadkastn), Birnen Williams 1000 kg (Eigner)
</commit_message>
<xml_diff>
--- a/Obst.xlsx
+++ b/Obst.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://herzjesugym-my.sharepoint.com/personal/denis_holub_herzjesugym_at/Documents/Radtour 2026/mapa-rozvozu-ovoce/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="11_A781F6A7B40E46671272A8D655D9D6FC3962F42C" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="11_26872C97A4337C719472A8D655D9D6FCC967E65A" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1520" yWindow="1520" windowWidth="28800" windowHeight="15370" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="72">
   <si>
     <t>Geliefert</t>
   </si>
@@ -228,6 +228,27 @@
   </si>
   <si>
     <t>Oberautal 12, 4642 Sattledt</t>
+  </si>
+  <si>
+    <t>Zwetschken</t>
+  </si>
+  <si>
+    <t>Gasthof Troadkastn</t>
+  </si>
+  <si>
+    <t>4894 Oberhofen am Irrsee</t>
+  </si>
+  <si>
+    <t>telefonisch bestellt +43 664 4233933 – Preis ergänzen</t>
+  </si>
+  <si>
+    <t>Birnen Williams</t>
+  </si>
+  <si>
+    <t>Haagweg 7, 5550 Radstadt</t>
+  </si>
+  <si>
+    <t>Preis ergänzen</t>
   </si>
 </sst>
 </file>
@@ -919,7 +940,7 @@
         <v>1.5</v>
       </c>
       <c r="E12" s="2">
-        <f t="shared" ref="E12:E27" si="0">C12*D12</f>
+        <f t="shared" ref="E12:E28" si="0">C12*D12</f>
         <v>960</v>
       </c>
       <c r="F12" t="s">
@@ -1263,9 +1284,26 @@
       <c r="G27" s="9"/>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A28" t="b">
-        <v>0</v>
-      </c>
+      <c r="A28" s="9" t="b">
+        <v>1</v>
+      </c>
+      <c r="B28" s="9" t="s">
+        <v>63</v>
+      </c>
+      <c r="C28" s="9">
+        <v>300</v>
+      </c>
+      <c r="D28" s="9">
+        <v>1.5</v>
+      </c>
+      <c r="E28" s="9">
+        <f t="shared" si="0"/>
+        <v>450</v>
+      </c>
+      <c r="F28" s="9" t="s">
+        <v>64</v>
+      </c>
+      <c r="G28" s="9"/>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A29" t="b">
@@ -1273,13 +1311,35 @@
       </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A30" t="b">
-        <v>0</v>
-      </c>
+      <c r="A30" s="9" t="b">
+        <v>0</v>
+      </c>
+      <c r="B30" s="9" t="s">
+        <v>65</v>
+      </c>
+      <c r="C30" s="9"/>
+      <c r="D30" s="9"/>
+      <c r="E30" s="9"/>
+      <c r="F30" s="9"/>
+      <c r="G30" s="9"/>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A31" t="b">
-        <v>0</v>
+      <c r="A31" s="9" t="b">
+        <v>0</v>
+      </c>
+      <c r="B31" s="9" t="s">
+        <v>66</v>
+      </c>
+      <c r="C31" s="9">
+        <v>600</v>
+      </c>
+      <c r="D31" s="9"/>
+      <c r="E31" s="9"/>
+      <c r="F31" s="9" t="s">
+        <v>67</v>
+      </c>
+      <c r="G31" s="9" t="s">
+        <v>68</v>
       </c>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.35">
@@ -1287,44 +1347,50 @@
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A33" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A34" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A33" s="9" t="b">
+        <v>0</v>
+      </c>
+      <c r="B33" s="9" t="s">
+        <v>69</v>
+      </c>
+      <c r="C33" s="9"/>
+      <c r="D33" s="9"/>
+      <c r="E33" s="9"/>
+      <c r="F33" s="9"/>
+      <c r="G33" s="9"/>
+    </row>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A34" s="9" t="b">
+        <v>0</v>
+      </c>
+      <c r="B34" s="9" t="s">
+        <v>6</v>
+      </c>
+      <c r="C34" s="9">
+        <v>1000</v>
+      </c>
+      <c r="D34" s="9"/>
+      <c r="E34" s="9"/>
+      <c r="F34" s="9" t="s">
+        <v>70</v>
+      </c>
+      <c r="G34" s="9" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A35" t="b">
-        <v>1</v>
-      </c>
-      <c r="B35" t="s">
-        <v>63</v>
-      </c>
-      <c r="C35">
-        <v>300</v>
-      </c>
-      <c r="D35">
-        <v>1.5</v>
-      </c>
-      <c r="E35">
-        <f>C35*D35</f>
-        <v>450</v>
-      </c>
-      <c r="F35" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.35">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A36" t="b">
         <v>0</v>
       </c>
       <c r="C36" s="3">
         <f>SUM(C2:C35)</f>
-        <v>15360</v>
+        <v>16960</v>
       </c>
       <c r="D36" s="3"/>
       <c r="E36" s="8">
@@ -1332,62 +1398,62 @@
         <v>21560</v>
       </c>
     </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A37" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A38" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A39" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A40" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A41" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A42" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A43" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A44" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A45" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A46" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A47" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A48" t="b">
         <v>0</v>
       </c>

</xml_diff>

<commit_message>
Zwetschken objednal Endesgrabner Johann (Gasthof Troadkastn)
</commit_message>
<xml_diff>
--- a/Obst.xlsx
+++ b/Obst.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://herzjesugym-my.sharepoint.com/personal/denis_holub_herzjesugym_at/Documents/Radtour 2026/mapa-rozvozu-ovoce/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\holub\AppData\Local\Temp\claude\C--Users-holub-OneDrive---Privatgymnasium-der-Herz-Jesu-Missionare-Radtour-2026\cbd12823-693e-4f3b-bb7d-65f09b0003cf\scratchpad\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="11_26872C97A4337C719472A8D655D9D6FCC967E65A" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{18F819F7-3EEC-4704-8E77-52B5672F6D22}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -233,7 +233,7 @@
     <t>Zwetschken</t>
   </si>
   <si>
-    <t>Gasthof Troadkastn</t>
+    <t>Endesgrabner Johann, Gasthof Troadkastn</t>
   </si>
   <si>
     <t>4894 Oberhofen am Irrsee</t>

</xml_diff>

<commit_message>
Nova objednavka: Herz Jesu skola, 300 kg Zwetschken
</commit_message>
<xml_diff>
--- a/Obst.xlsx
+++ b/Obst.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\holub\AppData\Local\Temp\claude\C--Users-holub-OneDrive---Privatgymnasium-der-Herz-Jesu-Missionare-Radtour-2026\cbd12823-693e-4f3b-bb7d-65f09b0003cf\scratchpad\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{18F819F7-3EEC-4704-8E77-52B5672F6D22}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{72B4FEF8-7174-4D09-8C4F-250F1CAF03F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="72">
   <si>
     <t>Geliefert</t>
   </si>
@@ -242,13 +242,13 @@
     <t>telefonisch bestellt +43 664 4233933 – Preis ergänzen</t>
   </si>
   <si>
+    <t>Preis ergänzen</t>
+  </si>
+  <si>
     <t>Birnen Williams</t>
   </si>
   <si>
     <t>Haagweg 7, 5550 Radstadt</t>
-  </si>
-  <si>
-    <t>Preis ergänzen</t>
   </si>
 </sst>
 </file>
@@ -1343,8 +1343,22 @@
       </c>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A32" t="b">
-        <v>0</v>
+      <c r="A32" s="9" t="b">
+        <v>0</v>
+      </c>
+      <c r="B32" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="C32" s="9">
+        <v>300</v>
+      </c>
+      <c r="D32" s="9"/>
+      <c r="E32" s="9"/>
+      <c r="F32" s="9" t="s">
+        <v>54</v>
+      </c>
+      <c r="G32" s="9" t="s">
+        <v>69</v>
       </c>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.35">
@@ -1352,7 +1366,7 @@
         <v>0</v>
       </c>
       <c r="B33" s="9" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="C33" s="9"/>
       <c r="D33" s="9"/>
@@ -1373,10 +1387,10 @@
       <c r="D34" s="9"/>
       <c r="E34" s="9"/>
       <c r="F34" s="9" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="G34" s="9" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.35">
@@ -1390,7 +1404,7 @@
       </c>
       <c r="C36" s="3">
         <f>SUM(C2:C35)</f>
-        <v>16960</v>
+        <v>17260</v>
       </c>
       <c r="D36" s="3"/>
       <c r="E36" s="8">

</xml_diff>

<commit_message>
Troadkastn: adresa Rabenschwand 48; ceny: Zwetschken 1,30, Birnen Williams 1,20 EUR/kg
</commit_message>
<xml_diff>
--- a/Obst.xlsx
+++ b/Obst.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\holub\AppData\Local\Temp\claude\C--Users-holub-OneDrive---Privatgymnasium-der-Herz-Jesu-Missionare-Radtour-2026\cbd12823-693e-4f3b-bb7d-65f09b0003cf\scratchpad\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{72B4FEF8-7174-4D09-8C4F-250F1CAF03F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D2907C78-BD1D-4BEC-ABEE-B3C20999772E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="71">
   <si>
     <t>Geliefert</t>
   </si>
@@ -236,13 +236,10 @@
     <t>Endesgrabner Johann, Gasthof Troadkastn</t>
   </si>
   <si>
-    <t>4894 Oberhofen am Irrsee</t>
-  </si>
-  <si>
-    <t>telefonisch bestellt +43 664 4233933 – Preis ergänzen</t>
-  </si>
-  <si>
-    <t>Preis ergänzen</t>
+    <t>Rabenschwand 48, 4894 Oberhofen am Irrsee</t>
+  </si>
+  <si>
+    <t>telefonisch bestellt +43 664 4233933</t>
   </si>
   <si>
     <t>Birnen Williams</t>
@@ -1333,8 +1330,13 @@
       <c r="C31" s="9">
         <v>600</v>
       </c>
-      <c r="D31" s="9"/>
-      <c r="E31" s="9"/>
+      <c r="D31" s="9">
+        <v>1.3</v>
+      </c>
+      <c r="E31" s="9">
+        <f>C31*D31</f>
+        <v>780</v>
+      </c>
       <c r="F31" s="9" t="s">
         <v>67</v>
       </c>
@@ -1352,21 +1354,24 @@
       <c r="C32" s="9">
         <v>300</v>
       </c>
-      <c r="D32" s="9"/>
-      <c r="E32" s="9"/>
+      <c r="D32" s="9">
+        <v>1.3</v>
+      </c>
+      <c r="E32" s="9">
+        <f>C32*D32</f>
+        <v>390</v>
+      </c>
       <c r="F32" s="9" t="s">
         <v>54</v>
       </c>
-      <c r="G32" s="9" t="s">
-        <v>69</v>
-      </c>
+      <c r="G32" s="9"/>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A33" s="9" t="b">
         <v>0</v>
       </c>
       <c r="B33" s="9" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C33" s="9"/>
       <c r="D33" s="9"/>
@@ -1384,14 +1389,17 @@
       <c r="C34" s="9">
         <v>1000</v>
       </c>
-      <c r="D34" s="9"/>
-      <c r="E34" s="9"/>
+      <c r="D34" s="9">
+        <v>1.2</v>
+      </c>
+      <c r="E34" s="9">
+        <f>C34*D34</f>
+        <v>1200</v>
+      </c>
       <c r="F34" s="9" t="s">
-        <v>71</v>
-      </c>
-      <c r="G34" s="9" t="s">
-        <v>69</v>
-      </c>
+        <v>70</v>
+      </c>
+      <c r="G34" s="9"/>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A35" t="b">
@@ -1409,7 +1417,7 @@
       <c r="D36" s="3"/>
       <c r="E36" s="8">
         <f>SUM(E2:E35)</f>
-        <v>21560</v>
+        <v>23930</v>
       </c>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
Nova objednavka: Gasteiger, 1600 kg Birnen Williams
</commit_message>
<xml_diff>
--- a/Obst.xlsx
+++ b/Obst.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\holub\AppData\Local\Temp\claude\C--Users-holub-OneDrive---Privatgymnasium-der-Herz-Jesu-Missionare-Radtour-2026\cbd12823-693e-4f3b-bb7d-65f09b0003cf\scratchpad\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D2907C78-BD1D-4BEC-ABEE-B3C20999772E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{32B6088B-F670-4A2A-BF3F-D76261503C14}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="71">
   <si>
     <t>Geliefert</t>
   </si>
@@ -1402,9 +1402,26 @@
       <c r="G34" s="9"/>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A35" t="b">
-        <v>0</v>
-      </c>
+      <c r="A35" s="9" t="b">
+        <v>0</v>
+      </c>
+      <c r="B35" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="C35" s="9">
+        <v>1600</v>
+      </c>
+      <c r="D35" s="9">
+        <v>1.2</v>
+      </c>
+      <c r="E35" s="9">
+        <f>C35*D35</f>
+        <v>1920</v>
+      </c>
+      <c r="F35" s="9" t="s">
+        <v>43</v>
+      </c>
+      <c r="G35" s="9"/>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A36" t="b">
@@ -1412,12 +1429,12 @@
       </c>
       <c r="C36" s="3">
         <f>SUM(C2:C35)</f>
-        <v>17260</v>
+        <v>18860</v>
       </c>
       <c r="D36" s="3"/>
       <c r="E36" s="8">
         <f>SUM(E2:E35)</f>
-        <v>23930</v>
+        <v>25850</v>
       </c>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
Nova objednavka: Daniel Steiner, 250 kg Zwetschken, Kuchl
</commit_message>
<xml_diff>
--- a/Obst.xlsx
+++ b/Obst.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\holub\AppData\Local\Temp\claude\C--Users-holub-OneDrive---Privatgymnasium-der-Herz-Jesu-Missionare-Radtour-2026\cbd12823-693e-4f3b-bb7d-65f09b0003cf\scratchpad\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{32B6088B-F670-4A2A-BF3F-D76261503C14}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F4CF3ADA-D901-41B5-959D-E1AB51452101}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="73">
   <si>
     <t>Geliefert</t>
   </si>
@@ -240,6 +240,12 @@
   </si>
   <si>
     <t>telefonisch bestellt +43 664 4233933</t>
+  </si>
+  <si>
+    <t>Daniel Steiner</t>
+  </si>
+  <si>
+    <t>Markt 30, 5431 Kuchl</t>
   </si>
   <si>
     <t>Birnen Williams</t>
@@ -683,7 +689,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H54"/>
+  <dimension ref="A1:H55"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="19" bestFit="1" customWidth="1"/>
@@ -1373,10 +1379,19 @@
       <c r="B33" s="9" t="s">
         <v>69</v>
       </c>
-      <c r="C33" s="9"/>
-      <c r="D33" s="9"/>
-      <c r="E33" s="9"/>
-      <c r="F33" s="9"/>
+      <c r="C33" s="9">
+        <v>250</v>
+      </c>
+      <c r="D33" s="9">
+        <v>1.3</v>
+      </c>
+      <c r="E33" s="9">
+        <f>C33*D33</f>
+        <v>325</v>
+      </c>
+      <c r="F33" s="9" t="s">
+        <v>70</v>
+      </c>
       <c r="G33" s="9"/>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.35">
@@ -1384,21 +1399,12 @@
         <v>0</v>
       </c>
       <c r="B34" s="9" t="s">
-        <v>6</v>
-      </c>
-      <c r="C34" s="9">
-        <v>1000</v>
-      </c>
-      <c r="D34" s="9">
-        <v>1.2</v>
-      </c>
-      <c r="E34" s="9">
-        <f>C34*D34</f>
-        <v>1200</v>
-      </c>
-      <c r="F34" s="9" t="s">
-        <v>70</v>
-      </c>
+        <v>71</v>
+      </c>
+      <c r="C34" s="9"/>
+      <c r="D34" s="9"/>
+      <c r="E34" s="9"/>
+      <c r="F34" s="9"/>
       <c r="G34" s="9"/>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.35">
@@ -1406,41 +1412,58 @@
         <v>0</v>
       </c>
       <c r="B35" s="9" t="s">
-        <v>42</v>
+        <v>6</v>
       </c>
       <c r="C35" s="9">
-        <v>1600</v>
+        <v>1000</v>
       </c>
       <c r="D35" s="9">
         <v>1.2</v>
       </c>
       <c r="E35" s="9">
         <f>C35*D35</f>
+        <v>1200</v>
+      </c>
+      <c r="F35" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="G35" s="9"/>
+    </row>
+    <row r="36" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A36" s="9" t="b">
+        <v>0</v>
+      </c>
+      <c r="B36" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="C36" s="9">
+        <v>1600</v>
+      </c>
+      <c r="D36" s="9">
+        <v>1.2</v>
+      </c>
+      <c r="E36" s="9">
+        <f>C36*D36</f>
         <v>1920</v>
       </c>
-      <c r="F35" s="9" t="s">
+      <c r="F36" s="9" t="s">
         <v>43</v>
       </c>
-      <c r="G35" s="9"/>
-    </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A36" t="b">
-        <v>0</v>
-      </c>
-      <c r="C36" s="3">
-        <f>SUM(C2:C35)</f>
-        <v>18860</v>
-      </c>
-      <c r="D36" s="3"/>
-      <c r="E36" s="8">
-        <f>SUM(E2:E35)</f>
-        <v>25850</v>
-      </c>
+      <c r="G36" s="9"/>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A37" t="b">
         <v>0</v>
       </c>
+      <c r="C37" s="3">
+        <f>SUM(C2:C36)</f>
+        <v>19110</v>
+      </c>
+      <c r="D37" s="3"/>
+      <c r="E37" s="8">
+        <f>SUM(E2:E36)</f>
+        <v>26175</v>
+      </c>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A38" t="b">
@@ -1524,6 +1547,11 @@
     </row>
     <row r="54" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A54" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="55" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A55" t="b">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Nova objednavka: Christian Schlick, 600 kg Birnen Williams, Zederhaus (Abholung Salzburg/Radstadt)
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Obst.xlsx
+++ b/Obst.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\holub\AppData\Local\Temp\claude\C--Users-holub-OneDrive---Privatgymnasium-der-Herz-Jesu-Missionare-Radtour-2026\cbd12823-693e-4f3b-bb7d-65f09b0003cf\scratchpad\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://herzjesugym-my.sharepoint.com/personal/denis_holub_herzjesugym_at/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F4CF3ADA-D901-41B5-959D-E1AB51452101}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="10" documentId="13_ncr:1_{F4CF3ADA-D901-41B5-959D-E1AB51452101}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F55E28A7-D2A6-4F71-A6A9-478900496C38}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="73">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="76">
   <si>
     <t>Geliefert</t>
   </si>
@@ -252,6 +252,15 @@
   </si>
   <si>
     <t>Haagweg 7, 5550 Radstadt</t>
+  </si>
+  <si>
+    <t>Christian Schlick</t>
+  </si>
+  <si>
+    <t>Zederhaus</t>
+  </si>
+  <si>
+    <t>Abholung in Salzburg oder Radstadt möglich</t>
   </si>
 </sst>
 </file>
@@ -259,8 +268,8 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
-    <numFmt numFmtId="44" formatCode="_-&quot;€&quot;\ * #,##0.00_-;\-&quot;€&quot;\ * #,##0.00_-;_-&quot;€&quot;\ * &quot;-&quot;??_-;_-@_-"/>
-    <numFmt numFmtId="164" formatCode="0\ &quot;kg&quot;"/>
+    <numFmt numFmtId="164" formatCode="_-&quot;€&quot;\ * #,##0.00_-;\-&quot;€&quot;\ * #,##0.00_-;_-&quot;€&quot;\ * &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="165" formatCode="0\ &quot;kg&quot;"/>
   </numFmts>
   <fonts count="7" x14ac:knownFonts="1">
     <font>
@@ -328,19 +337,19 @@
   </borders>
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="44" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="2"/>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="3">
@@ -689,7 +698,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H55"/>
+  <dimension ref="A1:H56"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="19" bestFit="1" customWidth="1"/>
@@ -1452,23 +1461,42 @@
       <c r="G36" s="9"/>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A37" t="b">
-        <v>0</v>
-      </c>
-      <c r="C37" s="3">
-        <f>SUM(C2:C36)</f>
-        <v>19110</v>
-      </c>
-      <c r="D37" s="3"/>
-      <c r="E37" s="8">
-        <f>SUM(E2:E36)</f>
-        <v>26175</v>
+      <c r="A37" s="9" t="b">
+        <v>0</v>
+      </c>
+      <c r="B37" s="9" t="s">
+        <v>73</v>
+      </c>
+      <c r="C37" s="9">
+        <v>600</v>
+      </c>
+      <c r="D37" s="9">
+        <v>1.2</v>
+      </c>
+      <c r="E37" s="9">
+        <f>C37*D37</f>
+        <v>720</v>
+      </c>
+      <c r="F37" s="9" t="s">
+        <v>74</v>
+      </c>
+      <c r="G37" s="9" t="s">
+        <v>75</v>
       </c>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A38" t="b">
         <v>0</v>
       </c>
+      <c r="C38" s="3">
+        <f>SUM(C2:C37)</f>
+        <v>19710</v>
+      </c>
+      <c r="D38" s="3"/>
+      <c r="E38" s="8">
+        <f>SUM(E2:E37)</f>
+        <v>26895</v>
+      </c>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A39" t="b">
@@ -1552,6 +1580,11 @@
     </row>
     <row r="55" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A55" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="56" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A56" t="b">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Nova objednavka: Johann Lackner, 300 kg Birnen Williams, Mariapfarr
</commit_message>
<xml_diff>
--- a/Obst.xlsx
+++ b/Obst.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://herzjesugym-my.sharepoint.com/personal/denis_holub_herzjesugym_at/Documents/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\holub\AppData\Local\Temp\claude\C--Users-holub-OneDrive---Privatgymnasium-der-Herz-Jesu-Missionare-Radtour-2026\cbd12823-693e-4f3b-bb7d-65f09b0003cf\scratchpad\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="10" documentId="13_ncr:1_{F4CF3ADA-D901-41B5-959D-E1AB51452101}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F55E28A7-D2A6-4F71-A6A9-478900496C38}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{457AF80B-2AC9-4DFA-B111-186DC245F920}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3800" yWindow="3800" windowWidth="28800" windowHeight="15370" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="76">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="78">
   <si>
     <t>Geliefert</t>
   </si>
@@ -261,6 +261,12 @@
   </si>
   <si>
     <t>Abholung in Salzburg oder Radstadt möglich</t>
+  </si>
+  <si>
+    <t>Johann Lackner</t>
+  </si>
+  <si>
+    <t>5571 Mariapfarr</t>
   </si>
 </sst>
 </file>
@@ -268,8 +274,8 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="_-&quot;€&quot;\ * #,##0.00_-;\-&quot;€&quot;\ * #,##0.00_-;_-&quot;€&quot;\ * &quot;-&quot;??_-;_-@_-"/>
-    <numFmt numFmtId="165" formatCode="0\ &quot;kg&quot;"/>
+    <numFmt numFmtId="44" formatCode="_-&quot;€&quot;\ * #,##0.00_-;\-&quot;€&quot;\ * #,##0.00_-;_-&quot;€&quot;\ * &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="164" formatCode="0\ &quot;kg&quot;"/>
   </numFmts>
   <fonts count="7" x14ac:knownFonts="1">
     <font>
@@ -337,19 +343,19 @@
   </borders>
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="44" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="2"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="3">
@@ -698,7 +704,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H56"/>
+  <dimension ref="A1:H57"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="19" bestFit="1" customWidth="1"/>
@@ -1485,23 +1491,40 @@
       </c>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A38" t="b">
-        <v>0</v>
-      </c>
-      <c r="C38" s="3">
-        <f>SUM(C2:C37)</f>
-        <v>19710</v>
-      </c>
-      <c r="D38" s="3"/>
-      <c r="E38" s="8">
-        <f>SUM(E2:E37)</f>
-        <v>26895</v>
-      </c>
+      <c r="A38" s="9" t="b">
+        <v>0</v>
+      </c>
+      <c r="B38" s="9" t="s">
+        <v>76</v>
+      </c>
+      <c r="C38" s="9">
+        <v>300</v>
+      </c>
+      <c r="D38" s="9">
+        <v>1.2</v>
+      </c>
+      <c r="E38" s="9">
+        <f>C38*D38</f>
+        <v>360</v>
+      </c>
+      <c r="F38" s="9" t="s">
+        <v>77</v>
+      </c>
+      <c r="G38" s="9"/>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A39" t="b">
         <v>0</v>
       </c>
+      <c r="C39" s="3">
+        <f>SUM(C2:C38)</f>
+        <v>20010</v>
+      </c>
+      <c r="D39" s="3"/>
+      <c r="E39" s="8">
+        <f>SUM(E2:E38)</f>
+        <v>27255</v>
+      </c>
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A40" t="b">
@@ -1585,6 +1608,11 @@
     </row>
     <row r="56" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A56" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="57" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A57" t="b">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Lackner: GPS souradnice centra Mariapfarr
</commit_message>
<xml_diff>
--- a/Obst.xlsx
+++ b/Obst.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\holub\AppData\Local\Temp\claude\C--Users-holub-OneDrive---Privatgymnasium-der-Herz-Jesu-Missionare-Radtour-2026\cbd12823-693e-4f3b-bb7d-65f09b0003cf\scratchpad\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{457AF80B-2AC9-4DFA-B111-186DC245F920}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B5CA2163-B135-4D07-9FB5-05226C3463BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3800" yWindow="3800" windowWidth="28800" windowHeight="15370" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2660" yWindow="2660" windowWidth="28800" windowHeight="15370" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="78">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="79">
   <si>
     <t>Geliefert</t>
   </si>
@@ -267,6 +267,9 @@
   </si>
   <si>
     <t>5571 Mariapfarr</t>
+  </si>
+  <si>
+    <t>(47.1513091, 13.7456747)</t>
   </si>
 </sst>
 </file>
@@ -1510,7 +1513,9 @@
       <c r="F38" s="9" t="s">
         <v>77</v>
       </c>
-      <c r="G38" s="9"/>
+      <c r="G38" s="9" t="s">
+        <v>78</v>
+      </c>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A39" t="b">

</xml_diff>

<commit_message>
Lackner navic 300 kg Zwetschken (Abholung Salzburg/Radstadt mozna)
</commit_message>
<xml_diff>
--- a/Obst.xlsx
+++ b/Obst.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\holub\AppData\Local\Temp\claude\C--Users-holub-OneDrive---Privatgymnasium-der-Herz-Jesu-Missionare-Radtour-2026\cbd12823-693e-4f3b-bb7d-65f09b0003cf\scratchpad\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B5CA2163-B135-4D07-9FB5-05226C3463BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3281B630-F1F6-4280-A79B-E5B5D5252644}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2660" yWindow="2660" windowWidth="28800" windowHeight="15370" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="79">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="80">
   <si>
     <t>Geliefert</t>
   </si>
@@ -248,6 +248,15 @@
     <t>Markt 30, 5431 Kuchl</t>
   </si>
   <si>
+    <t>Johann Lackner</t>
+  </si>
+  <si>
+    <t>5571 Mariapfarr</t>
+  </si>
+  <si>
+    <t>(47.1513091, 13.7456747) Abholung in Salzburg oder Radstadt möglich</t>
+  </si>
+  <si>
     <t>Birnen Williams</t>
   </si>
   <si>
@@ -261,12 +270,6 @@
   </si>
   <si>
     <t>Abholung in Salzburg oder Radstadt möglich</t>
-  </si>
-  <si>
-    <t>Johann Lackner</t>
-  </si>
-  <si>
-    <t>5571 Mariapfarr</t>
   </si>
   <si>
     <t>(47.1513091, 13.7456747)</t>
@@ -707,7 +710,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H57"/>
+  <dimension ref="A1:H58"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="19" bestFit="1" customWidth="1"/>
@@ -1419,32 +1422,34 @@
       <c r="B34" s="9" t="s">
         <v>71</v>
       </c>
-      <c r="C34" s="9"/>
-      <c r="D34" s="9"/>
-      <c r="E34" s="9"/>
-      <c r="F34" s="9"/>
-      <c r="G34" s="9"/>
+      <c r="C34" s="9">
+        <v>300</v>
+      </c>
+      <c r="D34" s="9">
+        <v>1.3</v>
+      </c>
+      <c r="E34" s="9">
+        <f>C34*D34</f>
+        <v>390</v>
+      </c>
+      <c r="F34" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="G34" s="9" t="s">
+        <v>73</v>
+      </c>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A35" s="9" t="b">
         <v>0</v>
       </c>
       <c r="B35" s="9" t="s">
-        <v>6</v>
-      </c>
-      <c r="C35" s="9">
-        <v>1000</v>
-      </c>
-      <c r="D35" s="9">
-        <v>1.2</v>
-      </c>
-      <c r="E35" s="9">
-        <f>C35*D35</f>
-        <v>1200</v>
-      </c>
-      <c r="F35" s="9" t="s">
-        <v>72</v>
-      </c>
+        <v>74</v>
+      </c>
+      <c r="C35" s="9"/>
+      <c r="D35" s="9"/>
+      <c r="E35" s="9"/>
+      <c r="F35" s="9"/>
       <c r="G35" s="9"/>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.35">
@@ -1452,20 +1457,20 @@
         <v>0</v>
       </c>
       <c r="B36" s="9" t="s">
-        <v>42</v>
+        <v>6</v>
       </c>
       <c r="C36" s="9">
-        <v>1600</v>
+        <v>1000</v>
       </c>
       <c r="D36" s="9">
         <v>1.2</v>
       </c>
       <c r="E36" s="9">
         <f>C36*D36</f>
-        <v>1920</v>
+        <v>1200</v>
       </c>
       <c r="F36" s="9" t="s">
-        <v>43</v>
+        <v>75</v>
       </c>
       <c r="G36" s="9"/>
     </row>
@@ -1474,24 +1479,22 @@
         <v>0</v>
       </c>
       <c r="B37" s="9" t="s">
-        <v>73</v>
+        <v>42</v>
       </c>
       <c r="C37" s="9">
-        <v>600</v>
+        <v>1600</v>
       </c>
       <c r="D37" s="9">
         <v>1.2</v>
       </c>
       <c r="E37" s="9">
         <f>C37*D37</f>
-        <v>720</v>
+        <v>1920</v>
       </c>
       <c r="F37" s="9" t="s">
-        <v>74</v>
-      </c>
-      <c r="G37" s="9" t="s">
-        <v>75</v>
-      </c>
+        <v>43</v>
+      </c>
+      <c r="G37" s="9"/>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A38" s="9" t="b">
@@ -1501,14 +1504,14 @@
         <v>76</v>
       </c>
       <c r="C38" s="9">
-        <v>300</v>
+        <v>600</v>
       </c>
       <c r="D38" s="9">
         <v>1.2</v>
       </c>
       <c r="E38" s="9">
         <f>C38*D38</f>
-        <v>360</v>
+        <v>720</v>
       </c>
       <c r="F38" s="9" t="s">
         <v>77</v>
@@ -1518,23 +1521,42 @@
       </c>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A39" t="b">
-        <v>0</v>
-      </c>
-      <c r="C39" s="3">
-        <f>SUM(C2:C38)</f>
-        <v>20010</v>
-      </c>
-      <c r="D39" s="3"/>
-      <c r="E39" s="8">
-        <f>SUM(E2:E38)</f>
-        <v>27255</v>
+      <c r="A39" s="9" t="b">
+        <v>0</v>
+      </c>
+      <c r="B39" s="9" t="s">
+        <v>71</v>
+      </c>
+      <c r="C39" s="9">
+        <v>300</v>
+      </c>
+      <c r="D39" s="9">
+        <v>1.2</v>
+      </c>
+      <c r="E39" s="9">
+        <f>C39*D39</f>
+        <v>360</v>
+      </c>
+      <c r="F39" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="G39" s="9" t="s">
+        <v>79</v>
       </c>
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A40" t="b">
         <v>0</v>
       </c>
+      <c r="C40" s="3">
+        <f>SUM(C2:C39)</f>
+        <v>20310</v>
+      </c>
+      <c r="D40" s="3"/>
+      <c r="E40" s="8">
+        <f>SUM(E2:E39)</f>
+        <v>27645</v>
+      </c>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A41" t="b">
@@ -1618,6 +1640,11 @@
     </row>
     <row r="57" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A57" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="58" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A58" t="b">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Nova objednavka: Armand (Pfarre Koppl), 100 kg Zwetschken + 100 kg Birnen Williams
</commit_message>
<xml_diff>
--- a/Obst.xlsx
+++ b/Obst.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\holub\AppData\Local\Temp\claude\C--Users-holub-OneDrive---Privatgymnasium-der-Herz-Jesu-Missionare-Radtour-2026\cbd12823-693e-4f3b-bb7d-65f09b0003cf\scratchpad\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3281B630-F1F6-4280-A79B-E5B5D5252644}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{94ABE3B3-E607-41C9-B360-4BEC08028B7E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2660" yWindow="2660" windowWidth="28800" windowHeight="15370" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="80">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="83">
   <si>
     <t>Geliefert</t>
   </si>
@@ -255,6 +255,15 @@
   </si>
   <si>
     <t>(47.1513091, 13.7456747) Abholung in Salzburg oder Radstadt möglich</t>
+  </si>
+  <si>
+    <t>Armand, Pfarre Koppl</t>
+  </si>
+  <si>
+    <t>5321 Koppl</t>
+  </si>
+  <si>
+    <t>Pfarre</t>
   </si>
   <si>
     <t>Birnen Williams</t>
@@ -710,7 +719,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H58"/>
+  <dimension ref="A1:H60"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="19" bestFit="1" customWidth="1"/>
@@ -1446,32 +1455,34 @@
       <c r="B35" s="9" t="s">
         <v>74</v>
       </c>
-      <c r="C35" s="9"/>
-      <c r="D35" s="9"/>
-      <c r="E35" s="9"/>
-      <c r="F35" s="9"/>
-      <c r="G35" s="9"/>
+      <c r="C35" s="9">
+        <v>100</v>
+      </c>
+      <c r="D35" s="9">
+        <v>1.3</v>
+      </c>
+      <c r="E35" s="9">
+        <f>C35*D35</f>
+        <v>130</v>
+      </c>
+      <c r="F35" s="9" t="s">
+        <v>75</v>
+      </c>
+      <c r="G35" s="9" t="s">
+        <v>76</v>
+      </c>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A36" s="9" t="b">
         <v>0</v>
       </c>
       <c r="B36" s="9" t="s">
-        <v>6</v>
-      </c>
-      <c r="C36" s="9">
-        <v>1000</v>
-      </c>
-      <c r="D36" s="9">
-        <v>1.2</v>
-      </c>
-      <c r="E36" s="9">
-        <f>C36*D36</f>
-        <v>1200</v>
-      </c>
-      <c r="F36" s="9" t="s">
-        <v>75</v>
-      </c>
+        <v>77</v>
+      </c>
+      <c r="C36" s="9"/>
+      <c r="D36" s="9"/>
+      <c r="E36" s="9"/>
+      <c r="F36" s="9"/>
       <c r="G36" s="9"/>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.35">
@@ -1479,20 +1490,20 @@
         <v>0</v>
       </c>
       <c r="B37" s="9" t="s">
-        <v>42</v>
+        <v>6</v>
       </c>
       <c r="C37" s="9">
-        <v>1600</v>
+        <v>1000</v>
       </c>
       <c r="D37" s="9">
         <v>1.2</v>
       </c>
       <c r="E37" s="9">
         <f>C37*D37</f>
-        <v>1920</v>
+        <v>1200</v>
       </c>
       <c r="F37" s="9" t="s">
-        <v>43</v>
+        <v>78</v>
       </c>
       <c r="G37" s="9"/>
     </row>
@@ -1501,72 +1512,108 @@
         <v>0</v>
       </c>
       <c r="B38" s="9" t="s">
-        <v>76</v>
+        <v>42</v>
       </c>
       <c r="C38" s="9">
-        <v>600</v>
+        <v>1600</v>
       </c>
       <c r="D38" s="9">
         <v>1.2</v>
       </c>
       <c r="E38" s="9">
         <f>C38*D38</f>
-        <v>720</v>
+        <v>1920</v>
       </c>
       <c r="F38" s="9" t="s">
-        <v>77</v>
-      </c>
-      <c r="G38" s="9" t="s">
-        <v>78</v>
-      </c>
+        <v>43</v>
+      </c>
+      <c r="G38" s="9"/>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A39" s="9" t="b">
         <v>0</v>
       </c>
       <c r="B39" s="9" t="s">
-        <v>71</v>
+        <v>79</v>
       </c>
       <c r="C39" s="9">
-        <v>300</v>
+        <v>600</v>
       </c>
       <c r="D39" s="9">
         <v>1.2</v>
       </c>
       <c r="E39" s="9">
         <f>C39*D39</f>
+        <v>720</v>
+      </c>
+      <c r="F39" s="9" t="s">
+        <v>80</v>
+      </c>
+      <c r="G39" s="9" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A40" s="9" t="b">
+        <v>0</v>
+      </c>
+      <c r="B40" s="9" t="s">
+        <v>71</v>
+      </c>
+      <c r="C40" s="9">
+        <v>300</v>
+      </c>
+      <c r="D40" s="9">
+        <v>1.2</v>
+      </c>
+      <c r="E40" s="9">
+        <f>C40*D40</f>
         <v>360</v>
       </c>
-      <c r="F39" s="9" t="s">
+      <c r="F40" s="9" t="s">
         <v>72</v>
       </c>
-      <c r="G39" s="9" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A40" t="b">
-        <v>0</v>
-      </c>
-      <c r="C40" s="3">
-        <f>SUM(C2:C39)</f>
-        <v>20310</v>
-      </c>
-      <c r="D40" s="3"/>
-      <c r="E40" s="8">
-        <f>SUM(E2:E39)</f>
-        <v>27645</v>
+      <c r="G40" s="9" t="s">
+        <v>82</v>
       </c>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A41" t="b">
-        <v>0</v>
+      <c r="A41" s="9" t="b">
+        <v>0</v>
+      </c>
+      <c r="B41" s="9" t="s">
+        <v>74</v>
+      </c>
+      <c r="C41" s="9">
+        <v>100</v>
+      </c>
+      <c r="D41" s="9">
+        <v>1.2</v>
+      </c>
+      <c r="E41" s="9">
+        <f>C41*D41</f>
+        <v>120</v>
+      </c>
+      <c r="F41" s="9" t="s">
+        <v>75</v>
+      </c>
+      <c r="G41" s="9" t="s">
+        <v>76</v>
       </c>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A42" t="b">
         <v>0</v>
       </c>
+      <c r="C42" s="3">
+        <f>SUM(C2:C41)</f>
+        <v>20510</v>
+      </c>
+      <c r="D42" s="3"/>
+      <c r="E42" s="8">
+        <f>SUM(E2:E41)</f>
+        <v>27895</v>
+      </c>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A43" t="b">
@@ -1645,6 +1692,16 @@
     </row>
     <row r="58" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A58" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="59" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A59" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="60" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A60" t="b">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Nova objednavka: Flockner, 200 kg Zwetschken za 1,10
</commit_message>
<xml_diff>
--- a/Obst.xlsx
+++ b/Obst.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\holub\AppData\Local\Temp\claude\C--Users-holub-OneDrive---Privatgymnasium-der-Herz-Jesu-Missionare-Radtour-2026\cbd12823-693e-4f3b-bb7d-65f09b0003cf\scratchpad\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{94ABE3B3-E607-41C9-B360-4BEC08028B7E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E6505AE5-B73C-4925-9D04-AD39552DB86E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="83">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="83">
   <si>
     <t>Geliefert</t>
   </si>
@@ -719,7 +719,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H60"/>
+  <dimension ref="A1:H61"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="19" bestFit="1" customWidth="1"/>
@@ -1370,7 +1370,7 @@
         <v>1.3</v>
       </c>
       <c r="E31" s="9">
-        <f>C31*D31</f>
+        <f t="shared" ref="E31:E36" si="1">C31*D31</f>
         <v>780</v>
       </c>
       <c r="F31" s="9" t="s">
@@ -1394,7 +1394,7 @@
         <v>1.3</v>
       </c>
       <c r="E32" s="9">
-        <f>C32*D32</f>
+        <f t="shared" si="1"/>
         <v>390</v>
       </c>
       <c r="F32" s="9" t="s">
@@ -1416,7 +1416,7 @@
         <v>1.3</v>
       </c>
       <c r="E33" s="9">
-        <f>C33*D33</f>
+        <f t="shared" si="1"/>
         <v>325</v>
       </c>
       <c r="F33" s="9" t="s">
@@ -1438,7 +1438,7 @@
         <v>1.3</v>
       </c>
       <c r="E34" s="9">
-        <f>C34*D34</f>
+        <f t="shared" si="1"/>
         <v>390</v>
       </c>
       <c r="F34" s="9" t="s">
@@ -1462,7 +1462,7 @@
         <v>1.3</v>
       </c>
       <c r="E35" s="9">
-        <f>C35*D35</f>
+        <f t="shared" si="1"/>
         <v>130</v>
       </c>
       <c r="F35" s="9" t="s">
@@ -1477,12 +1477,21 @@
         <v>0</v>
       </c>
       <c r="B36" s="9" t="s">
-        <v>77</v>
-      </c>
-      <c r="C36" s="9"/>
-      <c r="D36" s="9"/>
-      <c r="E36" s="9"/>
-      <c r="F36" s="9"/>
+        <v>45</v>
+      </c>
+      <c r="C36" s="9">
+        <v>200</v>
+      </c>
+      <c r="D36" s="9">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="E36" s="9">
+        <f t="shared" si="1"/>
+        <v>220.00000000000003</v>
+      </c>
+      <c r="F36" s="9" t="s">
+        <v>46</v>
+      </c>
       <c r="G36" s="9"/>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.35">
@@ -1490,21 +1499,12 @@
         <v>0</v>
       </c>
       <c r="B37" s="9" t="s">
-        <v>6</v>
-      </c>
-      <c r="C37" s="9">
-        <v>1000</v>
-      </c>
-      <c r="D37" s="9">
-        <v>1.2</v>
-      </c>
-      <c r="E37" s="9">
-        <f>C37*D37</f>
-        <v>1200</v>
-      </c>
-      <c r="F37" s="9" t="s">
-        <v>78</v>
-      </c>
+        <v>77</v>
+      </c>
+      <c r="C37" s="9"/>
+      <c r="D37" s="9"/>
+      <c r="E37" s="9"/>
+      <c r="F37" s="9"/>
       <c r="G37" s="9"/>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.35">
@@ -1512,20 +1512,20 @@
         <v>0</v>
       </c>
       <c r="B38" s="9" t="s">
-        <v>42</v>
+        <v>6</v>
       </c>
       <c r="C38" s="9">
-        <v>1600</v>
+        <v>1000</v>
       </c>
       <c r="D38" s="9">
         <v>1.2</v>
       </c>
       <c r="E38" s="9">
         <f>C38*D38</f>
-        <v>1920</v>
+        <v>1200</v>
       </c>
       <c r="F38" s="9" t="s">
-        <v>43</v>
+        <v>78</v>
       </c>
       <c r="G38" s="9"/>
     </row>
@@ -1534,47 +1534,45 @@
         <v>0</v>
       </c>
       <c r="B39" s="9" t="s">
-        <v>79</v>
+        <v>42</v>
       </c>
       <c r="C39" s="9">
-        <v>600</v>
+        <v>1600</v>
       </c>
       <c r="D39" s="9">
         <v>1.2</v>
       </c>
       <c r="E39" s="9">
         <f>C39*D39</f>
-        <v>720</v>
+        <v>1920</v>
       </c>
       <c r="F39" s="9" t="s">
-        <v>80</v>
-      </c>
-      <c r="G39" s="9" t="s">
-        <v>81</v>
-      </c>
+        <v>43</v>
+      </c>
+      <c r="G39" s="9"/>
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A40" s="9" t="b">
         <v>0</v>
       </c>
       <c r="B40" s="9" t="s">
-        <v>71</v>
+        <v>79</v>
       </c>
       <c r="C40" s="9">
-        <v>300</v>
+        <v>600</v>
       </c>
       <c r="D40" s="9">
         <v>1.2</v>
       </c>
       <c r="E40" s="9">
         <f>C40*D40</f>
-        <v>360</v>
+        <v>720</v>
       </c>
       <c r="F40" s="9" t="s">
-        <v>72</v>
+        <v>80</v>
       </c>
       <c r="G40" s="9" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.35">
@@ -1582,43 +1580,62 @@
         <v>0</v>
       </c>
       <c r="B41" s="9" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="C41" s="9">
-        <v>100</v>
+        <v>300</v>
       </c>
       <c r="D41" s="9">
         <v>1.2</v>
       </c>
       <c r="E41" s="9">
         <f>C41*D41</f>
+        <v>360</v>
+      </c>
+      <c r="F41" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="G41" s="9" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A42" s="9" t="b">
+        <v>0</v>
+      </c>
+      <c r="B42" s="9" t="s">
+        <v>74</v>
+      </c>
+      <c r="C42" s="9">
+        <v>100</v>
+      </c>
+      <c r="D42" s="9">
+        <v>1.2</v>
+      </c>
+      <c r="E42" s="9">
+        <f>C42*D42</f>
         <v>120</v>
       </c>
-      <c r="F41" s="9" t="s">
+      <c r="F42" s="9" t="s">
         <v>75</v>
       </c>
-      <c r="G41" s="9" t="s">
+      <c r="G42" s="9" t="s">
         <v>76</v>
-      </c>
-    </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A42" t="b">
-        <v>0</v>
-      </c>
-      <c r="C42" s="3">
-        <f>SUM(C2:C41)</f>
-        <v>20510</v>
-      </c>
-      <c r="D42" s="3"/>
-      <c r="E42" s="8">
-        <f>SUM(E2:E41)</f>
-        <v>27895</v>
       </c>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A43" t="b">
         <v>0</v>
       </c>
+      <c r="C43" s="3">
+        <f>SUM(C2:C42)</f>
+        <v>20710</v>
+      </c>
+      <c r="D43" s="3"/>
+      <c r="E43" s="8">
+        <f>SUM(E2:E42)</f>
+        <v>28115</v>
+      </c>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A44" t="b">
@@ -1702,6 +1719,11 @@
     </row>
     <row r="60" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A60" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="61" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A61" t="b">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Nove objednavky: Rosi Huber a Gasteiger po 600 kg Zwetschken za 1,10
</commit_message>
<xml_diff>
--- a/Obst.xlsx
+++ b/Obst.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\holub\AppData\Local\Temp\claude\C--Users-holub-OneDrive---Privatgymnasium-der-Herz-Jesu-Missionare-Radtour-2026\cbd12823-693e-4f3b-bb7d-65f09b0003cf\scratchpad\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E6505AE5-B73C-4925-9D04-AD39552DB86E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DA74A388-051C-470F-A802-17F24C21CB2E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="83">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="83">
   <si>
     <t>Geliefert</t>
   </si>
@@ -719,7 +719,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H61"/>
+  <dimension ref="A1:H63"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="19" bestFit="1" customWidth="1"/>
@@ -1370,7 +1370,7 @@
         <v>1.3</v>
       </c>
       <c r="E31" s="9">
-        <f t="shared" ref="E31:E36" si="1">C31*D31</f>
+        <f t="shared" ref="E31:E38" si="1">C31*D31</f>
         <v>780</v>
       </c>
       <c r="F31" s="9" t="s">
@@ -1499,12 +1499,21 @@
         <v>0</v>
       </c>
       <c r="B37" s="9" t="s">
-        <v>77</v>
-      </c>
-      <c r="C37" s="9"/>
-      <c r="D37" s="9"/>
-      <c r="E37" s="9"/>
-      <c r="F37" s="9"/>
+        <v>2</v>
+      </c>
+      <c r="C37" s="9">
+        <v>600</v>
+      </c>
+      <c r="D37" s="9">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="E37" s="9">
+        <f t="shared" si="1"/>
+        <v>660</v>
+      </c>
+      <c r="F37" s="9" t="s">
+        <v>3</v>
+      </c>
       <c r="G37" s="9"/>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.35">
@@ -1512,20 +1521,20 @@
         <v>0</v>
       </c>
       <c r="B38" s="9" t="s">
-        <v>6</v>
+        <v>42</v>
       </c>
       <c r="C38" s="9">
-        <v>1000</v>
+        <v>600</v>
       </c>
       <c r="D38" s="9">
-        <v>1.2</v>
+        <v>1.1000000000000001</v>
       </c>
       <c r="E38" s="9">
-        <f>C38*D38</f>
-        <v>1200</v>
+        <f t="shared" si="1"/>
+        <v>660</v>
       </c>
       <c r="F38" s="9" t="s">
-        <v>78</v>
+        <v>43</v>
       </c>
       <c r="G38" s="9"/>
     </row>
@@ -1534,21 +1543,12 @@
         <v>0</v>
       </c>
       <c r="B39" s="9" t="s">
-        <v>42</v>
-      </c>
-      <c r="C39" s="9">
-        <v>1600</v>
-      </c>
-      <c r="D39" s="9">
-        <v>1.2</v>
-      </c>
-      <c r="E39" s="9">
-        <f>C39*D39</f>
-        <v>1920</v>
-      </c>
-      <c r="F39" s="9" t="s">
-        <v>43</v>
-      </c>
+        <v>77</v>
+      </c>
+      <c r="C39" s="9"/>
+      <c r="D39" s="9"/>
+      <c r="E39" s="9"/>
+      <c r="F39" s="9"/>
       <c r="G39" s="9"/>
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.35">
@@ -1556,96 +1556,130 @@
         <v>0</v>
       </c>
       <c r="B40" s="9" t="s">
-        <v>79</v>
+        <v>6</v>
       </c>
       <c r="C40" s="9">
-        <v>600</v>
+        <v>1000</v>
       </c>
       <c r="D40" s="9">
         <v>1.2</v>
       </c>
       <c r="E40" s="9">
         <f>C40*D40</f>
-        <v>720</v>
+        <v>1200</v>
       </c>
       <c r="F40" s="9" t="s">
-        <v>80</v>
-      </c>
-      <c r="G40" s="9" t="s">
-        <v>81</v>
-      </c>
+        <v>78</v>
+      </c>
+      <c r="G40" s="9"/>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A41" s="9" t="b">
         <v>0</v>
       </c>
       <c r="B41" s="9" t="s">
-        <v>71</v>
+        <v>42</v>
       </c>
       <c r="C41" s="9">
-        <v>300</v>
+        <v>1600</v>
       </c>
       <c r="D41" s="9">
         <v>1.2</v>
       </c>
       <c r="E41" s="9">
         <f>C41*D41</f>
-        <v>360</v>
+        <v>1920</v>
       </c>
       <c r="F41" s="9" t="s">
-        <v>72</v>
-      </c>
-      <c r="G41" s="9" t="s">
-        <v>82</v>
-      </c>
+        <v>43</v>
+      </c>
+      <c r="G41" s="9"/>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A42" s="9" t="b">
         <v>0</v>
       </c>
       <c r="B42" s="9" t="s">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="C42" s="9">
-        <v>100</v>
+        <v>600</v>
       </c>
       <c r="D42" s="9">
         <v>1.2</v>
       </c>
       <c r="E42" s="9">
         <f>C42*D42</f>
+        <v>720</v>
+      </c>
+      <c r="F42" s="9" t="s">
+        <v>80</v>
+      </c>
+      <c r="G42" s="9" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="43" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A43" s="9" t="b">
+        <v>0</v>
+      </c>
+      <c r="B43" s="9" t="s">
+        <v>71</v>
+      </c>
+      <c r="C43" s="9">
+        <v>300</v>
+      </c>
+      <c r="D43" s="9">
+        <v>1.2</v>
+      </c>
+      <c r="E43" s="9">
+        <f>C43*D43</f>
+        <v>360</v>
+      </c>
+      <c r="F43" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="G43" s="9" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="44" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A44" s="9" t="b">
+        <v>0</v>
+      </c>
+      <c r="B44" s="9" t="s">
+        <v>74</v>
+      </c>
+      <c r="C44" s="9">
+        <v>100</v>
+      </c>
+      <c r="D44" s="9">
+        <v>1.2</v>
+      </c>
+      <c r="E44" s="9">
+        <f>C44*D44</f>
         <v>120</v>
       </c>
-      <c r="F42" s="9" t="s">
+      <c r="F44" s="9" t="s">
         <v>75</v>
       </c>
-      <c r="G42" s="9" t="s">
+      <c r="G44" s="9" t="s">
         <v>76</v>
-      </c>
-    </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A43" t="b">
-        <v>0</v>
-      </c>
-      <c r="C43" s="3">
-        <f>SUM(C2:C42)</f>
-        <v>20710</v>
-      </c>
-      <c r="D43" s="3"/>
-      <c r="E43" s="8">
-        <f>SUM(E2:E42)</f>
-        <v>28115</v>
-      </c>
-    </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A44" t="b">
-        <v>0</v>
       </c>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A45" t="b">
         <v>0</v>
       </c>
+      <c r="C45" s="3">
+        <f>SUM(C2:C44)</f>
+        <v>21910</v>
+      </c>
+      <c r="D45" s="3"/>
+      <c r="E45" s="8">
+        <f>SUM(E2:E44)</f>
+        <v>29435</v>
+      </c>
     </row>
     <row r="46" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A46" t="b">
@@ -1724,6 +1758,16 @@
     </row>
     <row r="61" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A61" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="62" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A62" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="63" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A63" t="b">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Nova objednavka: Rainer, 300 kg Zwetschken za 1,10, Gutau
</commit_message>
<xml_diff>
--- a/Obst.xlsx
+++ b/Obst.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\holub\AppData\Local\Temp\claude\C--Users-holub-OneDrive---Privatgymnasium-der-Herz-Jesu-Missionare-Radtour-2026\cbd12823-693e-4f3b-bb7d-65f09b0003cf\scratchpad\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DA74A388-051C-470F-A802-17F24C21CB2E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{04E16888-4E64-4BA5-9747-110D7359A3E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="83">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="85">
   <si>
     <t>Geliefert</t>
   </si>
@@ -264,6 +264,12 @@
   </si>
   <si>
     <t>Pfarre</t>
+  </si>
+  <si>
+    <t>Rainer</t>
+  </si>
+  <si>
+    <t>Erdmannsdorf 17, 4293 Gutau</t>
   </si>
   <si>
     <t>Birnen Williams</t>
@@ -719,7 +725,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H63"/>
+  <dimension ref="A1:H64"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="19" bestFit="1" customWidth="1"/>
@@ -1370,7 +1376,7 @@
         <v>1.3</v>
       </c>
       <c r="E31" s="9">
-        <f t="shared" ref="E31:E38" si="1">C31*D31</f>
+        <f t="shared" ref="E31:E39" si="1">C31*D31</f>
         <v>780</v>
       </c>
       <c r="F31" s="9" t="s">
@@ -1545,10 +1551,19 @@
       <c r="B39" s="9" t="s">
         <v>77</v>
       </c>
-      <c r="C39" s="9"/>
-      <c r="D39" s="9"/>
-      <c r="E39" s="9"/>
-      <c r="F39" s="9"/>
+      <c r="C39" s="9">
+        <v>300</v>
+      </c>
+      <c r="D39" s="9">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="E39" s="9">
+        <f t="shared" si="1"/>
+        <v>330</v>
+      </c>
+      <c r="F39" s="9" t="s">
+        <v>78</v>
+      </c>
       <c r="G39" s="9"/>
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.35">
@@ -1556,21 +1571,12 @@
         <v>0</v>
       </c>
       <c r="B40" s="9" t="s">
-        <v>6</v>
-      </c>
-      <c r="C40" s="9">
-        <v>1000</v>
-      </c>
-      <c r="D40" s="9">
-        <v>1.2</v>
-      </c>
-      <c r="E40" s="9">
-        <f>C40*D40</f>
-        <v>1200</v>
-      </c>
-      <c r="F40" s="9" t="s">
-        <v>78</v>
-      </c>
+        <v>79</v>
+      </c>
+      <c r="C40" s="9"/>
+      <c r="D40" s="9"/>
+      <c r="E40" s="9"/>
+      <c r="F40" s="9"/>
       <c r="G40" s="9"/>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.35">
@@ -1578,20 +1584,20 @@
         <v>0</v>
       </c>
       <c r="B41" s="9" t="s">
-        <v>42</v>
+        <v>6</v>
       </c>
       <c r="C41" s="9">
-        <v>1600</v>
+        <v>1000</v>
       </c>
       <c r="D41" s="9">
         <v>1.2</v>
       </c>
       <c r="E41" s="9">
         <f>C41*D41</f>
-        <v>1920</v>
+        <v>1200</v>
       </c>
       <c r="F41" s="9" t="s">
-        <v>43</v>
+        <v>80</v>
       </c>
       <c r="G41" s="9"/>
     </row>
@@ -1600,47 +1606,45 @@
         <v>0</v>
       </c>
       <c r="B42" s="9" t="s">
-        <v>79</v>
+        <v>42</v>
       </c>
       <c r="C42" s="9">
-        <v>600</v>
+        <v>1600</v>
       </c>
       <c r="D42" s="9">
         <v>1.2</v>
       </c>
       <c r="E42" s="9">
         <f>C42*D42</f>
-        <v>720</v>
+        <v>1920</v>
       </c>
       <c r="F42" s="9" t="s">
-        <v>80</v>
-      </c>
-      <c r="G42" s="9" t="s">
-        <v>81</v>
-      </c>
+        <v>43</v>
+      </c>
+      <c r="G42" s="9"/>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A43" s="9" t="b">
         <v>0</v>
       </c>
       <c r="B43" s="9" t="s">
-        <v>71</v>
+        <v>81</v>
       </c>
       <c r="C43" s="9">
-        <v>300</v>
+        <v>600</v>
       </c>
       <c r="D43" s="9">
         <v>1.2</v>
       </c>
       <c r="E43" s="9">
         <f>C43*D43</f>
-        <v>360</v>
+        <v>720</v>
       </c>
       <c r="F43" s="9" t="s">
-        <v>72</v>
+        <v>82</v>
       </c>
       <c r="G43" s="9" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.35">
@@ -1648,43 +1652,62 @@
         <v>0</v>
       </c>
       <c r="B44" s="9" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="C44" s="9">
-        <v>100</v>
+        <v>300</v>
       </c>
       <c r="D44" s="9">
         <v>1.2</v>
       </c>
       <c r="E44" s="9">
         <f>C44*D44</f>
+        <v>360</v>
+      </c>
+      <c r="F44" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="G44" s="9" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="45" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A45" s="9" t="b">
+        <v>0</v>
+      </c>
+      <c r="B45" s="9" t="s">
+        <v>74</v>
+      </c>
+      <c r="C45" s="9">
+        <v>100</v>
+      </c>
+      <c r="D45" s="9">
+        <v>1.2</v>
+      </c>
+      <c r="E45" s="9">
+        <f>C45*D45</f>
         <v>120</v>
       </c>
-      <c r="F44" s="9" t="s">
+      <c r="F45" s="9" t="s">
         <v>75</v>
       </c>
-      <c r="G44" s="9" t="s">
+      <c r="G45" s="9" t="s">
         <v>76</v>
-      </c>
-    </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A45" t="b">
-        <v>0</v>
-      </c>
-      <c r="C45" s="3">
-        <f>SUM(C2:C44)</f>
-        <v>21910</v>
-      </c>
-      <c r="D45" s="3"/>
-      <c r="E45" s="8">
-        <f>SUM(E2:E44)</f>
-        <v>29435</v>
       </c>
     </row>
     <row r="46" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A46" t="b">
         <v>0</v>
       </c>
+      <c r="C46" s="3">
+        <f>SUM(C2:C45)</f>
+        <v>22210</v>
+      </c>
+      <c r="D46" s="3"/>
+      <c r="E46" s="8">
+        <f>SUM(E2:E45)</f>
+        <v>29765</v>
+      </c>
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A47" t="b">
@@ -1768,6 +1791,11 @@
     </row>
     <row r="63" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A63" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="64" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A64" t="b">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Nova objednavka: Christof Moser, 1500 kg Zwetschken (Sorte Elena), cena k doplneni
</commit_message>
<xml_diff>
--- a/Obst.xlsx
+++ b/Obst.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\holub\AppData\Local\Temp\claude\C--Users-holub-OneDrive---Privatgymnasium-der-Herz-Jesu-Missionare-Radtour-2026\cbd12823-693e-4f3b-bb7d-65f09b0003cf\scratchpad\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{04E16888-4E64-4BA5-9747-110D7359A3E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0FC7E5C2-4ABD-4AEF-B816-D551397C4961}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="85">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="86">
   <si>
     <t>Geliefert</t>
   </si>
@@ -270,6 +270,9 @@
   </si>
   <si>
     <t>Erdmannsdorf 17, 4293 Gutau</t>
+  </si>
+  <si>
+    <t>Sorte Elena – Preis ergänzen</t>
   </si>
   <si>
     <t>Birnen Williams</t>
@@ -725,7 +728,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H64"/>
+  <dimension ref="A1:H65"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="19" bestFit="1" customWidth="1"/>
@@ -1571,34 +1574,31 @@
         <v>0</v>
       </c>
       <c r="B40" s="9" t="s">
-        <v>79</v>
-      </c>
-      <c r="C40" s="9"/>
+        <v>29</v>
+      </c>
+      <c r="C40" s="9">
+        <v>1500</v>
+      </c>
       <c r="D40" s="9"/>
       <c r="E40" s="9"/>
-      <c r="F40" s="9"/>
-      <c r="G40" s="9"/>
+      <c r="F40" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="G40" s="9" t="s">
+        <v>79</v>
+      </c>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A41" s="9" t="b">
         <v>0</v>
       </c>
       <c r="B41" s="9" t="s">
-        <v>6</v>
-      </c>
-      <c r="C41" s="9">
-        <v>1000</v>
-      </c>
-      <c r="D41" s="9">
-        <v>1.2</v>
-      </c>
-      <c r="E41" s="9">
-        <f>C41*D41</f>
-        <v>1200</v>
-      </c>
-      <c r="F41" s="9" t="s">
         <v>80</v>
       </c>
+      <c r="C41" s="9"/>
+      <c r="D41" s="9"/>
+      <c r="E41" s="9"/>
+      <c r="F41" s="9"/>
       <c r="G41" s="9"/>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.35">
@@ -1606,20 +1606,20 @@
         <v>0</v>
       </c>
       <c r="B42" s="9" t="s">
-        <v>42</v>
+        <v>6</v>
       </c>
       <c r="C42" s="9">
-        <v>1600</v>
+        <v>1000</v>
       </c>
       <c r="D42" s="9">
         <v>1.2</v>
       </c>
       <c r="E42" s="9">
         <f>C42*D42</f>
-        <v>1920</v>
+        <v>1200</v>
       </c>
       <c r="F42" s="9" t="s">
-        <v>43</v>
+        <v>81</v>
       </c>
       <c r="G42" s="9"/>
     </row>
@@ -1628,44 +1628,42 @@
         <v>0</v>
       </c>
       <c r="B43" s="9" t="s">
-        <v>81</v>
+        <v>42</v>
       </c>
       <c r="C43" s="9">
-        <v>600</v>
+        <v>1600</v>
       </c>
       <c r="D43" s="9">
         <v>1.2</v>
       </c>
       <c r="E43" s="9">
         <f>C43*D43</f>
-        <v>720</v>
+        <v>1920</v>
       </c>
       <c r="F43" s="9" t="s">
-        <v>82</v>
-      </c>
-      <c r="G43" s="9" t="s">
-        <v>83</v>
-      </c>
+        <v>43</v>
+      </c>
+      <c r="G43" s="9"/>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A44" s="9" t="b">
         <v>0</v>
       </c>
       <c r="B44" s="9" t="s">
-        <v>71</v>
+        <v>82</v>
       </c>
       <c r="C44" s="9">
-        <v>300</v>
+        <v>600</v>
       </c>
       <c r="D44" s="9">
         <v>1.2</v>
       </c>
       <c r="E44" s="9">
         <f>C44*D44</f>
-        <v>360</v>
+        <v>720</v>
       </c>
       <c r="F44" s="9" t="s">
-        <v>72</v>
+        <v>83</v>
       </c>
       <c r="G44" s="9" t="s">
         <v>84</v>
@@ -1676,43 +1674,62 @@
         <v>0</v>
       </c>
       <c r="B45" s="9" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="C45" s="9">
-        <v>100</v>
+        <v>300</v>
       </c>
       <c r="D45" s="9">
         <v>1.2</v>
       </c>
       <c r="E45" s="9">
         <f>C45*D45</f>
+        <v>360</v>
+      </c>
+      <c r="F45" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="G45" s="9" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="46" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A46" s="9" t="b">
+        <v>0</v>
+      </c>
+      <c r="B46" s="9" t="s">
+        <v>74</v>
+      </c>
+      <c r="C46" s="9">
+        <v>100</v>
+      </c>
+      <c r="D46" s="9">
+        <v>1.2</v>
+      </c>
+      <c r="E46" s="9">
+        <f>C46*D46</f>
         <v>120</v>
       </c>
-      <c r="F45" s="9" t="s">
+      <c r="F46" s="9" t="s">
         <v>75</v>
       </c>
-      <c r="G45" s="9" t="s">
+      <c r="G46" s="9" t="s">
         <v>76</v>
-      </c>
-    </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A46" t="b">
-        <v>0</v>
-      </c>
-      <c r="C46" s="3">
-        <f>SUM(C2:C45)</f>
-        <v>22210</v>
-      </c>
-      <c r="D46" s="3"/>
-      <c r="E46" s="8">
-        <f>SUM(E2:E45)</f>
-        <v>29765</v>
       </c>
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A47" t="b">
         <v>0</v>
       </c>
+      <c r="C47" s="3">
+        <f>SUM(C2:C46)</f>
+        <v>23710</v>
+      </c>
+      <c r="D47" s="3"/>
+      <c r="E47" s="8">
+        <f>SUM(E2:E46)</f>
+        <v>29765</v>
+      </c>
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A48" t="b">
@@ -1796,6 +1813,11 @@
     </row>
     <row r="64" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A64" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="65" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A65" t="b">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Moser: cena 1,10 EUR/kg
</commit_message>
<xml_diff>
--- a/Obst.xlsx
+++ b/Obst.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\holub\AppData\Local\Temp\claude\C--Users-holub-OneDrive---Privatgymnasium-der-Herz-Jesu-Missionare-Radtour-2026\cbd12823-693e-4f3b-bb7d-65f09b0003cf\scratchpad\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0FC7E5C2-4ABD-4AEF-B816-D551397C4961}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1CF0FF00-4C23-48DE-B413-4AD56E80FACB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -272,7 +272,7 @@
     <t>Erdmannsdorf 17, 4293 Gutau</t>
   </si>
   <si>
-    <t>Sorte Elena – Preis ergänzen</t>
+    <t>Sorte Elena</t>
   </si>
   <si>
     <t>Birnen Williams</t>
@@ -1379,7 +1379,7 @@
         <v>1.3</v>
       </c>
       <c r="E31" s="9">
-        <f t="shared" ref="E31:E39" si="1">C31*D31</f>
+        <f t="shared" ref="E31:E40" si="1">C31*D31</f>
         <v>780</v>
       </c>
       <c r="F31" s="9" t="s">
@@ -1579,8 +1579,13 @@
       <c r="C40" s="9">
         <v>1500</v>
       </c>
-      <c r="D40" s="9"/>
-      <c r="E40" s="9"/>
+      <c r="D40" s="9">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="E40" s="9">
+        <f t="shared" si="1"/>
+        <v>1650.0000000000002</v>
+      </c>
       <c r="F40" s="9" t="s">
         <v>30</v>
       </c>
@@ -1728,7 +1733,7 @@
       <c r="D47" s="3"/>
       <c r="E47" s="8">
         <f>SUM(E2:E46)</f>
-        <v>29765</v>
+        <v>31415</v>
       </c>
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
Doruceno Zwetschken: Flockner 200, Huber 600, Gasteiger 600, Rainer 300 kg
</commit_message>
<xml_diff>
--- a/Obst.xlsx
+++ b/Obst.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\holub\AppData\Local\Temp\claude\C--Users-holub-OneDrive---Privatgymnasium-der-Herz-Jesu-Missionare-Radtour-2026\cbd12823-693e-4f3b-bb7d-65f09b0003cf\scratchpad\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1CF0FF00-4C23-48DE-B413-4AD56E80FACB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FE374DC3-4721-4FCA-9E9A-F1F2AEC15664}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1483,7 +1483,7 @@
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A36" s="9" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B36" s="9" t="s">
         <v>45</v>
@@ -1505,7 +1505,7 @@
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A37" s="9" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B37" s="9" t="s">
         <v>2</v>
@@ -1527,7 +1527,7 @@
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A38" s="9" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B38" s="9" t="s">
         <v>42</v>
@@ -1549,7 +1549,7 @@
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A39" s="9" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B39" s="9" t="s">
         <v>77</v>

</xml_diff>

<commit_message>
Novy blok Apfel: Gerhard Bayer, 400 kg jablek, Kleinarl (cena k doplneni)
</commit_message>
<xml_diff>
--- a/Obst.xlsx
+++ b/Obst.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\holub\AppData\Local\Temp\claude\C--Users-holub-OneDrive---Privatgymnasium-der-Herz-Jesu-Missionare-Radtour-2026\cbd12823-693e-4f3b-bb7d-65f09b0003cf\scratchpad\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FE374DC3-4721-4FCA-9E9A-F1F2AEC15664}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{81E43F96-9152-478F-ABDC-E6A65017BE48}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="86">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="90">
   <si>
     <t>Geliefert</t>
   </si>
@@ -291,6 +291,18 @@
   </si>
   <si>
     <t>(47.1513091, 13.7456747)</t>
+  </si>
+  <si>
+    <t>Äpfel</t>
+  </si>
+  <si>
+    <t>Gerhard Bayer</t>
+  </si>
+  <si>
+    <t>Dorf 14, 5603 Kleinarl</t>
+  </si>
+  <si>
+    <t>Preis ergänzen</t>
   </si>
 </sst>
 </file>
@@ -728,7 +740,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H65"/>
+  <dimension ref="A1:H67"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="19" bestFit="1" customWidth="1"/>
@@ -1723,106 +1735,136 @@
       </c>
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A47" t="b">
-        <v>0</v>
-      </c>
-      <c r="C47" s="3">
-        <f>SUM(C2:C46)</f>
-        <v>23710</v>
-      </c>
-      <c r="D47" s="3"/>
-      <c r="E47" s="8">
-        <f>SUM(E2:E46)</f>
+      <c r="A47" s="9"/>
+      <c r="B47" s="9" t="s">
+        <v>86</v>
+      </c>
+      <c r="C47" s="9"/>
+      <c r="D47" s="9"/>
+      <c r="E47" s="9"/>
+      <c r="F47" s="9"/>
+      <c r="G47" s="9"/>
+    </row>
+    <row r="48" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A48" s="9" t="b">
+        <v>0</v>
+      </c>
+      <c r="B48" s="9" t="s">
+        <v>87</v>
+      </c>
+      <c r="C48" s="9">
+        <v>400</v>
+      </c>
+      <c r="D48" s="9"/>
+      <c r="E48" s="9"/>
+      <c r="F48" s="9" t="s">
+        <v>88</v>
+      </c>
+      <c r="G48" s="9" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="49" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A49" t="b">
+        <v>0</v>
+      </c>
+      <c r="C49" s="3">
+        <f>SUM(C2:C48)</f>
+        <v>24110</v>
+      </c>
+      <c r="D49" s="3"/>
+      <c r="E49" s="8">
+        <f>SUM(E2:E48)</f>
         <v>31415</v>
       </c>
     </row>
-    <row r="48" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A48" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="49" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A49" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="50" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A50" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="51" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A51" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="52" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A52" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="53" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A53" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="54" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A54" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="55" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A55" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="56" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A56" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="57" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A57" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="58" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A58" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="59" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A59" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="60" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A60" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="61" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A61" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="62" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A62" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="63" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A63" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="64" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A64" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="65" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A65" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="66" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A66" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="67" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A67" t="b">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Bayer: predbezna cena 0,70, Abholung Salzburg mozna
</commit_message>
<xml_diff>
--- a/Obst.xlsx
+++ b/Obst.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\holub\AppData\Local\Temp\claude\C--Users-holub-OneDrive---Privatgymnasium-der-Herz-Jesu-Missionare-Radtour-2026\cbd12823-693e-4f3b-bb7d-65f09b0003cf\scratchpad\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{81E43F96-9152-478F-ABDC-E6A65017BE48}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C6AB6DAC-895A-4FDF-BD81-5B5A0074CB5F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -302,7 +302,7 @@
     <t>Dorf 14, 5603 Kleinarl</t>
   </si>
   <si>
-    <t>Preis ergänzen</t>
+    <t>Abholung in Salzburg möglich – Preis 0,70 noch nicht fix vereinbart</t>
   </si>
 </sst>
 </file>
@@ -1755,8 +1755,13 @@
       <c r="C48" s="9">
         <v>400</v>
       </c>
-      <c r="D48" s="9"/>
-      <c r="E48" s="9"/>
+      <c r="D48" s="9">
+        <v>0.7</v>
+      </c>
+      <c r="E48" s="9">
+        <f>C48*D48</f>
+        <v>280</v>
+      </c>
       <c r="F48" s="9" t="s">
         <v>88</v>
       </c>
@@ -1775,7 +1780,7 @@
       <c r="D49" s="3"/>
       <c r="E49" s="8">
         <f>SUM(E2:E48)</f>
-        <v>31415</v>
+        <v>31695</v>
       </c>
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
Nova objednavka: Ferdinand Huber, 300 kg jablek, Kleinarl (cena k doplneni)
</commit_message>
<xml_diff>
--- a/Obst.xlsx
+++ b/Obst.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\holub\AppData\Local\Temp\claude\C--Users-holub-OneDrive---Privatgymnasium-der-Herz-Jesu-Missionare-Radtour-2026\cbd12823-693e-4f3b-bb7d-65f09b0003cf\scratchpad\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C6AB6DAC-895A-4FDF-BD81-5B5A0074CB5F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DE3616B8-1760-4D8B-93DB-BFD0CF0EB5AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="90">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="93">
   <si>
     <t>Geliefert</t>
   </si>
@@ -303,6 +303,15 @@
   </si>
   <si>
     <t>Abholung in Salzburg möglich – Preis 0,70 noch nicht fix vereinbart</t>
+  </si>
+  <si>
+    <t>Ferdinand Huber</t>
+  </si>
+  <si>
+    <t>Kreuzarlgasse 4, 5603 Kleinarl</t>
+  </si>
+  <si>
+    <t>Preis ergänzen</t>
   </si>
 </sst>
 </file>
@@ -740,7 +749,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H67"/>
+  <dimension ref="A1:H68"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="19" bestFit="1" customWidth="1"/>
@@ -1769,91 +1778,105 @@
         <v>89</v>
       </c>
     </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A49" t="b">
-        <v>0</v>
-      </c>
-      <c r="C49" s="3">
-        <f>SUM(C2:C48)</f>
-        <v>24110</v>
-      </c>
-      <c r="D49" s="3"/>
-      <c r="E49" s="8">
-        <f>SUM(E2:E48)</f>
+    <row r="49" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A49" s="9" t="b">
+        <v>0</v>
+      </c>
+      <c r="B49" s="9" t="s">
+        <v>90</v>
+      </c>
+      <c r="C49" s="9">
+        <v>300</v>
+      </c>
+      <c r="D49" s="9"/>
+      <c r="E49" s="9"/>
+      <c r="F49" s="9" t="s">
+        <v>91</v>
+      </c>
+      <c r="G49" s="9" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="50" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A50" t="b">
+        <v>0</v>
+      </c>
+      <c r="C50" s="3">
+        <f>SUM(C2:C49)</f>
+        <v>24410</v>
+      </c>
+      <c r="D50" s="3"/>
+      <c r="E50" s="8">
+        <f>SUM(E2:E49)</f>
         <v>31695</v>
       </c>
     </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A50" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A51" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A52" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A53" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A54" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A55" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="56" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A56" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A57" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="58" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A58" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="59" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A59" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="60" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A60" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="61" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A61" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="62" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A62" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="63" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A63" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="64" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A64" t="b">
         <v>0</v>
       </c>
@@ -1870,6 +1893,11 @@
     </row>
     <row r="67" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A67" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="68" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A68" t="b">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Ferdinand Huber: cena 0,75 EUR/kg
</commit_message>
<xml_diff>
--- a/Obst.xlsx
+++ b/Obst.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\holub\AppData\Local\Temp\claude\C--Users-holub-OneDrive---Privatgymnasium-der-Herz-Jesu-Missionare-Radtour-2026\cbd12823-693e-4f3b-bb7d-65f09b0003cf\scratchpad\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DE3616B8-1760-4D8B-93DB-BFD0CF0EB5AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{70610722-4ADD-45B7-AE7C-7E4555D91521}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="93">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="92">
   <si>
     <t>Geliefert</t>
   </si>
@@ -309,9 +309,6 @@
   </si>
   <si>
     <t>Kreuzarlgasse 4, 5603 Kleinarl</t>
-  </si>
-  <si>
-    <t>Preis ergänzen</t>
   </si>
 </sst>
 </file>
@@ -1788,14 +1785,17 @@
       <c r="C49" s="9">
         <v>300</v>
       </c>
-      <c r="D49" s="9"/>
-      <c r="E49" s="9"/>
+      <c r="D49" s="9">
+        <v>0.75</v>
+      </c>
+      <c r="E49" s="9">
+        <f>C49*D49</f>
+        <v>225</v>
+      </c>
       <c r="F49" s="9" t="s">
         <v>91</v>
       </c>
-      <c r="G49" s="9" t="s">
-        <v>92</v>
-      </c>
+      <c r="G49" s="9"/>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A50" t="b">
@@ -1808,7 +1808,7 @@
       <c r="D50" s="3"/>
       <c r="E50" s="8">
         <f>SUM(E2:E49)</f>
-        <v>31695</v>
+        <v>31920</v>
       </c>
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
Lackner: Urlaub 9.-18.9. (poznamka u obou objednavek)
</commit_message>
<xml_diff>
--- a/Obst.xlsx
+++ b/Obst.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\holub\AppData\Local\Temp\claude\C--Users-holub-OneDrive---Privatgymnasium-der-Herz-Jesu-Missionare-Radtour-2026\cbd12823-693e-4f3b-bb7d-65f09b0003cf\scratchpad\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{70610722-4ADD-45B7-AE7C-7E4555D91521}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3CC65E8C-8420-4941-B096-B3FDDF1543AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -254,7 +254,7 @@
     <t>5571 Mariapfarr</t>
   </si>
   <si>
-    <t>(47.1513091, 13.7456747) Abholung in Salzburg oder Radstadt möglich</t>
+    <t>(47.1513091, 13.7456747) Abholung in Salzburg oder Radstadt möglich – Urlaub 9.–18.9.!</t>
   </si>
   <si>
     <t>Armand, Pfarre Koppl</t>
@@ -290,7 +290,7 @@
     <t>Abholung in Salzburg oder Radstadt möglich</t>
   </si>
   <si>
-    <t>(47.1513091, 13.7456747)</t>
+    <t>(47.1513091, 13.7456747) – Urlaub 9.–18.9.!</t>
   </si>
   <si>
     <t>Äpfel</t>

</xml_diff>

<commit_message>
F. Huber: GPS centra Kleinarlu (Kreuzarlgasse v OSM neexistuje)
</commit_message>
<xml_diff>
--- a/Obst.xlsx
+++ b/Obst.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\holub\AppData\Local\Temp\claude\C--Users-holub-OneDrive---Privatgymnasium-der-Herz-Jesu-Missionare-Radtour-2026\cbd12823-693e-4f3b-bb7d-65f09b0003cf\scratchpad\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3CC65E8C-8420-4941-B096-B3FDDF1543AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1480FC60-B96D-450D-B334-38F22AE7C06C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="92">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="93">
   <si>
     <t>Geliefert</t>
   </si>
@@ -309,6 +309,9 @@
   </si>
   <si>
     <t>Kreuzarlgasse 4, 5603 Kleinarl</t>
+  </si>
+  <si>
+    <t>(47.2780439, 13.3193714)</t>
   </si>
 </sst>
 </file>
@@ -1795,7 +1798,9 @@
       <c r="F49" s="9" t="s">
         <v>91</v>
       </c>
-      <c r="G49" s="9"/>
+      <c r="G49" s="9" t="s">
+        <v>92</v>
+      </c>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A50" t="b">

</xml_diff>

<commit_message>
F. Huber: oprava ulice Kreuzsalgasse 4 + presne GPS domu
</commit_message>
<xml_diff>
--- a/Obst.xlsx
+++ b/Obst.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\holub\AppData\Local\Temp\claude\C--Users-holub-OneDrive---Privatgymnasium-der-Herz-Jesu-Missionare-Radtour-2026\cbd12823-693e-4f3b-bb7d-65f09b0003cf\scratchpad\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1480FC60-B96D-450D-B334-38F22AE7C06C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF088A87-3D46-4470-B1BB-0978B0D8E1A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -308,10 +308,10 @@
     <t>Ferdinand Huber</t>
   </si>
   <si>
-    <t>Kreuzarlgasse 4, 5603 Kleinarl</t>
-  </si>
-  <si>
-    <t>(47.2780439, 13.3193714)</t>
+    <t>Kreuzsalgasse 4, 5603 Kleinarl</t>
+  </si>
+  <si>
+    <t>(47.2765915, 13.3198029)</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
Nova objednavka: Thomas Waldhoer, 400 kg Zwetschken za 1,30, Puchkirchen
</commit_message>
<xml_diff>
--- a/Obst.xlsx
+++ b/Obst.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\holub\AppData\Local\Temp\claude\C--Users-holub-OneDrive---Privatgymnasium-der-Herz-Jesu-Missionare-Radtour-2026\cbd12823-693e-4f3b-bb7d-65f09b0003cf\scratchpad\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF088A87-3D46-4470-B1BB-0978B0D8E1A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CCA62851-0BD0-4A32-AD8D-99216514EE71}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="93">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="96">
   <si>
     <t>Geliefert</t>
   </si>
@@ -273,6 +273,15 @@
   </si>
   <si>
     <t>Sorte Elena</t>
+  </si>
+  <si>
+    <t>Thomas Waldhör</t>
+  </si>
+  <si>
+    <t>Roith 37, 4849 Puchkirchen</t>
+  </si>
+  <si>
+    <t>ca. 400 kg, Zustellung evtl. am Wochenende, Tel. 0664/4412155</t>
   </si>
   <si>
     <t>Birnen Williams</t>
@@ -749,7 +758,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H68"/>
+  <dimension ref="A1:H69"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="19" bestFit="1" customWidth="1"/>
@@ -1400,7 +1409,7 @@
         <v>1.3</v>
       </c>
       <c r="E31" s="9">
-        <f t="shared" ref="E31:E40" si="1">C31*D31</f>
+        <f t="shared" ref="E31:E41" si="1">C31*D31</f>
         <v>780</v>
       </c>
       <c r="F31" s="9" t="s">
@@ -1621,32 +1630,34 @@
       <c r="B41" s="9" t="s">
         <v>80</v>
       </c>
-      <c r="C41" s="9"/>
-      <c r="D41" s="9"/>
-      <c r="E41" s="9"/>
-      <c r="F41" s="9"/>
-      <c r="G41" s="9"/>
+      <c r="C41" s="9">
+        <v>400</v>
+      </c>
+      <c r="D41" s="9">
+        <v>1.3</v>
+      </c>
+      <c r="E41" s="9">
+        <f t="shared" si="1"/>
+        <v>520</v>
+      </c>
+      <c r="F41" s="9" t="s">
+        <v>81</v>
+      </c>
+      <c r="G41" s="9" t="s">
+        <v>82</v>
+      </c>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A42" s="9" t="b">
         <v>0</v>
       </c>
       <c r="B42" s="9" t="s">
-        <v>6</v>
-      </c>
-      <c r="C42" s="9">
-        <v>1000</v>
-      </c>
-      <c r="D42" s="9">
-        <v>1.2</v>
-      </c>
-      <c r="E42" s="9">
-        <f>C42*D42</f>
-        <v>1200</v>
-      </c>
-      <c r="F42" s="9" t="s">
-        <v>81</v>
-      </c>
+        <v>83</v>
+      </c>
+      <c r="C42" s="9"/>
+      <c r="D42" s="9"/>
+      <c r="E42" s="9"/>
+      <c r="F42" s="9"/>
       <c r="G42" s="9"/>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.35">
@@ -1654,20 +1665,20 @@
         <v>0</v>
       </c>
       <c r="B43" s="9" t="s">
-        <v>42</v>
+        <v>6</v>
       </c>
       <c r="C43" s="9">
-        <v>1600</v>
+        <v>1000</v>
       </c>
       <c r="D43" s="9">
         <v>1.2</v>
       </c>
       <c r="E43" s="9">
         <f>C43*D43</f>
-        <v>1920</v>
+        <v>1200</v>
       </c>
       <c r="F43" s="9" t="s">
-        <v>43</v>
+        <v>84</v>
       </c>
       <c r="G43" s="9"/>
     </row>
@@ -1676,47 +1687,45 @@
         <v>0</v>
       </c>
       <c r="B44" s="9" t="s">
-        <v>82</v>
+        <v>42</v>
       </c>
       <c r="C44" s="9">
-        <v>600</v>
+        <v>1600</v>
       </c>
       <c r="D44" s="9">
         <v>1.2</v>
       </c>
       <c r="E44" s="9">
         <f>C44*D44</f>
-        <v>720</v>
+        <v>1920</v>
       </c>
       <c r="F44" s="9" t="s">
-        <v>83</v>
-      </c>
-      <c r="G44" s="9" t="s">
-        <v>84</v>
-      </c>
+        <v>43</v>
+      </c>
+      <c r="G44" s="9"/>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A45" s="9" t="b">
         <v>0</v>
       </c>
       <c r="B45" s="9" t="s">
-        <v>71</v>
+        <v>85</v>
       </c>
       <c r="C45" s="9">
-        <v>300</v>
+        <v>600</v>
       </c>
       <c r="D45" s="9">
         <v>1.2</v>
       </c>
       <c r="E45" s="9">
         <f>C45*D45</f>
-        <v>360</v>
+        <v>720</v>
       </c>
       <c r="F45" s="9" t="s">
-        <v>72</v>
+        <v>86</v>
       </c>
       <c r="G45" s="9" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
     </row>
     <row r="46" spans="1:7" x14ac:dyDescent="0.35">
@@ -1724,59 +1733,59 @@
         <v>0</v>
       </c>
       <c r="B46" s="9" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="C46" s="9">
-        <v>100</v>
+        <v>300</v>
       </c>
       <c r="D46" s="9">
         <v>1.2</v>
       </c>
       <c r="E46" s="9">
         <f>C46*D46</f>
+        <v>360</v>
+      </c>
+      <c r="F46" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="G46" s="9" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="47" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A47" s="9" t="b">
+        <v>0</v>
+      </c>
+      <c r="B47" s="9" t="s">
+        <v>74</v>
+      </c>
+      <c r="C47" s="9">
+        <v>100</v>
+      </c>
+      <c r="D47" s="9">
+        <v>1.2</v>
+      </c>
+      <c r="E47" s="9">
+        <f>C47*D47</f>
         <v>120</v>
       </c>
-      <c r="F46" s="9" t="s">
+      <c r="F47" s="9" t="s">
         <v>75</v>
       </c>
-      <c r="G46" s="9" t="s">
+      <c r="G47" s="9" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="47" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A47" s="9"/>
-      <c r="B47" s="9" t="s">
-        <v>86</v>
-      </c>
-      <c r="C47" s="9"/>
-      <c r="D47" s="9"/>
-      <c r="E47" s="9"/>
-      <c r="F47" s="9"/>
-      <c r="G47" s="9"/>
-    </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A48" s="9" t="b">
-        <v>0</v>
-      </c>
+      <c r="A48" s="9"/>
       <c r="B48" s="9" t="s">
-        <v>87</v>
-      </c>
-      <c r="C48" s="9">
-        <v>400</v>
-      </c>
-      <c r="D48" s="9">
-        <v>0.7</v>
-      </c>
-      <c r="E48" s="9">
-        <f>C48*D48</f>
-        <v>280</v>
-      </c>
-      <c r="F48" s="9" t="s">
-        <v>88</v>
-      </c>
-      <c r="G48" s="9" t="s">
         <v>89</v>
       </c>
+      <c r="C48" s="9"/>
+      <c r="D48" s="9"/>
+      <c r="E48" s="9"/>
+      <c r="F48" s="9"/>
+      <c r="G48" s="9"/>
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A49" s="9" t="b">
@@ -1786,14 +1795,14 @@
         <v>90</v>
       </c>
       <c r="C49" s="9">
-        <v>300</v>
+        <v>400</v>
       </c>
       <c r="D49" s="9">
-        <v>0.75</v>
+        <v>0.7</v>
       </c>
       <c r="E49" s="9">
         <f>C49*D49</f>
-        <v>225</v>
+        <v>280</v>
       </c>
       <c r="F49" s="9" t="s">
         <v>91</v>
@@ -1803,23 +1812,42 @@
       </c>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A50" t="b">
-        <v>0</v>
-      </c>
-      <c r="C50" s="3">
-        <f>SUM(C2:C49)</f>
-        <v>24410</v>
-      </c>
-      <c r="D50" s="3"/>
-      <c r="E50" s="8">
-        <f>SUM(E2:E49)</f>
-        <v>31920</v>
+      <c r="A50" s="9" t="b">
+        <v>0</v>
+      </c>
+      <c r="B50" s="9" t="s">
+        <v>93</v>
+      </c>
+      <c r="C50" s="9">
+        <v>300</v>
+      </c>
+      <c r="D50" s="9">
+        <v>0.75</v>
+      </c>
+      <c r="E50" s="9">
+        <f>C50*D50</f>
+        <v>225</v>
+      </c>
+      <c r="F50" s="9" t="s">
+        <v>94</v>
+      </c>
+      <c r="G50" s="9" t="s">
+        <v>95</v>
       </c>
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A51" t="b">
         <v>0</v>
       </c>
+      <c r="C51" s="3">
+        <f>SUM(C2:C50)</f>
+        <v>24810</v>
+      </c>
+      <c r="D51" s="3"/>
+      <c r="E51" s="8">
+        <f>SUM(E2:E50)</f>
+        <v>32440</v>
+      </c>
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A52" t="b">
@@ -1903,6 +1931,11 @@
     </row>
     <row r="68" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A68" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="69" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A69" t="b">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Nova objednavka: Ernst Kadar, 400 kg Zwetschken za 1,10 (ab 8.9., Einwegkisten)
</commit_message>
<xml_diff>
--- a/Obst.xlsx
+++ b/Obst.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\holub\AppData\Local\Temp\claude\C--Users-holub-OneDrive---Privatgymnasium-der-Herz-Jesu-Missionare-Radtour-2026\cbd12823-693e-4f3b-bb7d-65f09b0003cf\scratchpad\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CCA62851-0BD0-4A32-AD8D-99216514EE71}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{25B17D36-C075-49C2-99B3-045D735E9375}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="96">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="118" uniqueCount="97">
   <si>
     <t>Geliefert</t>
   </si>
@@ -282,6 +282,9 @@
   </si>
   <si>
     <t>ca. 400 kg, Zustellung evtl. am Wochenende, Tel. 0664/4412155</t>
+  </si>
+  <si>
+    <t>Zustellung nach Hause erst ab Di 8.9.2026, Wunsch: Einwegkisten (nicht umfüllen)</t>
   </si>
   <si>
     <t>Birnen Williams</t>
@@ -758,7 +761,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H69"/>
+  <dimension ref="A1:H70"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="19" bestFit="1" customWidth="1"/>
@@ -1409,7 +1412,7 @@
         <v>1.3</v>
       </c>
       <c r="E31" s="9">
-        <f t="shared" ref="E31:E41" si="1">C31*D31</f>
+        <f t="shared" ref="E31:E42" si="1">C31*D31</f>
         <v>780</v>
       </c>
       <c r="F31" s="9" t="s">
@@ -1652,34 +1655,36 @@
         <v>0</v>
       </c>
       <c r="B42" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="C42" s="9">
+        <v>400</v>
+      </c>
+      <c r="D42" s="9">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="E42" s="9">
+        <f t="shared" si="1"/>
+        <v>440.00000000000006</v>
+      </c>
+      <c r="F42" s="9" t="s">
+        <v>22</v>
+      </c>
+      <c r="G42" s="9" t="s">
         <v>83</v>
       </c>
-      <c r="C42" s="9"/>
-      <c r="D42" s="9"/>
-      <c r="E42" s="9"/>
-      <c r="F42" s="9"/>
-      <c r="G42" s="9"/>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A43" s="9" t="b">
         <v>0</v>
       </c>
       <c r="B43" s="9" t="s">
-        <v>6</v>
-      </c>
-      <c r="C43" s="9">
-        <v>1000</v>
-      </c>
-      <c r="D43" s="9">
-        <v>1.2</v>
-      </c>
-      <c r="E43" s="9">
-        <f>C43*D43</f>
-        <v>1200</v>
-      </c>
-      <c r="F43" s="9" t="s">
         <v>84</v>
       </c>
+      <c r="C43" s="9"/>
+      <c r="D43" s="9"/>
+      <c r="E43" s="9"/>
+      <c r="F43" s="9"/>
       <c r="G43" s="9"/>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.35">
@@ -1687,20 +1692,20 @@
         <v>0</v>
       </c>
       <c r="B44" s="9" t="s">
-        <v>42</v>
+        <v>6</v>
       </c>
       <c r="C44" s="9">
-        <v>1600</v>
+        <v>1000</v>
       </c>
       <c r="D44" s="9">
         <v>1.2</v>
       </c>
       <c r="E44" s="9">
         <f>C44*D44</f>
-        <v>1920</v>
+        <v>1200</v>
       </c>
       <c r="F44" s="9" t="s">
-        <v>43</v>
+        <v>85</v>
       </c>
       <c r="G44" s="9"/>
     </row>
@@ -1709,44 +1714,42 @@
         <v>0</v>
       </c>
       <c r="B45" s="9" t="s">
-        <v>85</v>
+        <v>42</v>
       </c>
       <c r="C45" s="9">
-        <v>600</v>
+        <v>1600</v>
       </c>
       <c r="D45" s="9">
         <v>1.2</v>
       </c>
       <c r="E45" s="9">
         <f>C45*D45</f>
-        <v>720</v>
+        <v>1920</v>
       </c>
       <c r="F45" s="9" t="s">
-        <v>86</v>
-      </c>
-      <c r="G45" s="9" t="s">
-        <v>87</v>
-      </c>
+        <v>43</v>
+      </c>
+      <c r="G45" s="9"/>
     </row>
     <row r="46" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A46" s="9" t="b">
         <v>0</v>
       </c>
       <c r="B46" s="9" t="s">
-        <v>71</v>
+        <v>86</v>
       </c>
       <c r="C46" s="9">
-        <v>300</v>
+        <v>600</v>
       </c>
       <c r="D46" s="9">
         <v>1.2</v>
       </c>
       <c r="E46" s="9">
         <f>C46*D46</f>
-        <v>360</v>
+        <v>720</v>
       </c>
       <c r="F46" s="9" t="s">
-        <v>72</v>
+        <v>87</v>
       </c>
       <c r="G46" s="9" t="s">
         <v>88</v>
@@ -1757,102 +1760,121 @@
         <v>0</v>
       </c>
       <c r="B47" s="9" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="C47" s="9">
-        <v>100</v>
+        <v>300</v>
       </c>
       <c r="D47" s="9">
         <v>1.2</v>
       </c>
       <c r="E47" s="9">
         <f>C47*D47</f>
+        <v>360</v>
+      </c>
+      <c r="F47" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="G47" s="9" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="48" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A48" s="9" t="b">
+        <v>0</v>
+      </c>
+      <c r="B48" s="9" t="s">
+        <v>74</v>
+      </c>
+      <c r="C48" s="9">
+        <v>100</v>
+      </c>
+      <c r="D48" s="9">
+        <v>1.2</v>
+      </c>
+      <c r="E48" s="9">
+        <f>C48*D48</f>
         <v>120</v>
       </c>
-      <c r="F47" s="9" t="s">
+      <c r="F48" s="9" t="s">
         <v>75</v>
       </c>
-      <c r="G47" s="9" t="s">
+      <c r="G48" s="9" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="48" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A48" s="9"/>
-      <c r="B48" s="9" t="s">
-        <v>89</v>
-      </c>
-      <c r="C48" s="9"/>
-      <c r="D48" s="9"/>
-      <c r="E48" s="9"/>
-      <c r="F48" s="9"/>
-      <c r="G48" s="9"/>
-    </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A49" s="9" t="b">
-        <v>0</v>
-      </c>
+      <c r="A49" s="9"/>
       <c r="B49" s="9" t="s">
         <v>90</v>
       </c>
-      <c r="C49" s="9">
-        <v>400</v>
-      </c>
-      <c r="D49" s="9">
-        <v>0.7</v>
-      </c>
-      <c r="E49" s="9">
-        <f>C49*D49</f>
-        <v>280</v>
-      </c>
-      <c r="F49" s="9" t="s">
-        <v>91</v>
-      </c>
-      <c r="G49" s="9" t="s">
-        <v>92</v>
-      </c>
+      <c r="C49" s="9"/>
+      <c r="D49" s="9"/>
+      <c r="E49" s="9"/>
+      <c r="F49" s="9"/>
+      <c r="G49" s="9"/>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A50" s="9" t="b">
         <v>0</v>
       </c>
       <c r="B50" s="9" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="C50" s="9">
-        <v>300</v>
+        <v>400</v>
       </c>
       <c r="D50" s="9">
-        <v>0.75</v>
+        <v>0.7</v>
       </c>
       <c r="E50" s="9">
         <f>C50*D50</f>
+        <v>280</v>
+      </c>
+      <c r="F50" s="9" t="s">
+        <v>92</v>
+      </c>
+      <c r="G50" s="9" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="51" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A51" s="9" t="b">
+        <v>0</v>
+      </c>
+      <c r="B51" s="9" t="s">
+        <v>94</v>
+      </c>
+      <c r="C51" s="9">
+        <v>300</v>
+      </c>
+      <c r="D51" s="9">
+        <v>0.75</v>
+      </c>
+      <c r="E51" s="9">
+        <f>C51*D51</f>
         <v>225</v>
       </c>
-      <c r="F50" s="9" t="s">
-        <v>94</v>
-      </c>
-      <c r="G50" s="9" t="s">
+      <c r="F51" s="9" t="s">
         <v>95</v>
       </c>
-    </row>
-    <row r="51" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A51" t="b">
-        <v>0</v>
-      </c>
-      <c r="C51" s="3">
-        <f>SUM(C2:C50)</f>
-        <v>24810</v>
-      </c>
-      <c r="D51" s="3"/>
-      <c r="E51" s="8">
-        <f>SUM(E2:E50)</f>
-        <v>32440</v>
+      <c r="G51" s="9" t="s">
+        <v>96</v>
       </c>
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A52" t="b">
         <v>0</v>
       </c>
+      <c r="C52" s="3">
+        <f>SUM(C2:C51)</f>
+        <v>25210</v>
+      </c>
+      <c r="D52" s="3"/>
+      <c r="E52" s="8">
+        <f>SUM(E2:E51)</f>
+        <v>32880</v>
+      </c>
     </row>
     <row r="53" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A53" t="b">
@@ -1936,6 +1958,11 @@
     </row>
     <row r="69" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A69" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="70" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A70" t="b">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Kadar: adresa Altaussee 29
</commit_message>
<xml_diff>
--- a/Obst.xlsx
+++ b/Obst.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\holub\AppData\Local\Temp\claude\C--Users-holub-OneDrive---Privatgymnasium-der-Herz-Jesu-Missionare-Radtour-2026\cbd12823-693e-4f3b-bb7d-65f09b0003cf\scratchpad\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{25B17D36-C075-49C2-99B3-045D735E9375}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF38AA2F-FCB8-4250-A8FF-6C2CC44C46DC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="118" uniqueCount="97">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="118" uniqueCount="98">
   <si>
     <t>Geliefert</t>
   </si>
@@ -282,6 +282,9 @@
   </si>
   <si>
     <t>ca. 400 kg, Zustellung evtl. am Wochenende, Tel. 0664/4412155</t>
+  </si>
+  <si>
+    <t>Altaussee 29, 8992 Altaussee</t>
   </si>
   <si>
     <t>Zustellung nach Hause erst ab Di 8.9.2026, Wunsch: Einwegkisten (nicht umfüllen)</t>
@@ -1668,10 +1671,10 @@
         <v>440.00000000000006</v>
       </c>
       <c r="F42" s="9" t="s">
-        <v>22</v>
+        <v>83</v>
       </c>
       <c r="G42" s="9" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.35">
@@ -1679,7 +1682,7 @@
         <v>0</v>
       </c>
       <c r="B43" s="9" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="C43" s="9"/>
       <c r="D43" s="9"/>
@@ -1705,7 +1708,7 @@
         <v>1200</v>
       </c>
       <c r="F44" s="9" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="G44" s="9"/>
     </row>
@@ -1736,7 +1739,7 @@
         <v>0</v>
       </c>
       <c r="B46" s="9" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="C46" s="9">
         <v>600</v>
@@ -1749,10 +1752,10 @@
         <v>720</v>
       </c>
       <c r="F46" s="9" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="G46" s="9" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.35">
@@ -1776,7 +1779,7 @@
         <v>72</v>
       </c>
       <c r="G47" s="9" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.35">
@@ -1806,7 +1809,7 @@
     <row r="49" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A49" s="9"/>
       <c r="B49" s="9" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C49" s="9"/>
       <c r="D49" s="9"/>
@@ -1819,7 +1822,7 @@
         <v>0</v>
       </c>
       <c r="B50" s="9" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="C50" s="9">
         <v>400</v>
@@ -1832,10 +1835,10 @@
         <v>280</v>
       </c>
       <c r="F50" s="9" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="G50" s="9" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.35">
@@ -1843,7 +1846,7 @@
         <v>0</v>
       </c>
       <c r="B51" s="9" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="C51" s="9">
         <v>300</v>
@@ -1856,10 +1859,10 @@
         <v>225</v>
       </c>
       <c r="F51" s="9" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="G51" s="9" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
Kadar: GPS stredu Altaussee (Nominatim dava katastralni uzemi v horach)
</commit_message>
<xml_diff>
--- a/Obst.xlsx
+++ b/Obst.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\holub\AppData\Local\Temp\claude\C--Users-holub-OneDrive---Privatgymnasium-der-Herz-Jesu-Missionare-Radtour-2026\cbd12823-693e-4f3b-bb7d-65f09b0003cf\scratchpad\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF38AA2F-FCB8-4250-A8FF-6C2CC44C46DC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD0DCB17-7069-41E7-9164-DE7FB38D4AA8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -287,7 +287,7 @@
     <t>Altaussee 29, 8992 Altaussee</t>
   </si>
   <si>
-    <t>Zustellung nach Hause erst ab Di 8.9.2026, Wunsch: Einwegkisten (nicht umfüllen)</t>
+    <t>(47.6398954, 13.7640614) Zustellung nach Hause erst ab Di 8.9.2026, Wunsch: Einwegkisten (nicht umfüllen)</t>
   </si>
   <si>
     <t>Birnen Williams</t>

</xml_diff>

<commit_message>
Kadar: visne na stejnou adresu Altaussee 29 (jeden bod na mape)
</commit_message>
<xml_diff>
--- a/Obst.xlsx
+++ b/Obst.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\holub\AppData\Local\Temp\claude\C--Users-holub-OneDrive---Privatgymnasium-der-Herz-Jesu-Missionare-Radtour-2026\cbd12823-693e-4f3b-bb7d-65f09b0003cf\scratchpad\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD0DCB17-7069-41E7-9164-DE7FB38D4AA8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2E3D79DE-46D7-47DD-885B-BE226BBC9639}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="118" uniqueCount="98">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="118" uniqueCount="97">
   <si>
     <t>Geliefert</t>
   </si>
@@ -101,7 +101,7 @@
     <t>Ernst Kadar</t>
   </si>
   <si>
-    <t>8992 Altaussee</t>
+    <t>Altaussee 29, 8992 Altaussee</t>
   </si>
   <si>
     <t>abgeholt bei Kalteis (Waizenkirchen), für nächstes Jahr</t>
@@ -282,9 +282,6 @@
   </si>
   <si>
     <t>ca. 400 kg, Zustellung evtl. am Wochenende, Tel. 0664/4412155</t>
-  </si>
-  <si>
-    <t>Altaussee 29, 8992 Altaussee</t>
   </si>
   <si>
     <t>(47.6398954, 13.7640614) Zustellung nach Hause erst ab Di 8.9.2026, Wunsch: Einwegkisten (nicht umfüllen)</t>
@@ -1671,10 +1668,10 @@
         <v>440.00000000000006</v>
       </c>
       <c r="F42" s="9" t="s">
+        <v>22</v>
+      </c>
+      <c r="G42" s="9" t="s">
         <v>83</v>
-      </c>
-      <c r="G42" s="9" t="s">
-        <v>84</v>
       </c>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.35">
@@ -1682,7 +1679,7 @@
         <v>0</v>
       </c>
       <c r="B43" s="9" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="C43" s="9"/>
       <c r="D43" s="9"/>
@@ -1708,7 +1705,7 @@
         <v>1200</v>
       </c>
       <c r="F44" s="9" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="G44" s="9"/>
     </row>
@@ -1739,7 +1736,7 @@
         <v>0</v>
       </c>
       <c r="B46" s="9" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C46" s="9">
         <v>600</v>
@@ -1752,10 +1749,10 @@
         <v>720</v>
       </c>
       <c r="F46" s="9" t="s">
+        <v>87</v>
+      </c>
+      <c r="G46" s="9" t="s">
         <v>88</v>
-      </c>
-      <c r="G46" s="9" t="s">
-        <v>89</v>
       </c>
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.35">
@@ -1779,7 +1776,7 @@
         <v>72</v>
       </c>
       <c r="G47" s="9" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.35">
@@ -1809,7 +1806,7 @@
     <row r="49" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A49" s="9"/>
       <c r="B49" s="9" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C49" s="9"/>
       <c r="D49" s="9"/>
@@ -1822,7 +1819,7 @@
         <v>0</v>
       </c>
       <c r="B50" s="9" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="C50" s="9">
         <v>400</v>
@@ -1835,10 +1832,10 @@
         <v>280</v>
       </c>
       <c r="F50" s="9" t="s">
+        <v>92</v>
+      </c>
+      <c r="G50" s="9" t="s">
         <v>93</v>
-      </c>
-      <c r="G50" s="9" t="s">
-        <v>94</v>
       </c>
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.35">
@@ -1846,7 +1843,7 @@
         <v>0</v>
       </c>
       <c r="B51" s="9" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="C51" s="9">
         <v>300</v>
@@ -1859,10 +1856,10 @@
         <v>225</v>
       </c>
       <c r="F51" s="9" t="s">
+        <v>95</v>
+      </c>
+      <c r="G51" s="9" t="s">
         <v>96</v>
-      </c>
-      <c r="G51" s="9" t="s">
-        <v>97</v>
       </c>
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
Endesgrabner storno 2026 (OP, ozve se 2027); app: zrusene objednavky preskrtnute v rezimu Vse, mimo soucty a mapu
</commit_message>
<xml_diff>
--- a/Obst.xlsx
+++ b/Obst.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\holub\AppData\Local\Temp\claude\C--Users-holub-OneDrive---Privatgymnasium-der-Herz-Jesu-Missionare-Radtour-2026\cbd12823-693e-4f3b-bb7d-65f09b0003cf\scratchpad\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2E3D79DE-46D7-47DD-885B-BE226BBC9639}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ED65715C-0474-4D51-8809-AEDB19EF3389}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -239,7 +239,7 @@
     <t>Rabenschwand 48, 4894 Oberhofen am Irrsee</t>
   </si>
   <si>
-    <t>telefonisch bestellt +43 664 4233933</t>
+    <t>STORNIERT 2026 (OP) – ursprünglich 600 kg à 1,30 – meldet sich 2027 wieder, Tel. +43 664 4233933</t>
   </si>
   <si>
     <t>Daniel Steiner</t>
@@ -1406,15 +1406,10 @@
         <v>66</v>
       </c>
       <c r="C31" s="9">
-        <v>600</v>
-      </c>
-      <c r="D31" s="9">
-        <v>1.3</v>
-      </c>
-      <c r="E31" s="9">
-        <f t="shared" ref="E31:E42" si="1">C31*D31</f>
-        <v>780</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="D31" s="9"/>
+      <c r="E31" s="9"/>
       <c r="F31" s="9" t="s">
         <v>67</v>
       </c>
@@ -1436,7 +1431,7 @@
         <v>1.3</v>
       </c>
       <c r="E32" s="9">
-        <f t="shared" si="1"/>
+        <f t="shared" ref="E32:E42" si="1">C32*D32</f>
         <v>390</v>
       </c>
       <c r="F32" s="9" t="s">
@@ -1868,12 +1863,12 @@
       </c>
       <c r="C52" s="3">
         <f>SUM(C2:C51)</f>
-        <v>25210</v>
+        <v>24610</v>
       </c>
       <c r="D52" s="3"/>
       <c r="E52" s="8">
         <f>SUM(E2:E51)</f>
-        <v>32880</v>
+        <v>32100</v>
       </c>
     </row>
     <row r="53" spans="1:7" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
Nova objednavka: Friedl, 500 kg Zwetschken za 0,95, Esternberg
</commit_message>
<xml_diff>
--- a/Obst.xlsx
+++ b/Obst.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\holub\AppData\Local\Temp\claude\C--Users-holub-OneDrive---Privatgymnasium-der-Herz-Jesu-Missionare-Radtour-2026\cbd12823-693e-4f3b-bb7d-65f09b0003cf\scratchpad\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ED65715C-0474-4D51-8809-AEDB19EF3389}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{522C8E42-D5E9-44A8-955E-AA9CFEE3AE61}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="118" uniqueCount="97">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="99">
   <si>
     <t>Geliefert</t>
   </si>
@@ -285,6 +285,12 @@
   </si>
   <si>
     <t>(47.6398954, 13.7640614) Zustellung nach Hause erst ab Di 8.9.2026, Wunsch: Einwegkisten (nicht umfüllen)</t>
+  </si>
+  <si>
+    <t>Friedl</t>
+  </si>
+  <si>
+    <t>Pfarrhof 11, 4092 Esternberg</t>
   </si>
   <si>
     <t>Birnen Williams</t>
@@ -761,7 +767,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H70"/>
+  <dimension ref="A1:H71"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="19" bestFit="1" customWidth="1"/>
@@ -1431,7 +1437,7 @@
         <v>1.3</v>
       </c>
       <c r="E32" s="9">
-        <f t="shared" ref="E32:E42" si="1">C32*D32</f>
+        <f t="shared" ref="E32:E43" si="1">C32*D32</f>
         <v>390</v>
       </c>
       <c r="F32" s="9" t="s">
@@ -1676,10 +1682,19 @@
       <c r="B43" s="9" t="s">
         <v>84</v>
       </c>
-      <c r="C43" s="9"/>
-      <c r="D43" s="9"/>
-      <c r="E43" s="9"/>
-      <c r="F43" s="9"/>
+      <c r="C43" s="9">
+        <v>500</v>
+      </c>
+      <c r="D43" s="9">
+        <v>0.95</v>
+      </c>
+      <c r="E43" s="9">
+        <f t="shared" si="1"/>
+        <v>475</v>
+      </c>
+      <c r="F43" s="9" t="s">
+        <v>85</v>
+      </c>
       <c r="G43" s="9"/>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.35">
@@ -1687,21 +1702,12 @@
         <v>0</v>
       </c>
       <c r="B44" s="9" t="s">
-        <v>6</v>
-      </c>
-      <c r="C44" s="9">
-        <v>1000</v>
-      </c>
-      <c r="D44" s="9">
-        <v>1.2</v>
-      </c>
-      <c r="E44" s="9">
-        <f>C44*D44</f>
-        <v>1200</v>
-      </c>
-      <c r="F44" s="9" t="s">
-        <v>85</v>
-      </c>
+        <v>86</v>
+      </c>
+      <c r="C44" s="9"/>
+      <c r="D44" s="9"/>
+      <c r="E44" s="9"/>
+      <c r="F44" s="9"/>
       <c r="G44" s="9"/>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.35">
@@ -1709,20 +1715,20 @@
         <v>0</v>
       </c>
       <c r="B45" s="9" t="s">
-        <v>42</v>
+        <v>6</v>
       </c>
       <c r="C45" s="9">
-        <v>1600</v>
+        <v>1000</v>
       </c>
       <c r="D45" s="9">
         <v>1.2</v>
       </c>
       <c r="E45" s="9">
         <f>C45*D45</f>
-        <v>1920</v>
+        <v>1200</v>
       </c>
       <c r="F45" s="9" t="s">
-        <v>43</v>
+        <v>87</v>
       </c>
       <c r="G45" s="9"/>
     </row>
@@ -1731,47 +1737,45 @@
         <v>0</v>
       </c>
       <c r="B46" s="9" t="s">
-        <v>86</v>
+        <v>42</v>
       </c>
       <c r="C46" s="9">
-        <v>600</v>
+        <v>1600</v>
       </c>
       <c r="D46" s="9">
         <v>1.2</v>
       </c>
       <c r="E46" s="9">
         <f>C46*D46</f>
-        <v>720</v>
+        <v>1920</v>
       </c>
       <c r="F46" s="9" t="s">
-        <v>87</v>
-      </c>
-      <c r="G46" s="9" t="s">
-        <v>88</v>
-      </c>
+        <v>43</v>
+      </c>
+      <c r="G46" s="9"/>
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A47" s="9" t="b">
         <v>0</v>
       </c>
       <c r="B47" s="9" t="s">
-        <v>71</v>
+        <v>88</v>
       </c>
       <c r="C47" s="9">
-        <v>300</v>
+        <v>600</v>
       </c>
       <c r="D47" s="9">
         <v>1.2</v>
       </c>
       <c r="E47" s="9">
         <f>C47*D47</f>
-        <v>360</v>
+        <v>720</v>
       </c>
       <c r="F47" s="9" t="s">
-        <v>72</v>
+        <v>89</v>
       </c>
       <c r="G47" s="9" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.35">
@@ -1779,102 +1783,121 @@
         <v>0</v>
       </c>
       <c r="B48" s="9" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="C48" s="9">
-        <v>100</v>
+        <v>300</v>
       </c>
       <c r="D48" s="9">
         <v>1.2</v>
       </c>
       <c r="E48" s="9">
         <f>C48*D48</f>
+        <v>360</v>
+      </c>
+      <c r="F48" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="G48" s="9" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="49" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A49" s="9" t="b">
+        <v>0</v>
+      </c>
+      <c r="B49" s="9" t="s">
+        <v>74</v>
+      </c>
+      <c r="C49" s="9">
+        <v>100</v>
+      </c>
+      <c r="D49" s="9">
+        <v>1.2</v>
+      </c>
+      <c r="E49" s="9">
+        <f>C49*D49</f>
         <v>120</v>
       </c>
-      <c r="F48" s="9" t="s">
+      <c r="F49" s="9" t="s">
         <v>75</v>
       </c>
-      <c r="G48" s="9" t="s">
+      <c r="G49" s="9" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="49" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A49" s="9"/>
-      <c r="B49" s="9" t="s">
-        <v>90</v>
-      </c>
-      <c r="C49" s="9"/>
-      <c r="D49" s="9"/>
-      <c r="E49" s="9"/>
-      <c r="F49" s="9"/>
-      <c r="G49" s="9"/>
-    </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A50" s="9" t="b">
-        <v>0</v>
-      </c>
+      <c r="A50" s="9"/>
       <c r="B50" s="9" t="s">
-        <v>91</v>
-      </c>
-      <c r="C50" s="9">
-        <v>400</v>
-      </c>
-      <c r="D50" s="9">
-        <v>0.7</v>
-      </c>
-      <c r="E50" s="9">
-        <f>C50*D50</f>
-        <v>280</v>
-      </c>
-      <c r="F50" s="9" t="s">
         <v>92</v>
       </c>
-      <c r="G50" s="9" t="s">
-        <v>93</v>
-      </c>
+      <c r="C50" s="9"/>
+      <c r="D50" s="9"/>
+      <c r="E50" s="9"/>
+      <c r="F50" s="9"/>
+      <c r="G50" s="9"/>
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A51" s="9" t="b">
         <v>0</v>
       </c>
       <c r="B51" s="9" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="C51" s="9">
-        <v>300</v>
+        <v>400</v>
       </c>
       <c r="D51" s="9">
-        <v>0.75</v>
+        <v>0.7</v>
       </c>
       <c r="E51" s="9">
         <f>C51*D51</f>
+        <v>280</v>
+      </c>
+      <c r="F51" s="9" t="s">
+        <v>94</v>
+      </c>
+      <c r="G51" s="9" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="52" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A52" s="9" t="b">
+        <v>0</v>
+      </c>
+      <c r="B52" s="9" t="s">
+        <v>96</v>
+      </c>
+      <c r="C52" s="9">
+        <v>300</v>
+      </c>
+      <c r="D52" s="9">
+        <v>0.75</v>
+      </c>
+      <c r="E52" s="9">
+        <f>C52*D52</f>
         <v>225</v>
       </c>
-      <c r="F51" s="9" t="s">
-        <v>95</v>
-      </c>
-      <c r="G51" s="9" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="52" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A52" t="b">
-        <v>0</v>
-      </c>
-      <c r="C52" s="3">
-        <f>SUM(C2:C51)</f>
-        <v>24610</v>
-      </c>
-      <c r="D52" s="3"/>
-      <c r="E52" s="8">
-        <f>SUM(E2:E51)</f>
-        <v>32100</v>
+      <c r="F52" s="9" t="s">
+        <v>97</v>
+      </c>
+      <c r="G52" s="9" t="s">
+        <v>98</v>
       </c>
     </row>
     <row r="53" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A53" t="b">
         <v>0</v>
       </c>
+      <c r="C53" s="3">
+        <f>SUM(C2:C52)</f>
+        <v>25110</v>
+      </c>
+      <c r="D53" s="3"/>
+      <c r="E53" s="8">
+        <f>SUM(E2:E52)</f>
+        <v>32575</v>
+      </c>
     </row>
     <row r="54" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A54" t="b">
@@ -1958,6 +1981,11 @@
     </row>
     <row r="70" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A70" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="71" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A71" t="b">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Gasteiger: Birnen Williams 1600 -> 1000 kg (2 palety)
</commit_message>
<xml_diff>
--- a/Obst.xlsx
+++ b/Obst.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\holub\AppData\Local\Temp\claude\C--Users-holub-OneDrive---Privatgymnasium-der-Herz-Jesu-Missionare-Radtour-2026\cbd12823-693e-4f3b-bb7d-65f09b0003cf\scratchpad\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{522C8E42-D5E9-44A8-955E-AA9CFEE3AE61}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E7453CE5-3347-464D-A32C-F16907A27C17}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="99">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="100">
   <si>
     <t>Geliefert</t>
   </si>
@@ -297,6 +297,9 @@
   </si>
   <si>
     <t>Haagweg 7, 5550 Radstadt</t>
+  </si>
+  <si>
+    <t>2 Paletten, ca. 1000 kg (statt 1600)</t>
   </si>
   <si>
     <t>Christian Schlick</t>
@@ -1740,26 +1743,28 @@
         <v>42</v>
       </c>
       <c r="C46" s="9">
-        <v>1600</v>
+        <v>1000</v>
       </c>
       <c r="D46" s="9">
         <v>1.2</v>
       </c>
       <c r="E46" s="9">
         <f>C46*D46</f>
-        <v>1920</v>
+        <v>1200</v>
       </c>
       <c r="F46" s="9" t="s">
         <v>43</v>
       </c>
-      <c r="G46" s="9"/>
+      <c r="G46" s="9" t="s">
+        <v>88</v>
+      </c>
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A47" s="9" t="b">
         <v>0</v>
       </c>
       <c r="B47" s="9" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C47" s="9">
         <v>600</v>
@@ -1772,10 +1777,10 @@
         <v>720</v>
       </c>
       <c r="F47" s="9" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="G47" s="9" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.35">
@@ -1799,7 +1804,7 @@
         <v>72</v>
       </c>
       <c r="G48" s="9" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.35">
@@ -1829,7 +1834,7 @@
     <row r="50" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A50" s="9"/>
       <c r="B50" s="9" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="C50" s="9"/>
       <c r="D50" s="9"/>
@@ -1842,7 +1847,7 @@
         <v>0</v>
       </c>
       <c r="B51" s="9" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="C51" s="9">
         <v>400</v>
@@ -1855,10 +1860,10 @@
         <v>280</v>
       </c>
       <c r="F51" s="9" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="G51" s="9" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.35">
@@ -1866,7 +1871,7 @@
         <v>0</v>
       </c>
       <c r="B52" s="9" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="C52" s="9">
         <v>300</v>
@@ -1879,10 +1884,10 @@
         <v>225</v>
       </c>
       <c r="F52" s="9" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="G52" s="9" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
     </row>
     <row r="53" spans="1:7" x14ac:dyDescent="0.35">
@@ -1891,12 +1896,12 @@
       </c>
       <c r="C53" s="3">
         <f>SUM(C2:C52)</f>
-        <v>25110</v>
+        <v>24510</v>
       </c>
       <c r="D53" s="3"/>
       <c r="E53" s="8">
         <f>SUM(E2:E52)</f>
-        <v>32575</v>
+        <v>31855</v>
       </c>
     </row>
     <row r="54" spans="1:7" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
Doruceno Zwetschken: Waldhoer 400 kg, Herz Jesu 380 kg/350 EUR, Steiner 260 kg/290 EUR
</commit_message>
<xml_diff>
--- a/Obst.xlsx
+++ b/Obst.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\holub\AppData\Local\Temp\claude\C--Users-holub-OneDrive---Privatgymnasium-der-Herz-Jesu-Missionare-Radtour-2026\cbd12823-693e-4f3b-bb7d-65f09b0003cf\scratchpad\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E7453CE5-3347-464D-A32C-F16907A27C17}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{70F9DF02-08D9-4FC8-B20C-369C564F47D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="100">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="123" uniqueCount="102">
   <si>
     <t>Geliefert</t>
   </si>
@@ -242,10 +242,16 @@
     <t>STORNIERT 2026 (OP) – ursprünglich 600 kg à 1,30 – meldet sich 2027 wieder, Tel. +43 664 4233933</t>
   </si>
   <si>
+    <t>pauschal 350 €</t>
+  </si>
+  <si>
     <t>Daniel Steiner</t>
   </si>
   <si>
     <t>Markt 30, 5431 Kuchl</t>
+  </si>
+  <si>
+    <t>pauschal 290 €</t>
   </si>
   <si>
     <t>Johann Lackner</t>
@@ -1428,54 +1434,60 @@
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A32" s="9" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B32" s="9" t="s">
         <v>53</v>
       </c>
       <c r="C32" s="9">
-        <v>300</v>
+        <v>380</v>
       </c>
       <c r="D32" s="9">
-        <v>1.3</v>
+        <f>350/380</f>
+        <v>0.92105263157894735</v>
       </c>
       <c r="E32" s="9">
         <f t="shared" ref="E32:E43" si="1">C32*D32</f>
-        <v>390</v>
+        <v>350</v>
       </c>
       <c r="F32" s="9" t="s">
         <v>54</v>
       </c>
-      <c r="G32" s="9"/>
+      <c r="G32" s="9" t="s">
+        <v>69</v>
+      </c>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A33" s="9" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B33" s="9" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="C33" s="9">
-        <v>250</v>
+        <v>260</v>
       </c>
       <c r="D33" s="9">
-        <v>1.3</v>
+        <f>290/260</f>
+        <v>1.1153846153846154</v>
       </c>
       <c r="E33" s="9">
         <f t="shared" si="1"/>
-        <v>325</v>
+        <v>290</v>
       </c>
       <c r="F33" s="9" t="s">
-        <v>70</v>
-      </c>
-      <c r="G33" s="9"/>
+        <v>71</v>
+      </c>
+      <c r="G33" s="9" t="s">
+        <v>72</v>
+      </c>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A34" s="9" t="b">
         <v>0</v>
       </c>
       <c r="B34" s="9" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="C34" s="9">
         <v>300</v>
@@ -1488,10 +1500,10 @@
         <v>390</v>
       </c>
       <c r="F34" s="9" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="G34" s="9" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.35">
@@ -1499,7 +1511,7 @@
         <v>0</v>
       </c>
       <c r="B35" s="9" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="C35" s="9">
         <v>100</v>
@@ -1512,10 +1524,10 @@
         <v>130</v>
       </c>
       <c r="F35" s="9" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="G35" s="9" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.35">
@@ -1589,7 +1601,7 @@
         <v>1</v>
       </c>
       <c r="B39" s="9" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="C39" s="9">
         <v>300</v>
@@ -1602,7 +1614,7 @@
         <v>330</v>
       </c>
       <c r="F39" s="9" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="G39" s="9"/>
     </row>
@@ -1627,15 +1639,15 @@
         <v>30</v>
       </c>
       <c r="G40" s="9" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A41" s="9" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B41" s="9" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="C41" s="9">
         <v>400</v>
@@ -1648,10 +1660,10 @@
         <v>520</v>
       </c>
       <c r="F41" s="9" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="G41" s="9" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.35">
@@ -1675,7 +1687,7 @@
         <v>22</v>
       </c>
       <c r="G42" s="9" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.35">
@@ -1683,7 +1695,7 @@
         <v>0</v>
       </c>
       <c r="B43" s="9" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="C43" s="9">
         <v>500</v>
@@ -1696,7 +1708,7 @@
         <v>475</v>
       </c>
       <c r="F43" s="9" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="G43" s="9"/>
     </row>
@@ -1705,7 +1717,7 @@
         <v>0</v>
       </c>
       <c r="B44" s="9" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="C44" s="9"/>
       <c r="D44" s="9"/>
@@ -1731,7 +1743,7 @@
         <v>1200</v>
       </c>
       <c r="F45" s="9" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="G45" s="9"/>
     </row>
@@ -1756,7 +1768,7 @@
         <v>43</v>
       </c>
       <c r="G46" s="9" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.35">
@@ -1764,7 +1776,7 @@
         <v>0</v>
       </c>
       <c r="B47" s="9" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="C47" s="9">
         <v>600</v>
@@ -1777,10 +1789,10 @@
         <v>720</v>
       </c>
       <c r="F47" s="9" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="G47" s="9" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.35">
@@ -1788,7 +1800,7 @@
         <v>0</v>
       </c>
       <c r="B48" s="9" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="C48" s="9">
         <v>300</v>
@@ -1801,10 +1813,10 @@
         <v>360</v>
       </c>
       <c r="F48" s="9" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="G48" s="9" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.35">
@@ -1812,7 +1824,7 @@
         <v>0</v>
       </c>
       <c r="B49" s="9" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="C49" s="9">
         <v>100</v>
@@ -1825,16 +1837,16 @@
         <v>120</v>
       </c>
       <c r="F49" s="9" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="G49" s="9" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A50" s="9"/>
       <c r="B50" s="9" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="C50" s="9"/>
       <c r="D50" s="9"/>
@@ -1847,7 +1859,7 @@
         <v>0</v>
       </c>
       <c r="B51" s="9" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="C51" s="9">
         <v>400</v>
@@ -1860,10 +1872,10 @@
         <v>280</v>
       </c>
       <c r="F51" s="9" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="G51" s="9" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.35">
@@ -1871,7 +1883,7 @@
         <v>0</v>
       </c>
       <c r="B52" s="9" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="C52" s="9">
         <v>300</v>
@@ -1884,10 +1896,10 @@
         <v>225</v>
       </c>
       <c r="F52" s="9" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="G52" s="9" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
     </row>
     <row r="53" spans="1:7" x14ac:dyDescent="0.35">
@@ -1896,12 +1908,12 @@
       </c>
       <c r="C53" s="3">
         <f>SUM(C2:C52)</f>
-        <v>24510</v>
+        <v>24600</v>
       </c>
       <c r="D53" s="3"/>
       <c r="E53" s="8">
         <f>SUM(E2:E52)</f>
-        <v>31855</v>
+        <v>31780</v>
       </c>
     </row>
     <row r="54" spans="1:7" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
Doruceno: Gasteiger Birnen 1000 kg/1100 EUR, Kadar Zwetschken 400 kg/440 EUR
</commit_message>
<xml_diff>
--- a/Obst.xlsx
+++ b/Obst.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\holub\AppData\Local\Temp\claude\C--Users-holub-OneDrive---Privatgymnasium-der-Herz-Jesu-Missionare-Radtour-2026\cbd12823-693e-4f3b-bb7d-65f09b0003cf\scratchpad\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{70F9DF02-08D9-4FC8-B20C-369C564F47D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A763505-8ED7-45CC-A693-DCBE78EE4F3A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -305,7 +305,7 @@
     <t>Haagweg 7, 5550 Radstadt</t>
   </si>
   <si>
-    <t>2 Paletten, ca. 1000 kg (statt 1600)</t>
+    <t>2 Paletten, 1000 kg, 1100 €</t>
   </si>
   <si>
     <t>Christian Schlick</t>
@@ -1668,7 +1668,7 @@
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A42" s="9" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B42" s="9" t="s">
         <v>21</v>
@@ -1749,7 +1749,7 @@
     </row>
     <row r="46" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A46" s="9" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B46" s="9" t="s">
         <v>42</v>
@@ -1758,11 +1758,11 @@
         <v>1000</v>
       </c>
       <c r="D46" s="9">
-        <v>1.2</v>
+        <v>1.1000000000000001</v>
       </c>
       <c r="E46" s="9">
         <f>C46*D46</f>
-        <v>1200</v>
+        <v>1100</v>
       </c>
       <c r="F46" s="9" t="s">
         <v>43</v>
@@ -1913,7 +1913,7 @@
       <c r="D53" s="3"/>
       <c r="E53" s="8">
         <f>SUM(E2:E52)</f>
-        <v>31780</v>
+        <v>31680</v>
       </c>
     </row>
     <row r="54" spans="1:7" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
Datum doruceni: sloupec H (Geliefert am) doplnen zpetne z historie, app ho ukazuje u dorucenych
</commit_message>
<xml_diff>
--- a/Obst.xlsx
+++ b/Obst.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\holub\AppData\Local\Temp\claude\C--Users-holub-OneDrive---Privatgymnasium-der-Herz-Jesu-Missionare-Radtour-2026\cbd12823-693e-4f3b-bb7d-65f09b0003cf\scratchpad\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A763505-8ED7-45CC-A693-DCBE78EE4F3A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7116F453-F8D7-4E48-A21A-8A63A332FF16}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,12 +33,15 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="123" uniqueCount="102">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="103">
   <si>
     <t>Geliefert</t>
   </si>
   <si>
     <t>Weichsel</t>
+  </si>
+  <si>
+    <t>Geliefert am</t>
   </si>
   <si>
     <t>Rosi Huber</t>
@@ -345,9 +348,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="44" formatCode="_-&quot;€&quot;\ * #,##0.00_-;\-&quot;€&quot;\ * #,##0.00_-;_-&quot;€&quot;\ * &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="164" formatCode="0\ &quot;kg&quot;"/>
+    <numFmt numFmtId="166" formatCode="dd\.mm\.yyyy"/>
   </numFmts>
   <fonts count="7" x14ac:knownFonts="1">
     <font>
@@ -418,7 +422,7 @@
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="2"/>
     <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
@@ -429,6 +433,7 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="166" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Link" xfId="2" builtinId="8"/>
@@ -784,6 +789,7 @@
     <col min="4" max="4" width="8.36328125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="12" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="31.453125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="13" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.35">
@@ -793,13 +799,16 @@
       <c r="B1" t="s">
         <v>1</v>
       </c>
+      <c r="H1" s="9" t="s">
+        <v>2</v>
+      </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A2" t="b">
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C2" s="3">
         <v>600</v>
@@ -812,7 +821,10 @@
         <v>900</v>
       </c>
       <c r="F2" t="s">
-        <v>3</v>
+        <v>4</v>
+      </c>
+      <c r="H2" s="10">
+        <v>46229</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.35">
@@ -820,7 +832,7 @@
         <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C3" s="3">
         <v>410</v>
@@ -832,7 +844,10 @@
         <v>600</v>
       </c>
       <c r="F3" t="s">
-        <v>5</v>
+        <v>6</v>
+      </c>
+      <c r="H3" s="10">
+        <v>46233</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.35">
@@ -840,7 +855,7 @@
         <v>1</v>
       </c>
       <c r="B4" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C4" s="3">
         <v>1000</v>
@@ -853,7 +868,10 @@
         <v>1500</v>
       </c>
       <c r="F4" t="s">
-        <v>7</v>
+        <v>8</v>
+      </c>
+      <c r="H4" s="10">
+        <v>46233</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.35">
@@ -861,7 +879,7 @@
         <v>1</v>
       </c>
       <c r="B5" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C5" s="3">
         <v>200</v>
@@ -873,10 +891,13 @@
         <v>340</v>
       </c>
       <c r="F5" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="G5" t="s">
-        <v>10</v>
+        <v>11</v>
+      </c>
+      <c r="H5" s="10">
+        <v>46229</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.35">
@@ -884,7 +905,7 @@
         <v>1</v>
       </c>
       <c r="B6" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C6" s="3">
         <v>350</v>
@@ -897,7 +918,10 @@
         <v>525</v>
       </c>
       <c r="F6" t="s">
-        <v>12</v>
+        <v>13</v>
+      </c>
+      <c r="H6" s="10">
+        <v>46231</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.35">
@@ -905,7 +929,7 @@
         <v>1</v>
       </c>
       <c r="B7" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C7" s="3">
         <v>1000</v>
@@ -918,10 +942,13 @@
         <v>1500</v>
       </c>
       <c r="F7" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G7" t="s">
-        <v>15</v>
+        <v>16</v>
+      </c>
+      <c r="H7" s="10">
+        <v>46231</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.35">
@@ -929,7 +956,7 @@
         <v>1</v>
       </c>
       <c r="B8" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C8" s="3">
         <v>300</v>
@@ -942,10 +969,13 @@
         <v>450</v>
       </c>
       <c r="F8" s="5" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="G8" t="s">
-        <v>18</v>
+        <v>19</v>
+      </c>
+      <c r="H8" s="10">
+        <v>46238</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.35">
@@ -953,7 +983,7 @@
         <v>1</v>
       </c>
       <c r="B9" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C9" s="3">
         <v>400</v>
@@ -966,7 +996,10 @@
         <v>600</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
+      </c>
+      <c r="H9" s="10">
+        <v>46229</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.35">
@@ -974,7 +1007,7 @@
         <v>1</v>
       </c>
       <c r="B10" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C10" s="3">
         <v>200</v>
@@ -987,10 +1020,13 @@
         <v>300</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="G10" t="s">
-        <v>23</v>
+        <v>24</v>
+      </c>
+      <c r="H10" s="10">
+        <v>46231</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.35">
@@ -998,7 +1034,7 @@
         <v>1</v>
       </c>
       <c r="B11" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C11" s="3">
         <v>100</v>
@@ -1010,10 +1046,13 @@
         <v>170</v>
       </c>
       <c r="F11" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="G11" t="s">
-        <v>26</v>
+        <v>27</v>
+      </c>
+      <c r="H11" s="10">
+        <v>46229</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.35">
@@ -1021,7 +1060,7 @@
         <v>1</v>
       </c>
       <c r="B12" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C12" s="3">
         <v>640</v>
@@ -1034,7 +1073,10 @@
         <v>960</v>
       </c>
       <c r="F12" t="s">
-        <v>28</v>
+        <v>29</v>
+      </c>
+      <c r="H12" s="10">
+        <v>46233</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.35">
@@ -1042,7 +1084,7 @@
         <v>1</v>
       </c>
       <c r="B13" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C13" s="3">
         <v>900</v>
@@ -1055,7 +1097,10 @@
         <v>1125</v>
       </c>
       <c r="F13" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
+      </c>
+      <c r="H13" s="10">
+        <v>46229</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.35">
@@ -1063,7 +1108,7 @@
         <v>1</v>
       </c>
       <c r="B14" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C14" s="3">
         <v>1000</v>
@@ -1076,7 +1121,10 @@
         <v>1000</v>
       </c>
       <c r="F14" t="s">
-        <v>32</v>
+        <v>33</v>
+      </c>
+      <c r="H14" s="10">
+        <v>46229</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.35">
@@ -1084,7 +1132,7 @@
         <v>1</v>
       </c>
       <c r="B15" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C15" s="3">
         <v>60</v>
@@ -1097,7 +1145,10 @@
         <v>90</v>
       </c>
       <c r="F15" t="s">
-        <v>34</v>
+        <v>35</v>
+      </c>
+      <c r="H15" s="10">
+        <v>46233</v>
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.35">
@@ -1105,7 +1156,7 @@
         <v>1</v>
       </c>
       <c r="B16" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C16" s="3">
         <v>150</v>
@@ -1118,21 +1169,21 @@
         <v>225</v>
       </c>
       <c r="F16" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="G16" t="s">
-        <v>36</v>
-      </c>
-      <c r="H16">
-        <v>6607174862</v>
-      </c>
-    </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.35">
+        <v>37</v>
+      </c>
+      <c r="H16" s="10">
+        <v>46221</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A17" t="b">
         <v>1</v>
       </c>
       <c r="B17" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C17" s="3">
         <v>600</v>
@@ -1145,15 +1196,18 @@
         <v>840</v>
       </c>
       <c r="F17" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.35">
+        <v>39</v>
+      </c>
+      <c r="H17" s="10">
+        <v>46231</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A18" t="b">
         <v>1</v>
       </c>
       <c r="B18" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C18" s="3">
         <v>3000</v>
@@ -1166,18 +1220,21 @@
         <v>3900</v>
       </c>
       <c r="F18" s="6" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="G18" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.35">
+        <v>42</v>
+      </c>
+      <c r="H18" s="10">
+        <v>46231</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A19" t="b">
         <v>1</v>
       </c>
       <c r="B19" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C19" s="3">
         <v>500</v>
@@ -1190,18 +1247,21 @@
         <v>750</v>
       </c>
       <c r="F19" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="G19" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.35">
+        <v>45</v>
+      </c>
+      <c r="H19" s="10">
+        <v>46231</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A20" t="b">
         <v>1</v>
       </c>
       <c r="B20" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C20" s="3">
         <v>200</v>
@@ -1214,15 +1274,18 @@
         <v>300</v>
       </c>
       <c r="F20" s="4" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.35">
+        <v>47</v>
+      </c>
+      <c r="H20" s="10">
+        <v>46222</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A21" t="b">
         <v>1</v>
       </c>
       <c r="B21" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C21" s="3">
         <v>200</v>
@@ -1235,15 +1298,18 @@
         <v>300</v>
       </c>
       <c r="F21" s="5" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.35">
+        <v>49</v>
+      </c>
+      <c r="H21" s="10">
+        <v>46229</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A22" t="b">
         <v>1</v>
       </c>
       <c r="B22" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C22" s="3">
         <v>540</v>
@@ -1256,15 +1322,18 @@
         <v>810</v>
       </c>
       <c r="F22" s="5" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.35">
+        <v>51</v>
+      </c>
+      <c r="H22" s="10">
+        <v>46222</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A23" t="b">
         <v>1</v>
       </c>
       <c r="B23" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C23" s="3">
         <v>100</v>
@@ -1277,15 +1346,18 @@
         <v>150</v>
       </c>
       <c r="F23" s="7" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.35">
+        <v>53</v>
+      </c>
+      <c r="H23" s="10">
+        <v>46222</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A24" t="b">
         <v>1</v>
       </c>
       <c r="B24" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C24" s="3">
         <v>360</v>
@@ -1299,18 +1371,21 @@
         <v>400</v>
       </c>
       <c r="F24" s="7" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="G24" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.35">
+        <v>56</v>
+      </c>
+      <c r="H24" s="10">
+        <v>46222</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A25" t="b">
         <v>1</v>
       </c>
       <c r="B25" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C25">
         <v>950</v>
@@ -1323,18 +1398,21 @@
         <v>1425</v>
       </c>
       <c r="F25" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="G25" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.35">
+        <v>59</v>
+      </c>
+      <c r="H25" s="10">
+        <v>46233</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A26" s="9" t="b">
         <v>1</v>
       </c>
       <c r="B26" s="9" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C26" s="9">
         <v>300</v>
@@ -1347,16 +1425,19 @@
         <v>450</v>
       </c>
       <c r="F26" s="9" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="G26" s="9"/>
-    </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="H26" s="10">
+        <v>46231</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A27" s="9" t="b">
         <v>1</v>
       </c>
       <c r="B27" s="9" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C27" s="9">
         <v>1000</v>
@@ -1369,16 +1450,19 @@
         <v>1500</v>
       </c>
       <c r="F27" s="9" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="G27" s="9"/>
-    </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="H27" s="10">
+        <v>46238</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A28" s="9" t="b">
         <v>1</v>
       </c>
       <c r="B28" s="9" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="C28" s="9">
         <v>300</v>
@@ -1391,21 +1475,24 @@
         <v>450</v>
       </c>
       <c r="F28" s="9" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="G28" s="9"/>
-    </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="H28" s="10">
+        <v>46238</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A29" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A30" s="9" t="b">
         <v>0</v>
       </c>
       <c r="B30" s="9" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C30" s="9"/>
       <c r="D30" s="9"/>
@@ -1413,12 +1500,12 @@
       <c r="F30" s="9"/>
       <c r="G30" s="9"/>
     </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A31" s="9" t="b">
         <v>0</v>
       </c>
       <c r="B31" s="9" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C31" s="9">
         <v>0</v>
@@ -1426,18 +1513,18 @@
       <c r="D31" s="9"/>
       <c r="E31" s="9"/>
       <c r="F31" s="9" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="G31" s="9" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.35">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="32" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A32" s="9" t="b">
         <v>1</v>
       </c>
       <c r="B32" s="9" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C32" s="9">
         <v>380</v>
@@ -1451,18 +1538,21 @@
         <v>350</v>
       </c>
       <c r="F32" s="9" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="G32" s="9" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.35">
+        <v>70</v>
+      </c>
+      <c r="H32" s="10">
+        <v>46271</v>
+      </c>
+    </row>
+    <row r="33" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A33" s="9" t="b">
         <v>1</v>
       </c>
       <c r="B33" s="9" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C33" s="9">
         <v>260</v>
@@ -1476,18 +1566,21 @@
         <v>290</v>
       </c>
       <c r="F33" s="9" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="G33" s="9" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.35">
+        <v>73</v>
+      </c>
+      <c r="H33" s="10">
+        <v>46271</v>
+      </c>
+    </row>
+    <row r="34" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A34" s="9" t="b">
         <v>0</v>
       </c>
       <c r="B34" s="9" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="C34" s="9">
         <v>300</v>
@@ -1500,18 +1593,18 @@
         <v>390</v>
       </c>
       <c r="F34" s="9" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="G34" s="9" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.35">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="35" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A35" s="9" t="b">
         <v>0</v>
       </c>
       <c r="B35" s="9" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="C35" s="9">
         <v>100</v>
@@ -1524,18 +1617,18 @@
         <v>130</v>
       </c>
       <c r="F35" s="9" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="G35" s="9" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.35">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="36" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A36" s="9" t="b">
         <v>1</v>
       </c>
       <c r="B36" s="9" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C36" s="9">
         <v>200</v>
@@ -1548,16 +1641,19 @@
         <v>220.00000000000003</v>
       </c>
       <c r="F36" s="9" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="G36" s="9"/>
-    </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="H36" s="10">
+        <v>46264</v>
+      </c>
+    </row>
+    <row r="37" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A37" s="9" t="b">
         <v>1</v>
       </c>
       <c r="B37" s="9" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C37" s="9">
         <v>600</v>
@@ -1570,16 +1666,19 @@
         <v>660</v>
       </c>
       <c r="F37" s="9" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G37" s="9"/>
-    </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="H37" s="10">
+        <v>46264</v>
+      </c>
+    </row>
+    <row r="38" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A38" s="9" t="b">
         <v>1</v>
       </c>
       <c r="B38" s="9" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C38" s="9">
         <v>600</v>
@@ -1592,16 +1691,19 @@
         <v>660</v>
       </c>
       <c r="F38" s="9" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="G38" s="9"/>
-    </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="H38" s="10">
+        <v>46264</v>
+      </c>
+    </row>
+    <row r="39" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A39" s="9" t="b">
         <v>1</v>
       </c>
       <c r="B39" s="9" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C39" s="9">
         <v>300</v>
@@ -1614,16 +1716,19 @@
         <v>330</v>
       </c>
       <c r="F39" s="9" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="G39" s="9"/>
-    </row>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="H39" s="10">
+        <v>46264</v>
+      </c>
+    </row>
+    <row r="40" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A40" s="9" t="b">
         <v>0</v>
       </c>
       <c r="B40" s="9" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C40" s="9">
         <v>1500</v>
@@ -1636,18 +1741,18 @@
         <v>1650.0000000000002</v>
       </c>
       <c r="F40" s="9" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="G40" s="9" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.35">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="41" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A41" s="9" t="b">
         <v>1</v>
       </c>
       <c r="B41" s="9" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="C41" s="9">
         <v>400</v>
@@ -1660,18 +1765,21 @@
         <v>520</v>
       </c>
       <c r="F41" s="9" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="G41" s="9" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.35">
+        <v>85</v>
+      </c>
+      <c r="H41" s="10">
+        <v>46271</v>
+      </c>
+    </row>
+    <row r="42" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A42" s="9" t="b">
         <v>1</v>
       </c>
       <c r="B42" s="9" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C42" s="9">
         <v>400</v>
@@ -1684,18 +1792,21 @@
         <v>440.00000000000006</v>
       </c>
       <c r="F42" s="9" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="G42" s="9" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.35">
+        <v>86</v>
+      </c>
+      <c r="H42" s="10">
+        <v>46273</v>
+      </c>
+    </row>
+    <row r="43" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A43" s="9" t="b">
         <v>0</v>
       </c>
       <c r="B43" s="9" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="C43" s="9">
         <v>500</v>
@@ -1708,16 +1819,16 @@
         <v>475</v>
       </c>
       <c r="F43" s="9" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="G43" s="9"/>
     </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A44" s="9" t="b">
         <v>0</v>
       </c>
       <c r="B44" s="9" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C44" s="9"/>
       <c r="D44" s="9"/>
@@ -1725,12 +1836,12 @@
       <c r="F44" s="9"/>
       <c r="G44" s="9"/>
     </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A45" s="9" t="b">
         <v>0</v>
       </c>
       <c r="B45" s="9" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C45" s="9">
         <v>1000</v>
@@ -1743,16 +1854,16 @@
         <v>1200</v>
       </c>
       <c r="F45" s="9" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="G45" s="9"/>
     </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A46" s="9" t="b">
         <v>1</v>
       </c>
       <c r="B46" s="9" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C46" s="9">
         <v>1000</v>
@@ -1765,18 +1876,21 @@
         <v>1100</v>
       </c>
       <c r="F46" s="9" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="G46" s="9" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="47" spans="1:7" x14ac:dyDescent="0.35">
+        <v>91</v>
+      </c>
+      <c r="H46" s="10">
+        <v>46273</v>
+      </c>
+    </row>
+    <row r="47" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A47" s="9" t="b">
         <v>0</v>
       </c>
       <c r="B47" s="9" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="C47" s="9">
         <v>600</v>
@@ -1789,18 +1903,18 @@
         <v>720</v>
       </c>
       <c r="F47" s="9" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="G47" s="9" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="48" spans="1:7" x14ac:dyDescent="0.35">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="48" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A48" s="9" t="b">
         <v>0</v>
       </c>
       <c r="B48" s="9" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="C48" s="9">
         <v>300</v>
@@ -1813,10 +1927,10 @@
         <v>360</v>
       </c>
       <c r="F48" s="9" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="G48" s="9" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.35">
@@ -1824,7 +1938,7 @@
         <v>0</v>
       </c>
       <c r="B49" s="9" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="C49" s="9">
         <v>100</v>
@@ -1837,16 +1951,16 @@
         <v>120</v>
       </c>
       <c r="F49" s="9" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="G49" s="9" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A50" s="9"/>
       <c r="B50" s="9" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="C50" s="9"/>
       <c r="D50" s="9"/>
@@ -1859,7 +1973,7 @@
         <v>0</v>
       </c>
       <c r="B51" s="9" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="C51" s="9">
         <v>400</v>
@@ -1872,10 +1986,10 @@
         <v>280</v>
       </c>
       <c r="F51" s="9" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="G51" s="9" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.35">
@@ -1883,7 +1997,7 @@
         <v>0</v>
       </c>
       <c r="B52" s="9" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C52" s="9">
         <v>300</v>
@@ -1896,10 +2010,10 @@
         <v>225</v>
       </c>
       <c r="F52" s="9" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="G52" s="9" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
     </row>
     <row r="53" spans="1:7" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
Armand (Pfarre Koppl): GPS fary u kostela (Nominatim daval nahodny dum)
</commit_message>
<xml_diff>
--- a/Obst.xlsx
+++ b/Obst.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\holub\AppData\Local\Temp\claude\C--Users-holub-OneDrive---Privatgymnasium-der-Herz-Jesu-Missionare-Radtour-2026\cbd12823-693e-4f3b-bb7d-65f09b0003cf\scratchpad\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7116F453-F8D7-4E48-A21A-8A63A332FF16}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BB315073-98AA-4FA6-893C-737A8B3FCE33}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -272,7 +272,7 @@
     <t>5321 Koppl</t>
   </si>
   <si>
-    <t>Pfarre</t>
+    <t>(47.8081289, 13.1570363) Pfarre (bei der Pfarrkirche, Dorfstraße)</t>
   </si>
   <si>
     <t>Rainer</t>
@@ -351,7 +351,7 @@
   <numFmts count="3">
     <numFmt numFmtId="44" formatCode="_-&quot;€&quot;\ * #,##0.00_-;\-&quot;€&quot;\ * #,##0.00_-;_-&quot;€&quot;\ * &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="164" formatCode="0\ &quot;kg&quot;"/>
-    <numFmt numFmtId="166" formatCode="dd\.mm\.yyyy"/>
+    <numFmt numFmtId="165" formatCode="dd\.mm\.yyyy"/>
   </numFmts>
   <fonts count="7" x14ac:knownFonts="1">
     <font>
@@ -433,7 +433,7 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="166" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="165" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Link" xfId="2" builtinId="8"/>

</xml_diff>

<commit_message>
Kadar: presne GPS domu Altaussee 29 (Photon)
</commit_message>
<xml_diff>
--- a/Obst.xlsx
+++ b/Obst.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\holub\AppData\Local\Temp\claude\C--Users-holub-OneDrive---Privatgymnasium-der-Herz-Jesu-Missionare-Radtour-2026\cbd12823-693e-4f3b-bb7d-65f09b0003cf\scratchpad\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BB315073-98AA-4FA6-893C-737A8B3FCE33}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C01E1CC1-24C8-42CF-B66A-DF571E37CC5C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -293,7 +293,7 @@
     <t>ca. 400 kg, Zustellung evtl. am Wochenende, Tel. 0664/4412155</t>
   </si>
   <si>
-    <t>(47.6398954, 13.7640614) Zustellung nach Hause erst ab Di 8.9.2026, Wunsch: Einwegkisten (nicht umfüllen)</t>
+    <t>(47.6422225, 13.7605517) Zustellung nach Hause erst ab Di 8.9.2026, Wunsch: Einwegkisten (nicht umfüllen)</t>
   </si>
   <si>
     <t>Friedl</t>

</xml_diff>

<commit_message>
Nova objednavka: Kadar 400 kg Birnen Williams za 1,20 (ab ca. 28.9.)
</commit_message>
<xml_diff>
--- a/Obst.xlsx
+++ b/Obst.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\holub\AppData\Local\Temp\claude\C--Users-holub-OneDrive---Privatgymnasium-der-Herz-Jesu-Missionare-Radtour-2026\cbd12823-693e-4f3b-bb7d-65f09b0003cf\scratchpad\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C01E1CC1-24C8-42CF-B66A-DF571E37CC5C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C120A24-9E17-4E71-BD2F-A536ECF52B35}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="103">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="127" uniqueCount="104">
   <si>
     <t>Geliefert</t>
   </si>
@@ -321,6 +321,9 @@
   </si>
   <si>
     <t>(47.1513091, 13.7456747) – Urlaub 9.–18.9.!</t>
+  </si>
+  <si>
+    <t>(47.6422225, 13.7605517) Zustellung erst ab ca. 28.9.</t>
   </si>
   <si>
     <t>Äpfel</t>
@@ -781,7 +784,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H71"/>
+  <dimension ref="A1:H72"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="19" bestFit="1" customWidth="1"/>
@@ -1850,7 +1853,7 @@
         <v>1.2</v>
       </c>
       <c r="E45" s="9">
-        <f>C45*D45</f>
+        <f t="shared" ref="E45:E50" si="2">C45*D45</f>
         <v>1200</v>
       </c>
       <c r="F45" s="9" t="s">
@@ -1872,7 +1875,7 @@
         <v>1.1000000000000001</v>
       </c>
       <c r="E46" s="9">
-        <f>C46*D46</f>
+        <f t="shared" si="2"/>
         <v>1100</v>
       </c>
       <c r="F46" s="9" t="s">
@@ -1899,7 +1902,7 @@
         <v>1.2</v>
       </c>
       <c r="E47" s="9">
-        <f>C47*D47</f>
+        <f t="shared" si="2"/>
         <v>720</v>
       </c>
       <c r="F47" s="9" t="s">
@@ -1923,7 +1926,7 @@
         <v>1.2</v>
       </c>
       <c r="E48" s="9">
-        <f>C48*D48</f>
+        <f t="shared" si="2"/>
         <v>360</v>
       </c>
       <c r="F48" s="9" t="s">
@@ -1933,7 +1936,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="49" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A49" s="9" t="b">
         <v>0</v>
       </c>
@@ -1947,7 +1950,7 @@
         <v>1.2</v>
       </c>
       <c r="E49" s="9">
-        <f>C49*D49</f>
+        <f t="shared" si="2"/>
         <v>120</v>
       </c>
       <c r="F49" s="9" t="s">
@@ -1957,130 +1960,150 @@
         <v>79</v>
       </c>
     </row>
-    <row r="50" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A50" s="9"/>
+    <row r="50" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A50" s="9" t="b">
+        <v>0</v>
+      </c>
       <c r="B50" s="9" t="s">
+        <v>22</v>
+      </c>
+      <c r="C50" s="9">
+        <v>400</v>
+      </c>
+      <c r="D50" s="9">
+        <v>1.2</v>
+      </c>
+      <c r="E50" s="9">
+        <f t="shared" si="2"/>
+        <v>480</v>
+      </c>
+      <c r="F50" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="G50" s="9" t="s">
         <v>96</v>
       </c>
-      <c r="C50" s="9"/>
-      <c r="D50" s="9"/>
-      <c r="E50" s="9"/>
-      <c r="F50" s="9"/>
-      <c r="G50" s="9"/>
-    </row>
-    <row r="51" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A51" s="9" t="b">
-        <v>0</v>
-      </c>
+      <c r="H50" s="9"/>
+    </row>
+    <row r="51" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A51" s="9"/>
       <c r="B51" s="9" t="s">
         <v>97</v>
       </c>
-      <c r="C51" s="9">
+      <c r="C51" s="9"/>
+      <c r="D51" s="9"/>
+      <c r="E51" s="9"/>
+      <c r="F51" s="9"/>
+      <c r="G51" s="9"/>
+    </row>
+    <row r="52" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A52" s="9" t="b">
+        <v>0</v>
+      </c>
+      <c r="B52" s="9" t="s">
+        <v>98</v>
+      </c>
+      <c r="C52" s="9">
         <v>400</v>
       </c>
-      <c r="D51" s="9">
+      <c r="D52" s="9">
         <v>0.7</v>
-      </c>
-      <c r="E51" s="9">
-        <f>C51*D51</f>
-        <v>280</v>
-      </c>
-      <c r="F51" s="9" t="s">
-        <v>98</v>
-      </c>
-      <c r="G51" s="9" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="52" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A52" s="9" t="b">
-        <v>0</v>
-      </c>
-      <c r="B52" s="9" t="s">
-        <v>100</v>
-      </c>
-      <c r="C52" s="9">
-        <v>300</v>
-      </c>
-      <c r="D52" s="9">
-        <v>0.75</v>
       </c>
       <c r="E52" s="9">
         <f>C52*D52</f>
+        <v>280</v>
+      </c>
+      <c r="F52" s="9" t="s">
+        <v>99</v>
+      </c>
+      <c r="G52" s="9" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="53" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A53" s="9" t="b">
+        <v>0</v>
+      </c>
+      <c r="B53" s="9" t="s">
+        <v>101</v>
+      </c>
+      <c r="C53" s="9">
+        <v>300</v>
+      </c>
+      <c r="D53" s="9">
+        <v>0.75</v>
+      </c>
+      <c r="E53" s="9">
+        <f>C53*D53</f>
         <v>225</v>
       </c>
-      <c r="F52" s="9" t="s">
-        <v>101</v>
-      </c>
-      <c r="G52" s="9" t="s">
+      <c r="F53" s="9" t="s">
         <v>102</v>
       </c>
-    </row>
-    <row r="53" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A53" t="b">
-        <v>0</v>
-      </c>
-      <c r="C53" s="3">
-        <f>SUM(C2:C52)</f>
-        <v>24600</v>
-      </c>
-      <c r="D53" s="3"/>
-      <c r="E53" s="8">
-        <f>SUM(E2:E52)</f>
-        <v>31680</v>
-      </c>
-    </row>
-    <row r="54" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="G53" s="9" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="54" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A54" t="b">
         <v>0</v>
       </c>
-    </row>
-    <row r="55" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="C54" s="3">
+        <f>SUM(C2:C53)</f>
+        <v>25000</v>
+      </c>
+      <c r="D54" s="3"/>
+      <c r="E54" s="8">
+        <f>SUM(E2:E53)</f>
+        <v>32160</v>
+      </c>
+    </row>
+    <row r="55" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A55" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="56" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A56" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="57" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A57" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="58" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A58" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="59" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A59" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="60" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A60" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="61" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A61" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="62" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A62" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="63" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A63" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="64" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A64" t="b">
         <v>0</v>
       </c>
@@ -2117,6 +2140,11 @@
     </row>
     <row r="71" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A71" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="72" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A72" t="b">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Doruceno 9.9.: Friedl 500 kg Zwetschken za 0,95
</commit_message>
<xml_diff>
--- a/Obst.xlsx
+++ b/Obst.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\holub\AppData\Local\Temp\claude\C--Users-holub-OneDrive---Privatgymnasium-der-Herz-Jesu-Missionare-Radtour-2026\cbd12823-693e-4f3b-bb7d-65f09b0003cf\scratchpad\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C120A24-9E17-4E71-BD2F-A536ECF52B35}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7CBB3165-CBC1-432F-81A6-81D169BC028D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1806,7 +1806,7 @@
     </row>
     <row r="43" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A43" s="9" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B43" s="9" t="s">
         <v>87</v>
@@ -1825,6 +1825,9 @@
         <v>88</v>
       </c>
       <c r="G43" s="9"/>
+      <c r="H43" s="10">
+        <v>46274</v>
+      </c>
     </row>
     <row r="44" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A44" s="9" t="b">

</xml_diff>